<commit_message>
vault backup: 2026-04-27 14:45:52
</commit_message>
<xml_diff>
--- a/content/Consulting/05_Tobe전략/아이디어풀/아이디어_상세설명_260427.xlsx
+++ b/content/Consulting/05_Tobe전략/아이디어풀/아이디어_상세설명_260427.xlsx
@@ -691,7 +691,7 @@
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="70" customWidth="1" min="5" max="5"/>
     <col width="52" customWidth="1" min="6" max="6"/>
   </cols>
@@ -728,7 +728,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="260" customHeight="1">
+    <row r="2" ht="104" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>A-1</t>
@@ -736,7 +736,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>A. 투자·자산 관련</t>
+          <t>A. 투자·자산</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>자녀가 저축하면 부모 계좌에서 자동으로 N% 매칭 이체</t>
+          <t>자녀 저축 시 부모 계좌에서 설정 비율만큼 자동 매칭 이체</t>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
@@ -766,7 +766,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">자녀가 일정 금액을 저축하면, 부모 계좌에서 설정한 비율(예: 50%, 100%, 200%)만큼 자동으로 자녀 계좌에 추가 입금되는 구조다. 부모가 "저축하면 내가 보태줄게"라는 약속을 앱이 자동으로 실행해준다.
+            <t xml:space="preserve">자녀가 저축을 실행하면, 부모가 사전에 설정한 비율(예: 50%·100%·200%)에 따라 부모 계좌에서 자녀 계좌로 매칭 금액이 자동 입금된다. "저축하면 보태주겠다"는 부모의 약속을 앱이 대신 집행하는 구조다.
 </t>
           </r>
           <r>
@@ -784,31 +784,10 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">1. 부모가 앱에서 매칭 비율 설정 (0.5x ~ 3x)
-2. 자녀가 저축 실행
-3. 저축 감지 즉시 부모 계좌에서 자동 매칭 이체
-4. 자녀에게 "엄마/아빠가 OO원 보태줬어요!" 알림 발송
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 참고
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>· 적용 스테이지
-- S2 (10~13세): 부모가 조건 설계, 자녀가 선택 — 매칭 저축 첫 경험
-- S3 (14~15세): 자녀가 목표·비율 직접 제안, 부모가 검토·수락
-- S4 (16~18세): 포괄 허락 범위 안에서 자동 운영</t>
+            <t>1. 부모가 매칭 비율을 0.5x ~ 3x 사이에서 설정한다.
+2. 자녀가 저축을 실행한다.
+3. 저축 감지 즉시 부모 계좌에서 매칭 금액이 자동 이체된다.
+4. 자녀에게 매칭 결과가 알림으로 안내된다.</t>
           </r>
         </is>
       </c>
@@ -829,16 +808,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>- 저축 행동에 즉각적인 외재적 보상 연결 → 행동 반복 동기 강화
-- "내가 노력하면 더 커진다"는 경험 → 복리 개념의 직관적 체득
-- 부모 의도(저축 장려)와 자녀 행동(저축)을 앱이 매개 → 갈등 없는 구조
-- SEED OK RCT 연구: 인출 제한+매칭 구조일 때 장기 저축 효과 가장 높음
-&gt; "아낀 만큼 엄마가 보태줬어!" — 매칭 입금 확인 순간이 핵심 감정 전환점</t>
+            <t>저축 행동에 즉각적인 보상이 연결되어 반복 동기가 강화된다. 노력에 비례한 결과를 직접 확인함으로써 복리 개념을 직관적으로 학습한다. 해외 실증 연구(SEED OK RCT, CSA)는 인출 제한과 매칭 구조가 결합될 때 장기 저축 효과가 가장 크다고 보고한다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="3" ht="182" customHeight="1">
+    <row r="3" ht="104" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>A-1-1</t>
@@ -846,17 +821,17 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>A. 투자·자산 관련</t>
+          <t>A. 투자·자산</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>매칭 비중 연동 인출 제한 구조</t>
+          <t>매칭 비중 연동 인출 제한</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>부모 매칭 비중이 높을수록 인출 불가 기간이 길어지는 구조</t>
+          <t>부모 매칭 비중에 따른 인출 제한 기간 자동 차등화</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
@@ -876,7 +851,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">부모가 매칭하는 비율이 높을수록 해당 자금의 인출 잠금 기간이 자동으로 길어진다. 매칭 비율이 곧 자금의 목적(단기 소비 vs 장기 자산)을 결정하는 구조다.
+            <t xml:space="preserve">부모가 자녀 저축에 보태는 매칭 비중이 높을수록 해당 자금의 인출 제한 기간이 길어진다. 부모의 개입 수준 자체가 자금의 성격(단기 소비용 vs 장기 자산형성용)을 결정한다.
 </t>
           </r>
           <r>
@@ -894,11 +869,9 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>| 매칭 비율 예시 | 성격 | 인출 가능 기간 |
-|---|---|---|
-| 자녀 1만원 + 부모 1천원 (10%) | 단기 소비용 | 단기 인출 가능 |
-| 자녀 1만원 + 부모 5만원 (500%) | 중기 목표 | 3~6개월 잠금 |
-| 자녀 1만원 + 부모 10만원 (1000%) | 장기 자산형성용 (증여 목적) | 장기 묶임 |</t>
+            <t>1. 자녀 저축액 대비 약 10% 수준의 매칭은 단기 인출이 가능한 자금으로 분류된다.
+2. 100% 이상의 큰 매칭은 장기 묶임 자금(증여 목적)으로 분류된다.
+3. 매칭 비중이 임계치를 넘으면 자녀 화면에 자금 성격이 명시적으로 표시된다.</t>
           </r>
         </is>
       </c>
@@ -919,14 +892,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>- 부모의 개입 수준 = 자금의 성격을 결정
-- 높은 매칭 → 부모가 크게 베팅 → 자녀도 장기 관점 유지해야 할 동기 생성
-- "이건 오래 묻어두는 돈"이라는 개념을 UI에서 자연스럽게 전달</t>
+            <t>부모의 개입 수준이 자금의 용도와 성격을 결정하는 신호로 작동한다. 목적이 다른 자금이 동일 계좌 안에서 시각적으로 분리되어 자녀의 자금 성격 학습이 용이해진다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="4" ht="169" customHeight="1">
+    <row r="4" ht="104" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>A-2</t>
@@ -934,7 +905,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>A. 투자·자산 관련</t>
+          <t>A. 투자·자산</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -944,7 +915,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>계좌 A는 장기 자산형성(인출 제한), 계좌 B는 단기 물건 구매 목표</t>
+          <t>장기 자산 계좌와 단기 목표 계좌의 분리 운용</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -964,15 +935,53 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>두 개의 계좌로 자녀 자산을 분리 운용한다.
-- 계좌 A (투자계좌): 장기 자산 형성용. 인출 제한. 복리 운용.
-- 계좌 B (목표계좌): 단기 구매 목표용. 언제든 인출 가능.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr"/>
+            <t xml:space="preserve">계좌 A는 인출이 제한된 장기 자산 형성용으로, 계좌 B는 단기 물건 구매를 위한 목표 저축용으로 분리된다. UI 상 계좌 A가 더 크고 화려하게 표시되어 자녀의 시각적 우선순위를 유도한다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 계좌 A는 인출이 제한된 장기 운용 자산을 보관한다.
+2. 계좌 B는 단기 구매 목표를 위한 자금을 보관한다.
+3. 메인 화면에서 계좌 A가 시각적으로 우선 노출된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>SEED OK RCT 및 CSA 연구는 인출 제한 구조가 적용된 계좌일 때 장기 저축 효과가 가장 크다고 보고한다. 두 계좌 구조는 자금의 시계열별 성격을 자녀가 직관적으로 인식하도록 돕는다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="5" ht="143" customHeight="1">
+    <row r="5" ht="104" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>A-3</t>
@@ -980,17 +989,17 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>A. 투자·자산 관련</t>
+          <t>A. 투자·자산</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>행동 포인트 → 소수 ETF/주식 전환</t>
+          <t>행동 포인트 → 소수 ETF·주식 전환</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>미션 달성·절약 행동 등으로 모은 포인트를 실제 소수 주식으로 전환</t>
+          <t>미션·절약 행동으로 적립한 포인트의 실제 소수 주식 전환</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -1010,7 +1019,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">앱 내 미션 달성, 절약, 퀴즈 정답 등으로 쌓인 포인트를 실제 주식(소수 단위)으로 전환할 수 있는 기능. 게임 포인트처럼 느껴지지만 실제 자산이 된다.
+            <t xml:space="preserve">자녀가 미션 달성·절약 등 다양한 행동으로 적립한 포인트를 실제 소수 단위 주식 또는 ETF로 전환한다. 작은 행동이 자산 형성으로 이어지는 경로가 시각적으로 드러난다.
 </t>
           </r>
           <r>
@@ -1028,10 +1037,9 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 미션 달성 / 절약 감지 / 퀴즈 완료 → 포인트 적립
-2. 일정 포인트 쌓이면 "주식으로 전환할까요?" 알림
-3. 자녀가 원하는 종목(삼성전자, ETF 등) 소수 단위로 전환
-4. "첫 주주가 됐어요!" 확인 화면</t>
+            <t>1. 자녀가 미션 달성·절약 등 행동으로 포인트를 적립한다.
+2. 포인트가 임계치에 도달하면 소수 주식·ETF 전환 옵션이 활성화된다.
+3. 자녀가 종목을 선택하면 포인트가 실제 주식 단위로 전환된다.</t>
           </r>
         </is>
       </c>
@@ -1052,14 +1060,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>- 금융 행동(포인트)과 투자 결과(주식)를 직접 연결
-- "나는 이제 삼성전자 주주야"라는 정체성 형성 → [[G-2]] 투자자 명함과 연계
-- 소수 주식이기 때문에 부담 없이 시작 가능</t>
+            <t>행동의 결과가 자산 보유로 직접 이어지므로 행동 동기가 지속된다. 작은 단위의 자산 보유 경험이 누적되며 투자자 정체성이 형성된다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="6" ht="156" customHeight="1">
+    <row r="6" ht="104" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>A-4</t>
@@ -1067,7 +1073,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>A. 투자·자산 관련</t>
+          <t>A. 투자·자산</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -1077,7 +1083,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>출생 시 2천만원(10년 주기 비과세 증여)을 하나은행에서 미리 운용하도록 유도</t>
+          <t>출생 시점 비과세 증여 한도를 활용한 시드 자금 사전 운용</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -1097,7 +1103,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">한국 세법상 미성년자에게 10년 주기로 2천만원까지 증여세 없이 증여 가능하다. 출생 직후 이 한도를 활용해 아이부자 계좌에서 ETF 등으로 장기 운용하면, 성년이 될 때 유의미한 시드머니가 형성된다.
+            <t xml:space="preserve">자녀 출생 시점에 적용되는 미성년 비과세 증여 한도(10년 단위 2,000만원)를 활용해 시드 자금을 조성하고, 하나은행에서 미리 운용하도록 유도한다.
 </t>
           </r>
           <r>
@@ -1115,16 +1121,35 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 출산 직후 부모에게 "비과세 증여 한도 안내" 자동 발송
-2. 아이부자 계좌 개설 유도
-3. 증여 자금으로 ETF 자동 투자 연결
-4. 10년 후 두 번째 한도(초등→중학교 전환 시) 리마인드</t>
-          </r>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr"/>
+            <t>1. 자녀 출생 직후 부모에게 비과세 한도 활용 시뮬레이션이 제공된다.
+2. 한도 내 입금 시 자동으로 운용 포트폴리오에 배치된다.
+3. 성장 기간 동안 누적 수익이 자녀의 학자금·결혼 자금 등 목표와 연결된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>출생 시점부터 18년의 운용 기간이 확보되어 복리 효과가 극대화된다. 부모가 가장 적극적으로 자녀의 미래를 설계하는 시점에 하나은행과의 장기 관계가 형성된다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="7" ht="169" customHeight="1">
+    <row r="7" ht="104" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>A-6</t>
@@ -1132,7 +1157,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>A. 투자·자산 관련</t>
+          <t>A. 투자·자산</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1142,7 +1167,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>내가 지금까지 받은 패시브 인컴 총액 항상 표시. 이자·배당 누적합이 기념일이 됨</t>
+          <t>자녀가 받은 배당·이자의 누적 합계 상시 시각화</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -1162,7 +1187,27 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>앱 홈 화면에 "내가 지금까지 받은 패시브 인컴 총액"을 항상 표시한다. 이자 12원, 배당 340원... 숫자가 작더라도 누적합이 쌓이며 기념일이 된다.</t>
+            <t xml:space="preserve">자녀가 지금까지 받은 패시브 인컴(이자·배당)의 총액이 메인 화면에 항상 표시된다. 이자 12원, 배당 340원 등 작은 단위라도 누적 합계가 점차 의미 있는 숫자로 성장한다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 이자·배당 발생 시 누적 합계에 자동 반영된다.
+2. 메인 화면 상단에 누적 패시브 인컴 카운터가 상시 노출된다.
+3. 특정 임계치(예: 누적 1만원, 10만원) 도달 시 기념 알림과 카드가 발급된다.</t>
           </r>
         </is>
       </c>
@@ -1183,15 +1228,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>&gt; "이자 12원, 배당 340원... 어느새 내 돈이 1만원 벌었어!"
-작은 숫자도 누적되면 의미를 갖는다. 최초 배당 수령일, 누적 패시브 인컴 1만원 돌파일 등이 자산 형성의 기념일로 기록된다.
-- 금액이 작아도 "돈이 돈을 번다"는 경험 자체가 목적
-- 배당·이자 발생 시 즉시 알림 → 반복 앱 오픈 유도</t>
+            <t>작은 인커밍이 사라지지 않고 누적된다는 가시성을 통해 자산 성장 감각을 일상적으로 체득한다. 누적 합계가 자녀의 자산 정체성으로 자리잡는다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="8" ht="182" customHeight="1">
+    <row r="8" ht="104" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>A-7</t>
@@ -1199,7 +1241,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>A. 투자·자산 관련</t>
+          <t>A. 투자·자산</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1209,7 +1251,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>계좌 생성일부터 현재까지 성장 히스토리 타임라인 시각화</t>
+          <t>계좌 개설부터 현재까지의 금융 여정 타임라인 시각화</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -1229,33 +1271,27 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">계좌 개설일부터 현재까지의 금융 여정을 타임라인으로 시각화한다. "7살 때 첫 배당금 340원, 지금은 월 3,200원"처럼 성장 스토리가 쌓인다.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 참고
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>· 타임라인 예시
-```
-📅 2024.01.01 — 계좌 개설
-💰 2024.03.15 — 첫 배당금 340원 수령
-🎯 2024.06.01 — 첫 목표 달성 (닌텐도 스위치)
-📈 2024.12.31 — 연간 수익률 +8.3%
-💎 2025.03.15 — 배당금 3,200원 (작년 대비 9배)
-🏆 2025.09.01 — 누적 자산 100만원 돌파
-```</t>
+            <t xml:space="preserve">계좌 개설일부터 현재까지의 주요 금융 이벤트(첫 매수, 첫 배당, 목표 달성, 자산 마일스톤 등)가 시간 순으로 정렬되어 자녀의 금융 여정이 하나의 스토리로 시각화된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 주요 금융 이벤트가 발생하면 자동으로 타임라인에 기록된다.
+2. 각 이벤트는 날짜·금액·이모지와 함께 카드 형태로 표시된다.
+3. 성년 도달 시 18년의 여정 전체가 졸업 페이지로 정리된다.</t>
           </r>
         </is>
       </c>
@@ -1276,14 +1312,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>- 이탈 비용 상승: 쌓인 히스토리가 많을수록 앱을 떠나기 어려움
-- 성장 서사 형성: "나는 5년째 투자하는 사람"이라는 정체성
-- S5 성년 전환 시 "18년의 여정" 졸업 페이지로 완성</t>
+            <t>쌓인 히스토리가 많을수록 앱 이탈 비용이 높아진다. "5년째 투자해 온 사람"이라는 투자자 정체성이 형성되며 장기 사용으로 이어진다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="9" ht="130" customHeight="1">
+    <row r="9" ht="104" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>A-8</t>
@@ -1291,7 +1325,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>A. 투자·자산 관련</t>
+          <t>A. 투자·자산</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1301,7 +1335,7 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>보유 종목 관련 뉴스 발생 시 '오늘 네 ○○ 주식이 +340원 올랐어요' 알림</t>
+          <t>보유 종목 관련 뉴스를 자녀 자산 변동과 직접 연결</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -1321,13 +1355,53 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>경제 뉴스나 시장 이벤트가 발생했을 때, 추상적 뉴스가 아니라 "내 계좌와 어떤 관계가 있는지"로 번역해서 전달한다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr"/>
+            <t xml:space="preserve">자녀가 보유한 종목과 관련된 시장 이벤트가 발생하면 "오늘 네 OO 주식이 +340원 올랐다" 형태로 자녀의 자산 변동에 직접 연결한 알림이 제공된다. 미보유 종목에 대해서는 "갖고 있었다면 얼마가 됐을까" 형식으로 학습 시뮬레이션이 노출된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 자녀 보유 종목의 가격 변동·실적 발표·뉴스가 모니터링된다.
+2. 보유 종목 관련 이벤트는 자녀 자산 변동액과 함께 알림으로 전송된다.
+3. 미보유 종목 이벤트는 가상 시뮬레이션 카드로 학습 콘텐츠화된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>거시 경제 뉴스가 추상적 정보가 아닌 자녀의 자산 숫자에 연결된 실감 정보로 전환된다. 시장과 자산의 인과관계를 자연스럽게 학습한다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="10" ht="156" customHeight="1">
+    <row r="10" ht="104" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>A-9</t>
@@ -1335,7 +1409,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>A. 투자·자산 관련</t>
+          <t>A. 투자·자산</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1345,7 +1419,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>투자가 처음으로 마이너스가 될 때 자동으로 교육 푸시 발송</t>
+          <t>투자가 처음 마이너스가 되는 시점의 학습 콘텐츠 자동 푸시</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -1365,7 +1439,27 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>자녀 투자 계좌가 처음으로 마이너스가 됐을 때, 감정적 대응이 아니라 교육 기회로 전환하는 자동 가이드를 발송한다.</t>
+            <t xml:space="preserve">자녀의 투자 자산이 처음 손실 구간에 진입할 때 자동으로 교육 콘텐츠가 활성화된다. 손실 발생 직후가 학습 동기가 가장 높은 시점이라는 점을 활용해 자산 변동의 원리가 자연스럽게 전달된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 투자 자산의 손익률이 마이너스로 전환되는 시점을 시스템이 자동 감지한다.
+2. 감지 즉시 손실 원인과 시장 메커니즘을 설명하는 미니 콘텐츠가 푸시된다.
+3. 콘텐츠 학습 후 자녀의 감정 상태와 대응 의지를 묻는 인터랙션이 추가된다.</t>
           </r>
         </is>
       </c>
@@ -1386,12 +1480,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>손실이 무서운 것이 아니라 "투자의 일부"임을 처음 경험하는 순간. 이 경험을 잘 통과한 자녀는 장기 투자자가 된다.</t>
+            <t>손실 경험이 회피해야 할 부정적 사건이 아닌 학습 자원으로 재구성된다. 첫 손실 시점에 형성된 인식 프레임이 이후 장기 투자 행동의 기반이 된다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="11" ht="156" customHeight="1">
+    <row r="11" ht="104" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>A-10</t>
@@ -1399,17 +1493,17 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>A. 투자·자산 관련</t>
+          <t>A. 투자·자산</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>졸업 카운트다운</t>
+          <t>졸업 카운트다운 (성인 전환 예고)</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>지금 이 속도로 계속하면 18세에 얼마가 됩니까 — 항상 표시</t>
+          <t>현재 페이스 기준 18세 도달 시점의 예상 자산 상시 표시</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
@@ -1429,13 +1523,53 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>홈 화면에 "지금 속도로 가면 18세에 OO만원"을 항상 표시한다. 성인이 되는 날이 구체적인 목표가 되고, 하나은행 성인 상품으로의 자연스러운 연결이 완성된다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr"/>
+            <t xml:space="preserve">현재의 저축·투자 페이스를 그대로 유지할 경우 자녀가 18세에 도달하는 시점의 예상 자산이 메인 화면에 항상 표시된다. 성년 도달 시점이 자녀에게 가시적인 목표가 되며, 하나은행 성인 상품과의 자연스러운 연결 지점이 된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 현재 자산·저축률·투자 수익률을 기반으로 18세 도달 시점의 예상 자산이 매일 재계산된다.
+2. 예상 금액이 메인 화면 상단에 D-day와 함께 표시된다.
+3. 성년 도달이 가까워지면 하나은행 성인 상품으로의 자동 이관 흐름이 활성화된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>성년 시점이 추상적 미래가 아닌 가시적 목표로 인식된다. 18년의 자산 형성 여정이 하나은행 성인 상품으로 자연스럽게 이어진다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="12" ht="351" customHeight="1">
+    <row r="12" ht="117" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>A-11</t>
@@ -1443,7 +1577,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>A. 투자·자산 관련</t>
+          <t>A. 투자·자산</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1453,7 +1587,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>자녀의 모든 수익(이자·배당·매칭금·세뱃돈)을 디폴트로 재투자 슬롯에 자동 배치</t>
+          <t>자녀의 모든 수익을 기본값으로 재투자에 자동 배치</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -1473,7 +1607,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">한국 부자의 94%가 투자 수익을 재투자한다. 대중부유층 86%, 일반대중 74%로 격차가 분명하며, 하나금융연구소는 이 차이를 "재투자 습관의 차이가 부의 격차를 만드는 메커니즘"이라고 명시했다. 자녀에게는 이 행동 패턴 자체를 디폴트 설정으로 학습시킨다.
+            <t xml:space="preserve">한국 부자의 94%는 투자 수익을 재투자한다. 일반 대중(74%) 대비 격차가 분명한 이 행동 패턴이 부의 격차를 만드는 핵심 메커니즘이라는 분석에 기반한다. 자녀의 모든 인커밍(이자·배당·매칭금·세뱃돈·친척 송금)을 의사결정 단계 없이 기본값으로 재투자 슬롯에 배치한다.
 </t>
           </r>
           <r>
@@ -1491,32 +1625,10 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">1. 자녀 계좌에 인커밍이 발생할 때마다(이자, 배당, 매칭금, 세뱃돈, 친척 송금) 자동 캡처
-2. 수익은 재투자 슬롯에 1차 배치 (디폴트 ON)
-3. 자녀가 원하면 "이번 분 회수" 버튼으로 소비/저축 슬롯으로 이동
-4. 매월 리포트: "이번 달 자동 재투자 12,400원 → 신규 자산 +5,200원, 누적 +OO원"
-5. 분기별 "재투자율" 표시 — 부자 평균(94%)·대중부유층(86%)·일반대중(74%) 비교 막대
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 참고
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>· 적용 스테이지
-- S2 (10~13세): 부모가 디폴트 ON, 자녀는 회수 버튼만 학습
-- S3 (14~15세): 자녀가 재투자율을 직접 조정 (50%~100%)
-- S4 (16~18세): 종목별·자산군별 재투자 비율 세분화</t>
+            <t>1. 자녀 계좌에 인커밍이 발생할 때마다 시스템이 자동으로 인식한다.
+2. 수익은 별도 동의 없이 재투자 슬롯에 우선 배치된다(기본값 ON).
+3. 자녀가 원할 경우 "이번 분 회수" 버튼으로 소비·저축 슬롯으로 이동시킬 수 있다.
+4. 매월 재투자 결과 리포트와 분기별 재투자율 통계가 제공된다.</t>
           </r>
         </is>
       </c>
@@ -1537,8 +1649,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">부자가 의식적으로 결정하는 것이 아니라, 부의 순환이 그들에겐 기본값라는 점에서 출발한다. 의사결정 의사결정 단계를 단순화하면 자녀도 동일한 패턴을 행동 패턴으로 누적할 수 있다. 작은 인커밍(이자 12원, 배당 340원)이 사라지지 않고 자산으로 누적되는 가시적 경험이 핵심.
-&gt; "오늘 들어온 배당 340원이 자동으로 ETF 0.0024주가 됐어요." — 알림이 곧 자산 성장 피드백
+            <t xml:space="preserve">의사결정 단계가 단순화되어 자산가의 행동 패턴이 자녀의 기본값으로 자리잡는다. 작은 단위의 수익이 사라지지 않고 자산으로 누적되는 가시성을 통해 복리 개념을 일상적으로 체득한다.
 </t>
           </r>
           <r>
@@ -1556,12 +1667,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>기존 [[A-3]] 행동 포인트→주식 전환은 "행동 보상의 변환". 모든 수익(이자·배당) 자체가 기본값으로 다시 시드가 되는 자동 흐름이다.</t>
+            <t>기존 행동 포인트 전환 기능이 행동에 대한 보상의 변환 구조라면, 본 아이디어는 모든 종류의 수익이 기본값으로 다시 시드가 되는 자동 흐름이라는 점에서 구분된다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="13" ht="247" customHeight="1">
+    <row r="13" ht="130" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>A-12</t>
@@ -1569,7 +1680,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>A. 투자·자산 관련</t>
+          <t>A. 투자·자산</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1579,7 +1690,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>자녀가 알 만한 글로벌 브랜드 1주 매수 + 환율·배당 미니퀘스트로 해외주식 진입 모듈화</t>
+          <t>글로벌 친숙 브랜드 1주 매수와 환율·배당 학습 미니퀘스트</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
@@ -1599,7 +1710,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">K-EMILLI의 해외주식 비중은 30%로 일반 부자(24%)의 1.25배다. 영리치 30대의 46%는 취업 이전에 주식을 시작했다. 자녀가 일찍부터 해외주식 진입로에 노출되는 것이 K-EMILLI 패턴의 출발점이다.
+            <t xml:space="preserve">K-EMILLI(50세 이하 자산 60억대 직장인 부자)의 해외주식 비중은 30%로 일반 부자(24%)의 1.25배다. 영리치 30대의 46%는 취업 이전에 주식을 시작했다. 자녀가 일찍부터 해외주식 진입로에 노출되는 것이 K-EMILLI 행동 패턴의 출발점이라는 가설에 기반한다.
 </t>
           </r>
           <r>
@@ -1617,12 +1728,11 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 자녀 친숙 브랜드 큐레이션 (닌텐도, 디즈니, 애플, 로블록스, 맥도날드, 스타벅스)
-2. 종목 선택 시 "이 회사가 뭐 하는 곳일까요" 60초 카드 (제품·매출·본사 위치)
-3. 환율 기초 학습: "1달러 = 1,400원, 너의 13,000원으로 9.3달러어치"
-4. 첫 1주 매수 (소수점 매수 활용)
-5. 첫 배당 수령 시 "달러 배당이 뭔지" 미니퀘스트 + 자동 원화 환전 옵션
-6. "내 해외주식 지도" — 매수한 회사들이 세계지도 위에 핀으로 표시</t>
+            <t>1. 닌텐도·디즈니·애플·로블록스 등 자녀 친숙 브랜드가 종목 큐레이션에 우선 배치된다.
+2. 종목 선택 시 회사 소개 카드와 환율 기초 학습 미니퀘스트가 노출된다.
+3. 소수점 매수 기능을 통해 첫 1주를 매수한다.
+4. 첫 배당 수령 시 달러 배당 개념과 자동 원화 환전 옵션을 학습한다.
+5. 매수한 종목들이 세계지도 위에 핀으로 표시되어 글로벌 자산 보유 감각이 시각화된다.</t>
           </r>
         </is>
       </c>
@@ -1643,7 +1753,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">K-EMILLI 패턴(해외주식 30%)을 자녀가 학습 단계에서 자연스럽게 흡수. 글로벌 브랜드는 자녀에게 친숙해 진입 마찰이 낮고, 환율·배당 같은 추가 학습 요소가 자연스럽게 따라온다.
+            <t xml:space="preserve">K-EMILLI의 해외주식 비중을 자녀가 학습 단계에서 자연스럽게 흡수한다. 글로벌 친숙 브랜드는 진입 장벽이 낮고, 환율·배당 등 부가 학습 요소가 자연스럽게 따라온다.
 </t>
           </r>
           <r>
@@ -1661,12 +1771,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>기존 [[A-3]] [[A-4]]는 한국 주식·ETF 위주. 해외주식 진입 자체가 별도 모듈로 처음 정의된다.</t>
+            <t>기존 투자 모듈은 한국 주식·ETF 위주이며, 해외주식 진입을 위한 별도 모듈은 본 아이디어가 처음 정의한다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="14" ht="338" customHeight="1">
+    <row r="14" ht="182" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>A-13</t>
@@ -1674,7 +1784,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>A. 투자·자산 관련</t>
+          <t>A. 투자·자산</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1684,7 +1794,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>부모 보유 종목을 매도 없이 자녀 계좌로 직접 이전. 증여 대체 출고 절차를 앱 내에서 자동화</t>
+          <t>부모 보유 종목의 매도 없이 자녀 계좌로 직접 이전</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
@@ -1704,7 +1814,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">한국 부자가 자녀에게 이전하는 자산의 80%가 현금·예금, 29%가 주식이며, 50대 이하 부자는 주식 비중이 더 높아 세대 교체와 함께 주식 이전이 주류화되고 있다. 매도→입금→재매수의 3단계 마찰을 제거하고, 부모가 좋다고 판단한 종목을 그대로 자녀에게 넘기는 흐름을 1-탭으로 만든다.
+            <t xml:space="preserve">한국 부자가 자녀에게 이전하는 자산의 80%가 현금·예금이고 29%가 주식이며, 50대 이하 부자는 주식 비중이 더 높다. 세대 교체와 함께 주식 이전이 주류화되는 흐름에 대응해, 매도→입금→재매수의 3단계 마찰을 제거한 1-탭 증여 흐름을 제공한다.
 </t>
           </r>
           <r>
@@ -1722,12 +1832,11 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">1. 부모 종목 선택 → 이전 수량 지정
-2. 자녀 명의 증권계좌 자동 개설(없을 시) — 법정대리인 동의 흐름 포함
-3. 증여 대체 출고 신청서 자동 작성
-4. 증여재산 평가(증여일 전후 2개월 종가 평균) 자동 계산
-5. 비과세 한도 잔여 자동 조회 → 한도 내 처리
-6. 증여세 신고서 자동 생성 + 신고 기한(증여일 속한 달 말일부터 3개월) 캘린더 연동
+            <t xml:space="preserve">1. 부모가 보유 종목과 이전 수량을 선택한다.
+2. 자녀 명의 증권계좌가 없을 경우 법정대리인 동의 흐름과 함께 자동 개설된다.
+3. 증여 대체 출고 신청서가 자동 작성되고 증여재산 평가(증여일 전후 2개월 종가 평균)가 자동 계산된다.
+4. 비과세 한도 잔여를 자동 조회해 한도 내에서 처리된다.
+5. 증여세 신고서가 자동 생성되고 신고 기한이 캘린더에 등록된다.
 </t>
           </r>
           <r>
@@ -1745,7 +1854,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>한국 증권사들이 정식으로 운영하는 절차다. 미성년 자녀의 경우 법정대리인(부모) 동의 + 자녀 명의 증권계좌만 있으면 가능하며, 비과세 한도(미성년 10년 2,000만원, 성년 5,000만원) 내에서는 증여세 0원으로 처리된다. 매도가 없어 부모의 양도세 부담도 없다.</t>
+            <t>한국 증권사들이 정식으로 운영하는 절차이며, 미성년 자녀의 경우 법정대리인 동의와 자녀 명의 증권계좌만 있으면 가능하다. 비과세 한도(미성년 10년 2,000만원, 성년 5,000만원) 내에서는 증여세가 발생하지 않으며, 매도가 없어 부모의 양도세 부담도 없다.</t>
           </r>
         </is>
       </c>
@@ -1766,7 +1875,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">부모가 신뢰하는 종목이 그대로 자녀의 첫 종목이 된다 — 부모의 종목 선택 노하우가 자산과 함께 이전되는 효과. 매도 마찰 제거로 부모의 실행 장벽도 낮다. 50대 이하 부자에게 직접 매칭되는 행동 패턴.
+            <t xml:space="preserve">부모가 신뢰하는 종목이 그대로 자녀의 첫 종목이 된다. 부모의 종목 선택 노하우가 자산과 함께 이전되며, 매도 마찰이 없어 부모의 실행 장벽도 낮아진다.
 </t>
           </r>
           <r>
@@ -1784,12 +1893,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>기존 [[A-4]] 출생 직후 비과세 증여는 현금 운용 유도. 부모의 기존 종목을 자녀 계좌로 그대로 이전하는 다른 트랙이다.</t>
+            <t>기존 출생 직후 비과세 증여가 현금 운용 유도에 초점이 있다면, 본 아이디어는 부모의 기존 종목을 자녀 계좌로 그대로 이전하는 별도 트랙이다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="15" ht="260" customHeight="1">
+    <row r="15" ht="130" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>A-14</t>
@@ -1797,7 +1906,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>A. 투자·자산 관련</t>
+          <t>A. 투자·자산</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1807,7 +1916,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>새 종목·ETF 첫 매수 전 30~60초 미니 학습 통과 의무 — 통과 시 매수 버튼 활성화</t>
+          <t>신규 종목·ETF 첫 매수 전 미니 학습 통과 의무화</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -1827,7 +1936,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">한국 부자 본인들이 꼽은 자산관리 1위 지혜는 "지속적인 금융지식 습득(15.0%)". K-EMILLI의 47%가 "공부를 먼저 하고 투자한다"는 원칙을 따르며, 이는 일반 부자(39%)보다 1.2배 높다. 학습 → 투자 시퀀스를 UX로 강제한다.
+            <t xml:space="preserve">한국 부자가 꼽은 자산관리 1위 지혜는 "지속적인 금융지식 습득"(15.0%)이다. K-EMILLI의 47%는 "공부를 먼저 하고 투자한다"는 원칙을 따르며, 일반 부자(39%) 대비 1.2배 높다. 학습 → 투자의 시퀀스를 UX 차원에서 강제한다.
 </t>
           </r>
           <r>
@@ -1845,12 +1954,11 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 새 종목·ETF 매수 화면 진입 시 학습 게이트 활성화
-2. 카드 1: "이 회사가 뭐 하는 곳일까요" 30초 (제품·매출·CEO)
-3. 카드 2: PER·배당수익률·52주 변동폭 등 핵심 지표 30초
-4. 카드 3 (퀴즈): 3문항 미니 퀴즈 — 통과 시 매수 버튼 활성화
-5. 통과 후에는 동일 종목 3개월 패스 (반복 학습 면제)
-6. 학습 완료 카드는 "투자 노트"에 누적 — 자녀 본인의 학습 히스토리</t>
+            <t>1. 신규 종목·ETF 매수 화면 진입 시 학습 게이트가 활성화된다.
+2. 회사 정보(제품·매출·CEO)를 30초 카드로 학습한다.
+3. PER·배당수익률·52주 변동폭 등 핵심 지표를 30초 카드로 학습한다.
+4. 3문항 미니 퀴즈 통과 시에만 매수 버튼이 활성화된다.
+5. 통과 후에는 동일 종목 3개월 패스가 적용되며, 학습 카드는 "투자 노트"에 누적된다.</t>
           </r>
         </is>
       </c>
@@ -1871,7 +1979,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">K-EMILLI 47%의 "先공부後투자" 행동을 기본값으로 강제. 매수 직전이 학습 동기 최고점이라는 점에서 효율적이다. 사후 손실 가이드([[A-9]])와 짝을 이루어 사전·사후 학습 사이클이 완성된다.
+            <t xml:space="preserve">K-EMILLI의 "先공부後투자" 행동 원칙이 자녀의 투자 의사결정 기본값으로 자리잡는다. 매수 직전이 학습 동기가 가장 높은 시점이라는 점에서 학습 효율이 극대화된다.
 </t>
           </r>
           <r>
@@ -1889,7 +1997,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>기존 [[A-9]] 첫 손실 가이드는 손실 후 사후 교육. 매수 전 사전 게이팅으로 시점이 다르다.</t>
+            <t>기존 첫 손실 가이드가 손실 발생 후 사후 교육이라면, 본 아이디어는 매수 전 사전 학습 게이팅으로 시점이 다르다. 두 기능이 결합되면 사전·사후 학습 사이클이 완성된다.</t>
           </r>
         </is>
       </c>
@@ -1902,7 +2010,7 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>B. 소비·저축 행동 관련</t>
+          <t>B. 소비·저축 행동</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
@@ -1912,7 +2020,7 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>현재 소비 패턴 기반으로 목표 달성 시뮬레이션 제공</t>
+          <t>현재 소비 패턴 기반 목표 달성 시뮬레이션 알림</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -1932,7 +2040,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">현재 소비 패턴을 기반으로 목표 달성 시점을 자동 계산해서 알려준다.
+            <t xml:space="preserve">현재의 소비 패턴을 기반으로 자녀가 목표한 물품의 도달 시점이 자동 계산되어 "이렇게 쓰면 에어팟까지 6개월" 형태로 안내된다.
 </t>
           </r>
           <r>
@@ -1950,16 +2058,35 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 소비 패턴 30일 분석
-2. 현재 속도로 목표 달성 예상일 계산
-3. "이 항목 줄이면 OO일 단축" 제안
-4. 주간 소비 리포트에 함께 표시</t>
-          </r>
-        </is>
-      </c>
-      <c r="F16" s="11" t="inlineStr"/>
+            <t>1. 자녀의 소비 패턴이 일별·주별로 분석된다.
+2. 현재 페이스 유지 시 목표 물품의 도달 시점이 자동 계산된다.
+3. 주요 분기점(목표 50%, 80% 등)에 알림이 발송된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>추상적 소비 결정이 구체적 시간 단위로 환산되어 자녀의 자기 조절 행동이 유도된다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="17" ht="143" customHeight="1">
+    <row r="17" ht="104" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
           <t>B-2</t>
@@ -1967,7 +2094,7 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>B. 소비·저축 행동 관련</t>
+          <t>B. 소비·저축 행동</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
@@ -1977,7 +2104,7 @@
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>용돈 수령 직후 소비 패턴 기반으로 저축·투자 비율 개인화 추천</t>
+          <t>용돈 수령 직후 소비·저축·투자 비율 개인화 추천</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
@@ -1997,7 +2124,27 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>용돈이 들어오는 순간, 소비 패턴을 분석해 "저축은 이 정도, 투자는 이 정도 하면 좋아요"라고 자동 제안한다.</t>
+            <t xml:space="preserve">용돈 수령 직후 자녀의 최근 소비 패턴이 분석되어 "이번 달은 저축 OO원, 투자 OO원, 소비 OO원이 적절하다"는 개인화 가이드가 제시된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 용돈 입금 즉시 분배 추천 화면이 노출된다.
+2. 최근 소비 패턴과 목표 진척도를 기반으로 비율이 자동 산출된다.
+3. 자녀가 수정 또는 수락하면 즉시 분배가 실행된다.</t>
           </r>
         </is>
       </c>
@@ -2018,14 +2165,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>- 제안이지 강제가 아님 — 자녀가 직접 조정 가능
-- 과거 패턴 기반이라 "나한테 맞는" 느낌
-- [[C-3]] AI 대화형 UI와 결합하면 "얼마 쓸 거야?" 대화로 자연화</t>
+            <t>수령 시점이 의사결정 동기가 가장 높은 순간이라는 점을 활용해 분배 행동이 자연스럽게 유도된다. 무계획 소비가 사전에 차단된다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="18" ht="117" customHeight="1">
+    <row r="18" ht="104" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
         <is>
           <t>B-3</t>
@@ -2033,17 +2178,17 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>B. 소비·저축 행동 관련</t>
+          <t>B. 소비·저축 행동</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>위시리스트 기능 → 매칭 목표 자동제안</t>
+          <t>위시리스트 → 매칭 목표 자동 제안</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>자녀가 갖고 싶은 물건을 위시리스트에 등록하면 부모에게 저축 목표 자동 제안</t>
+          <t>자녀 위시리스트 등록 시 부모 매칭 저축 목표 자동 제안</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
@@ -2063,13 +2208,53 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>자녀가 원하는 물건을 앱에서 위시리스트에 추가하면, 자동으로 부모에게 "이 목표로 저축해볼래?" 제안 알림이 전송된다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F18" s="11" t="inlineStr"/>
+            <t xml:space="preserve">자녀가 갖고 싶은 물건이나 투자 상품을 위시리스트에 등록하면 부모에게 "이 목표로 함께 저축해보시겠습니까"라는 매칭 저축 제안이 자동 발송된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 자녀가 위시리스트에 항목을 추가한다.
+2. 부모에게 매칭 저축 제안 알림이 전송된다.
+3. 부모가 수락하면 해당 목표 전용 저축 트랙이 활성화된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>자녀의 욕구가 부모와의 협업 목표로 전환된다. 단순 구매 요청이 함께 모으는 활동으로 재구성된다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="19" ht="156" customHeight="1">
+    <row r="19" ht="104" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
         <is>
           <t>B-4</t>
@@ -2077,7 +2262,7 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>B. 소비·저축 행동 관련</t>
+          <t>B. 소비·저축 행동</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -2087,7 +2272,7 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>물건 선택 → 목표 시기 설정 → 부모 기여 설정 → 월 저축액 자동 계산</t>
+          <t>자동차 옵션 카탈로그 형태로 구성된 저축 플래너</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
@@ -2107,13 +2292,54 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>"자동차 살 때 옵션 설정하는 느낌"으로 저축 계획을 세운다. 페이지 단위 프로세스가 아니라 AI 대화처럼 자연스럽게 진행된다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F19" s="11" t="inlineStr"/>
+            <t xml:space="preserve">자동차 구매 시 옵션을 선택하듯, 자녀가 사고 싶은 물건과 목표 시기를 정하면 부모 분담 비율을 슬라이더로 조정할 수 있다. 월 저축액과 도달 시점이 즉시 자동 계산된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 자녀가 목표 물건과 희망 도달 시기를 입력한다.
+2. 부모 분담 비율(최대 50%)을 슬라이더로 설정한다.
+3. 월별 저축액과 도달 일자가 실시간 계산되어 표시된다.
+4. 자녀와 부모가 모두 동의하면 자동 저축 트랙으로 변환된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>단계별 페이지가 아닌 한 화면 옵션 설정 형태로 구성되어 작업 부담이 최소화된다. 결정 과정이 게임처럼 재구성되어 진입 마찰이 낮아진다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="20" ht="143" customHeight="1">
+    <row r="20" ht="104" customHeight="1">
       <c r="A20" s="7" t="inlineStr">
         <is>
           <t>B-5</t>
@@ -2121,7 +2347,7 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>B. 소비·저축 행동 관련</t>
+          <t>B. 소비·저축 행동</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -2131,7 +2357,7 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>부모가 선수금을 걸어두고 자녀가 나머지를 분할 저축. 실패 시 부모가 몫을 가져감</t>
+          <t>부모 선수금 + 자녀 분할 저축 + 실패 시 패널티 구조</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -2151,7 +2377,28 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>부모가 먼저 일정 금액(선수금)을 걸어두고, 자녀가 나머지를 매달 분할 저축하는 구조. 중간에 저축 목표를 달성하지 못하면 패널티가 발생한다.</t>
+            <t xml:space="preserve">부모가 먼저 선수금(예: 60만원)을 걸어두고, 자녀가 나머지 금액(예: 40만원)을 매월 분할 저축한다. 중간에 저축이 실패하면 부모가 모은 선수금을 회수하는 패널티 구조가 적용된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 부모가 목표액 중 일부를 선수금으로 잠금 예치한다.
+2. 자녀에게 잔여 금액의 월별 분할 저축 일정이 부여된다.
+3. 성공 시 선수금이 자녀에게 이전된다.
+4. 실패 시 부모가 선수금을 회수한다.</t>
           </r>
         </is>
       </c>
@@ -2172,14 +2419,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>&gt; "아이가 사고 싶은 걸 그냥 사주지 마시고, 일부 보태고 일부는 아이가 모으는 경험을 하게 해주세요."
-- 부모의 무조건적 소비 지원을 구조화된 교육 기회로 전환
-- 실패해도 괜찮음 — 실패 자체가 학습</t>
+            <t>부모의 무조건적 지원이 아닌 함께 모으는 경험이 형성된다. 패널티 구조는 자녀의 책임감과 약속 이행 동기를 강화한다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="21" ht="117" customHeight="1">
+    <row r="21" ht="104" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
         <is>
           <t>B-7</t>
@@ -2187,7 +2432,7 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>B. 소비·저축 행동 관련</t>
+          <t>B. 소비·저축 행동</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -2197,7 +2442,7 @@
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>세뱃돈/조부모 송금 등 이벤트성 돈을 1-탭으로 투자 시드로 전환</t>
+          <t>이벤트성 일시 수령 자금의 1-탭 투자 시드 전환</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
@@ -2217,13 +2462,53 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>세뱃돈, 생일 선물, 조부모 송금 등 일시적으로 들어오는 목돈을 쉽게 투자 시드로 전환할 수 있도록 지원한다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F21" s="11" t="inlineStr"/>
+            <t xml:space="preserve">세뱃돈, 조부모 송금 등 일시적으로 수령한 이벤트성 자금을 1-탭으로 투자 시드로 전환할 수 있다. "세뱃돈 절반을 투자하면 여름방학에 얼마가 될까" 형태의 시뮬레이션이 함께 제공된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 이벤트성 송금이 감지되면 시드 전환 추천 알림이 발송된다.
+2. 전환 비율(전액·절반·1/3 등)을 선택할 수 있다.
+3. 선택 즉시 투자 슬롯으로 이체되며, 미래 시뮬레이션이 함께 표시된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>흔히 소비로 흘러가는 이벤트성 자금이 자산 형성으로 회수된다. 일시 수령액이 장기 자산으로 전환되는 경험이 누적된다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="22" ht="130" customHeight="1">
+    <row r="22" ht="104" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
         <is>
           <t>B-8</t>
@@ -2231,7 +2516,7 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>B. 소비·저축 행동 관련</t>
+          <t>B. 소비·저축 행동</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -2241,7 +2526,7 @@
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>자녀 소비가 평소 대비 감소한 주를 자동 감지 → 매칭 배율 동적 증가</t>
+          <t>자녀 절약 행동 자동 감지 시 매칭 배율 동적 상향</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -2261,7 +2546,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">자녀가 평소보다 덜 쓴 주를 자동으로 감지해, 그 주에 한해 매칭 배율을 높여준다. 절약이 즉각적인 보상으로 연결된다.
+            <t xml:space="preserve">자녀의 주간 소비가 평소 대비 감소한 경우 시스템이 자동으로 절약 행동을 인식해 "이번 주 매칭 2.5배 찬스" 형태로 매칭 배율을 동적으로 상향 조정한다.
 </t>
           </r>
           <r>
@@ -2279,16 +2564,35 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 주간 소비 분석 → 평균 대비 N% 감소 감지
-2. 부모에게 알림: "OO이가 이번 주 평소보다 덜 썼어요. 매칭 강화해볼까요? [강화하기]"
-3. 부모 수락 시: "이번 주 매칭 2.5배 찬스!" 자녀 알림 발송
-4. 자녀가 저축 → 부스트된 매칭 적용</t>
-          </r>
-        </is>
-      </c>
-      <c r="F22" s="11" t="inlineStr"/>
+            <t>1. 주간 소비 패턴이 평균과 비교 분석된다.
+2. 기준 이상 절약이 감지되면 매칭 배율 상향 알림이 발송된다.
+3. 해당 주 동안의 추가 저축에 상향된 배율이 적용된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>절약 행동이 즉각적 보상으로 연결된다. 자녀의 자기 조절 행동이 일회성이 아닌 반복 동기로 강화된다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="23" ht="130" customHeight="1">
+    <row r="23" ht="104" customHeight="1">
       <c r="A23" s="12" t="inlineStr">
         <is>
           <t>C-2</t>
@@ -2296,7 +2600,7 @@
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>C. AI·개인화 관련</t>
+          <t>C. AI·개인화</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
@@ -2306,7 +2610,7 @@
       </c>
       <c r="D23" s="15" t="inlineStr">
         <is>
-          <t>또래 평균 저축률 비교, 자녀 금융 성장도 시각화 제공</t>
+          <t>또래 평균 대비 자녀의 금융 행동 비교 시각화</t>
         </is>
       </c>
       <c r="E23" s="16" t="inlineStr">
@@ -2326,13 +2630,53 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>부모에게 "이 나이 아이들 평균 저축률은 얼마인지", "우리 아이의 금융 성장도는 또래 대비 어떤지"를 AI가 분석해서 제공한다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F23" s="16" t="inlineStr"/>
+            <t xml:space="preserve">동년배 평균 저축률 등이 자녀의 데이터와 비교되어 시각화된다. 절대 금액이 아닌 용돈 대비 저축률 또는 소비 대비 저축률 등 상대 지표로 표시된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 자녀의 저축·소비·투자 데이터가 일별 집계된다.
+2. 동년배 평균과 비교한 리포트가 부모 화면에 제공된다.
+3. 특이 패턴 감지 시 부모에게 인사이트가 제안된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F23" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>절대 금액이 아닌 상대 지표가 사용되어 자산 격차에 의한 위화감이 제거된다. 부모의 비교 본능이 자녀의 행동 개선으로 전환된다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="24" ht="143" customHeight="1">
+    <row r="24" ht="104" customHeight="1">
       <c r="A24" s="12" t="inlineStr">
         <is>
           <t>C-3</t>
@@ -2340,7 +2684,7 @@
       </c>
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t>C. AI·개인화 관련</t>
+          <t>C. AI·개인화</t>
         </is>
       </c>
       <c r="C24" s="14" t="inlineStr">
@@ -2350,7 +2694,7 @@
       </c>
       <c r="D24" s="15" t="inlineStr">
         <is>
-          <t>단계별 페이지 없이 AI와 대화하듯 계획 자동 생성</t>
+          <t>단계별 페이지가 아닌 AI 대화 형태의 자연스러운 설정 흐름</t>
         </is>
       </c>
       <c r="E24" s="16" t="inlineStr">
@@ -2370,7 +2714,27 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>"기능처럼 안 생겼으면 좋겠다"는 설계 원칙. 페이지를 넘기며 설정하는 방식이 아니라, AI와 대화하듯 자연스럽게 목표를 설정한다.</t>
+            <t xml:space="preserve">기능 설정이 페이지 단위 프로세스가 아닌 AI 대화 형태로 구성된다. "뭐 사고 싶은데 어떻게 해야 되지" 같은 자연어 입력에 대해 계획이 자동 생성되며, 한 화면에서 기본값을 먼저 제시하고 수정만 팝업으로 처리된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 자녀의 자연어 입력에 대해 AI가 기본 계획을 생성한다.
+2. 한 화면에 추천값이 먼저 표시된다.
+3. 수정이 필요한 항목만 탭하면 팝업으로 변경된다.</t>
           </r>
         </is>
       </c>
@@ -2391,14 +2755,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>- 서비스가 먼저 기본값 제안 → 자녀는 수정만 탭
-- 한 화면에서 모든 설정 완료 (팝업으로 처리)
-- "단계별 페이지는 답답하다" — 자연스러운 대화 흐름</t>
+            <t>단계별 페이지의 답답함이 제거되고, 기능이 도구처럼 노출되지 않는다. 사용 마찰이 낮아져 진입 장벽이 줄어든다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="25" ht="130" customHeight="1">
+    <row r="25" ht="104" customHeight="1">
       <c r="A25" s="12" t="inlineStr">
         <is>
           <t>C-4</t>
@@ -2406,7 +2768,7 @@
       </c>
       <c r="B25" s="13" t="inlineStr">
         <is>
-          <t>C. AI·개인화 관련</t>
+          <t>C. AI·개인화</t>
         </is>
       </c>
       <c r="C25" s="14" t="inlineStr">
@@ -2416,7 +2778,7 @@
       </c>
       <c r="D25" s="15" t="inlineStr">
         <is>
-          <t>서비스가 먼저 나이·지역·패턴 기반 기본 용돈 세팅을 제안</t>
+          <t>지역·연령 데이터 기반 용돈 기본 세팅 자동 제안</t>
         </is>
       </c>
       <c r="E25" s="16" t="inlineStr">
@@ -2436,13 +2798,53 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>"송파구 사는 8살이면 용돈은 한 달에 한 번 이 정도씩 주시고..." — 서비스가 먼저 기본 세팅을 제안한다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F25" s="16" t="inlineStr"/>
+            <t xml:space="preserve">"송파구 거주 8세는 한 달 OO원이 적절하다" 등 지역·연령별 데이터를 기반으로 서비스가 먼저 용돈 기본 세팅을 제안한다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 자녀의 거주 지역, 연령, 학제 정보가 입력된다.
+2. 동일 조건의 통계를 기반으로 용돈 기준값이 자동 생성된다.
+3. 부모는 추천값을 수락하거나 부분 수정할 수 있다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F25" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>백지 상태에서 결정해야 하는 부담이 제거된다. 부모의 의사결정 부하가 낮아져 도입 마찰이 줄어든다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="26" ht="273" customHeight="1">
+    <row r="26" ht="104" customHeight="1">
       <c r="A26" s="12" t="inlineStr">
         <is>
           <t>C-5</t>
@@ -2450,7 +2852,7 @@
       </c>
       <c r="B26" s="13" t="inlineStr">
         <is>
-          <t>C. AI·개인화 관련</t>
+          <t>C. AI·개인화</t>
         </is>
       </c>
       <c r="C26" s="14" t="inlineStr">
@@ -2460,7 +2862,7 @@
       </c>
       <c r="D26" s="15" t="inlineStr">
         <is>
-          <t>K-EMILLI(50세 이하·자산 60억대 직장인 부자)의 평균 포트폴리오를 벤치마크로 자녀 자산과의 갭 시각화</t>
+          <t>K-EMILLI 평균 포트폴리오를 벤치마크로 자녀 자산 갭 시각화</t>
         </is>
       </c>
       <c r="E26" s="16" t="inlineStr">
@@ -2480,7 +2882,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">최근 10년 내 부자 반열에 진입한 K-EMILLI는 평균 51세·연소득 5억·총자산 60억대의 회사원·공무원 그룹이다. 이들의 부 형성 2위 요인은 주식 투자 성공(36%)이며, ETF 보유 57%·해외주식 30%로 일반 부자(각 53%·24%)보다 적극적이다. 막연한 "부자처럼"이 아니라 정량 기준점을 자녀에게 제시.
+            <t xml:space="preserve">최근 10년 내 부자 반열에 오른 K-EMILLI(평균 51세·자산 60억대 직장인)의 평균 포트폴리오 구성이 벤치마크로 제공된다. 자녀 포트폴리오와의 갭이 정량 비교되며, 미래 페르소나 모델링이 유도된다.
 </t>
           </r>
           <r>
@@ -2498,11 +2900,10 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 자녀 포트폴리오 자동 분석: 주식 비율, ETF 비율, 해외주식 비율, 현금 비율
-2. K-EMILLI 평균과 비교 차트 (4개 축 레이더 그래프)
-3. 갭 메우기 추천: "K-EMILLI는 ETF 57%, 너는 ETF 20% — 갭 메우려면 OO원 ETF 추가"
-4. 매월 1회 리포트: "K-EMILLI에 더 가까워졌어요" 또는 "더 멀어졌어요"
-5. 18세 시점 시뮬: "지금 페이스로 가면 50세에 K-EMILLI 평균에 도달할 확률 OO%"</t>
+            <t>1. 자녀 포트폴리오의 자산군별 비중이 자동 분석된다.
+2. K-EMILLI 평균(주식 75%·ETF 57%·해외주식 30% 등)과 4축 레이더 그래프로 비교된다.
+3. 갭이 큰 항목에 대해 "ETF 비중을 OO원 늘리면 평균에 도달한다" 형태로 액션이 추천된다.
+4. 월간 리포트와 18세·50세 시점 시뮬레이션이 함께 제공된다.</t>
           </r>
         </is>
       </c>
@@ -2523,7 +2924,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">평균값 통계나 또래 비교가 아니라, 자녀가 미래에 닮을 모델 페르소나를 제시한다는 점이 다르다. K-EMILLI는 천억 자산가가 아니라 평범한 직장인 출신 부자라, 자녀와 부모 모두에게 도달 가능한 모델로 인식된다.
+            <t xml:space="preserve">막연한 "부자처럼"이 정량 기준점으로 구체화된다. K-EMILLI는 천억 자산가가 아닌 평범한 직장인 출신 부자이므로 자녀와 부모 모두에게 도달 가능한 모델로 인식된다.
 </t>
           </r>
           <r>
@@ -2541,12 +2942,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>기존 [[C-2]] 부모 AI는 "또래 자녀 비교"(동년배 평균값). 미래 페르소나 비교로, 시간 축이 다르다.</t>
+            <t>기존 부모 AI 어시스턴트가 동년배 평균 비교(현재 시점)에 초점을 둔다면, 본 아이디어는 미래에 닮을 페르소나와의 비교라는 점에서 시간 축이 다르다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="27" ht="286" customHeight="1">
+    <row r="27" ht="104" customHeight="1">
       <c r="A27" s="12" t="inlineStr">
         <is>
           <t>C-6</t>
@@ -2554,7 +2955,7 @@
       </c>
       <c r="B27" s="13" t="inlineStr">
         <is>
-          <t>C. AI·개인화 관련</t>
+          <t>C. AI·개인화</t>
         </is>
       </c>
       <c r="C27" s="14" t="inlineStr">
@@ -2564,7 +2965,7 @@
       </c>
       <c r="D27" s="15" t="inlineStr">
         <is>
-          <t>익명화된 동년배 자녀의 자산 형성 케이스를 카드로 큐레이션 — 또래 모델링</t>
+          <t>익명화된 동년배 자산 형성 사례를 카드 형태로 큐레이션</t>
         </is>
       </c>
       <c r="E27" s="16" t="inlineStr">
@@ -2584,7 +2985,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">한국 미성년자 주식 보유 규모는 약 7조원, 계좌 수는 2019년부터 2024년까지 7.7배 성장. 영리치의 5%가 미성년·학창시절에 주식을 시작했다. 또래의 실재를 자녀에게 데이터가 아니라 스토리로 노출한다.
+            <t xml:space="preserve">한국 미성년자 주식 보유 규모는 약 7조원, 계좌 수는 5년간 7.7배 성장했다. 영리치의 5%는 미성년기에 주식을 시작했다. 또래의 실재가 데이터가 아닌 개별 스토리로 자녀에게 노출된다.
 </t>
           </r>
           <r>
@@ -2602,18 +3003,10 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 케이스 카드 (익명화)
-```
-📇 케이스 #042
-9살 김OO · 부산 거주 · 시작 2024.03
-첫 매수: 코스피200 ETF 1주
-3년 누적: +18.2% (130만원 → 154만원)
-특이점: 매월 세뱃돈+용돈의 30% 자동 적립
-```
-2. 케이스 라이브러리: 연령별·전략별·시작 시점별 필터
-3. "내 모델" 즐겨찾기 — 자녀가 닮고 싶은 케이스 3개 선택
-4. 패턴 매칭 알림: "너는 케이스 #042와 비슷한 경로야 (적립 시점·종목 일치율 80%)"
-5. 케이스 자체에 자녀가 기여 — 일정 자산 도달 시 본인 케이스가 익명으로 라이브러리에 합류</t>
+            <t>1. 익명화된 또래 사례가 카드 형태로 큐레이션된다(연령·전략·시작 시점별 필터).
+2. 자녀가 닮고 싶은 사례 3개를 "내 모델"로 즐겨찾기할 수 있다.
+3. 패턴 매칭 알고리즘이 자녀의 행동과 유사한 사례를 추천한다.
+4. 자녀가 일정 자산에 도달하면 본인 사례가 익명으로 라이브러리에 합류한다.</t>
           </r>
         </is>
       </c>
@@ -2634,7 +3027,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">평균값 통계가 아니라 개별 사례 스토리는 정상화 효과가 강하다. "나 같은 애가 있다"는 인식이 행동의 지속 동기로 작용. 또래 모델링은 청소년기 정체성 형성과 직결된다.
+            <t xml:space="preserve">평균값 통계가 아닌 개별 스토리는 정상화 효과가 강하다. 또래 모델링은 청소년기 정체성 형성에 직결되며, 행동의 지속 동기로 작용한다.
 </t>
           </r>
           <r>
@@ -2652,12 +3045,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>기존 [[C-2]] 부모 AI 또래 비교는 평균값 통계. 개별 사례 스토리 큐레이션으로 결이 다르다.</t>
+            <t>기존 부모 AI 어시스턴트의 또래 비교가 평균값 통계라면, 본 아이디어는 개별 사례 스토리 큐레이션이라는 점에서 결이 다르다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="28" ht="130" customHeight="1">
+    <row r="28" ht="104" customHeight="1">
       <c r="A28" s="17" t="inlineStr">
         <is>
           <t>D-1</t>
@@ -2665,17 +3058,17 @@
       </c>
       <c r="B28" s="18" t="inlineStr">
         <is>
-          <t>D. 권한 이양·성장 시스템</t>
+          <t>D. 권한 이양·성장</t>
         </is>
       </c>
       <c r="C28" s="19" t="inlineStr">
         <is>
-          <t>자녀 금융 신용 점수 시스템</t>
+          <t>자녀 금융 신용 점수</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
         <is>
-          <t>저축률·목표 달성률·부모 약속 이행률 기반 점수 → 점수 상승 시 자율 한도 자동 확대</t>
+          <t>저축률·목표 달성률·약속 이행률 기반 신용 점수와 자율 한도 자동 확대</t>
         </is>
       </c>
       <c r="E28" s="21" t="inlineStr">
@@ -2695,13 +3088,53 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>저축률, 목표 달성률, 부모와의 약속 이행률을 종합한 "금융 신용 점수"를 계산한다. 점수가 높아지면 자율 한도가 자동으로 확대된다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F28" s="21" t="inlineStr"/>
+            <t xml:space="preserve">자녀의 저축률·목표 달성률·부모 약속 이행률 등을 종합한 금융 신용 점수가 산출된다. 점수 상승 시 자율 소비·투자 한도가 자동으로 확대된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 자녀의 저축·소비·약속 이행 데이터가 점수에 누적 반영된다.
+2. 점수가 임계치를 넘으면 자율 한도가 자동 확대된다.
+3. 성년 도달 시 누적 점수가 하나은행 금리 우대 등 실제 혜택과 연계된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F28" s="21" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>권한 확대가 부모의 자의적 판단이 아닌 데이터 기반으로 이루어진다. 자녀의 행동이 정량 평가되어 권한과 책임의 비례 관계가 명확해진다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="29" ht="130" customHeight="1">
+    <row r="29" ht="104" customHeight="1">
       <c r="A29" s="17" t="inlineStr">
         <is>
           <t>D-2</t>
@@ -2709,17 +3142,17 @@
       </c>
       <c r="B29" s="18" t="inlineStr">
         <is>
-          <t>D. 권한 이양·성장 시스템</t>
+          <t>D. 권한 이양·성장</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>부모-자녀 금융 계약서 기능</t>
+          <t>부모-자녀 금융 계약서</t>
         </is>
       </c>
       <c r="D29" s="20" t="inlineStr">
         <is>
-          <t>공식 약속을 앱에 기록 — 달성하면 다음 권한이 열림</t>
+          <t>부모와 자녀 간의 금융 약속을 공식 문서로 기록</t>
         </is>
       </c>
       <c r="E29" s="21" t="inlineStr">
@@ -2739,11 +3172,51 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>"네가 몇 살까지 이만큼 모으면 다음부터는 용돈을 6개월에 한 번 목돈으로 줄게" — 구두 약속이 아닌 앱에 공식으로 기록된 계약서.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F29" s="21" t="inlineStr"/>
+            <t xml:space="preserve">"네가 OO세까지 OO원을 모으면 다음부터 용돈을 6개월에 한 번 목돈으로 지급한다" 형태의 부모-자녀 약속이 공식 계약서로 기록된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 부모와 자녀가 함께 약속 조건을 입력한다.
+2. 양측이 디지털 서명하면 계약서가 발효된다.
+3. 조건 충족 시점에 자동으로 약속 이행 절차가 실행된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F29" s="21" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>암묵적 약속이 명시적 문서로 전환되어 양측의 신뢰와 책임이 강화된다. 자녀에게는 첫 계약 경험으로 작용한다.</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="30" ht="104" customHeight="1">
       <c r="A30" s="17" t="inlineStr">
@@ -2753,17 +3226,17 @@
       </c>
       <c r="B30" s="18" t="inlineStr">
         <is>
-          <t>D. 권한 이양·성장 시스템</t>
+          <t>D. 권한 이양·성장</t>
         </is>
       </c>
       <c r="C30" s="19" t="inlineStr">
         <is>
-          <t>연간 용돈 일괄 지급 전환 자격</t>
+          <t>연간 용돈 일괄 지급 자격</t>
         </is>
       </c>
       <c r="D30" s="20" t="inlineStr">
         <is>
-          <t>금융 퀴즈 + 신용 점수 + 계약 이행 기반으로 자격 심사 → 통과 시 연 단위 목돈 전환</t>
+          <t>금융 퀴즈·신용 점수·계약 이행 기반 자격 심사</t>
         </is>
       </c>
       <c r="E30" s="21" t="inlineStr">
@@ -2783,13 +3256,53 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>일정 조건을 충족하면 용돈 지급 방식을 일/주/월 단위에서 분기/연 단위 목돈으로 전환할 수 있다. "같은 돈이지만 더 오래 굴러요"라는 장기 관점 훈련.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F30" s="21" t="inlineStr"/>
+            <t xml:space="preserve">금융 퀴즈, 신용 점수, 계약 이행 이력을 종합한 자격 심사를 통과한 자녀에게 용돈이 연 단위 목돈으로 일괄 지급된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 자녀가 금융 퀴즈에 응시한다.
+2. 신용 점수와 계약 이행 이력이 자동 집계된다.
+3. 자격 통과 시 부모는 연 단위 일괄 지급 옵션을 활성화할 수 있다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F30" s="21" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>단순 용돈 수령에서 자기 자금 관리로 권한이 이양된다. 일괄 지급된 자금을 12개월 동안 분배·운용하는 경험이 자산 관리 역량으로 누적된다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="31" ht="156" customHeight="1">
+    <row r="31" ht="104" customHeight="1">
       <c r="A31" s="17" t="inlineStr">
         <is>
           <t>D-4</t>
@@ -2797,7 +3310,7 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>D. 권한 이양·성장 시스템</t>
+          <t>D. 권한 이양·성장</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
@@ -2807,7 +3320,7 @@
       </c>
       <c r="D31" s="20" t="inlineStr">
         <is>
-          <t>나이 들수록 화면이 복잡해짐 — 19세에는 완전한 자산 관리 화면</t>
+          <t>연령에 따른 메인 화면 정보 복잡도 단계적 확장</t>
         </is>
       </c>
       <c r="E31" s="21" t="inlineStr">
@@ -2827,11 +3340,51 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>"이 화면 변화를 만들어내는 서비스가 돼야 한다" — 나이에 따라 앱 화면 자체가 달라진다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F31" s="21" t="inlineStr"/>
+            <t xml:space="preserve">어린 시절에는 저금통과 용돈 요청 중심의 단순한 화면이, 성장과 함께 자산·주식·투자 방법 등 복잡한 정보가 점진적으로 노출된다. 19세에는 완전한 자산 관리 화면으로 전환된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 연령·학제·신용 점수에 따라 화면 구성 단계가 자동 전환된다.
+2. 각 단계에서 새 기능이 단계적으로 노출된다.
+3. 전환 시 레벨업 애니메이션과 안내 카드가 제공된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F31" s="21" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>복잡도 증가가 자녀의 인지 발달과 보조를 맞춘다. 동일한 앱 안에서 18년의 성장 경험이 시각적으로 형성된다.</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="32" ht="104" customHeight="1">
       <c r="A32" s="17" t="inlineStr">
@@ -2841,17 +3394,17 @@
       </c>
       <c r="B32" s="18" t="inlineStr">
         <is>
-          <t>D. 권한 이양·성장 시스템</t>
+          <t>D. 권한 이양·성장</t>
         </is>
       </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
-          <t>제안 투표 기능 (매칭금 배분 자녀 참여)</t>
+          <t>제안 투표 (매칭금 배분 자녀 참여)</t>
         </is>
       </c>
       <c r="D32" s="20" t="inlineStr">
         <is>
-          <t>매칭금 일부를 자녀가 제안·투표하여 배분</t>
+          <t>매칭금 일부 배분에 대한 자녀 직접 제안·투표</t>
         </is>
       </c>
       <c r="E32" s="21" t="inlineStr">
@@ -2871,13 +3424,53 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>매칭금의 일부를 어떻게 배분할지 자녀가 직접 제안하고 투표할 수 있다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F32" s="21" t="inlineStr"/>
+            <t xml:space="preserve">부모의 매칭금 일부를 자녀가 어떻게 배분할지 제안하고 투표한다. "네 한 표가 이번 달 매칭금의 30%를 움직인다"는 메시지로 참여 동기가 강화된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 이번 달 매칭금 중 자녀 결정권 비율이 사전 합의된다.
+2. 자녀가 배분 방식을 제안하고 가족 투표가 이루어진다.
+3. 투표 결과에 따라 매칭금이 자동 배분된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F32" s="21" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>수동적 수령자가 아닌 능동적 의사결정자로 자녀의 역할이 전환된다. 자금에 대한 주인 의식이 형성된다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="33" ht="156" customHeight="1">
+    <row r="33" ht="104" customHeight="1">
       <c r="A33" s="17" t="inlineStr">
         <is>
           <t>D-6</t>
@@ -2885,7 +3478,7 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>D. 권한 이양·성장 시스템</t>
+          <t>D. 권한 이양·성장</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
@@ -2895,7 +3488,7 @@
       </c>
       <c r="D33" s="20" t="inlineStr">
         <is>
-          <t>관찰자→선택자→제안자→운용자→독립견습 단계 전환 구조</t>
+          <t>관찰자→선택자→제안자→운용자→독립견습 5단계 자율성 이양</t>
         </is>
       </c>
       <c r="E33" s="21" t="inlineStr">
@@ -2915,11 +3508,51 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>자녀의 금융 자율성이 단계적으로 확대되는 5단계 프레임. 각 단계에서 자녀의 권한 범위가 자동으로 확대된다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F33" s="21" t="inlineStr"/>
+            <t xml:space="preserve">관찰자, 선택자, 제안자, 운용자, 독립견습의 5단계로 자녀의 자율성이 이양된다. 연령·학제·부모 판단의 3축으로 단계 전환이 결정되며, 각 단계에서 권한 범위가 자동 확대된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 현재 단계에 따라 자녀의 권한 범위와 기본값이 다르게 적용된다.
+2. 전환 조건(연령·학제·부모 판단) 충족 시 다음 단계가 활성화된다.
+3. 단계 전환 시 새 권한과 책임이 안내된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F33" s="21" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>권한 이양이 일회성 이벤트가 아닌 단계적 구조로 정착한다. 자녀의 성장 단계에 맞는 자율성이 보장된다.</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="34" ht="104" customHeight="1">
       <c r="A34" s="17" t="inlineStr">
@@ -2929,7 +3562,7 @@
       </c>
       <c r="B34" s="18" t="inlineStr">
         <is>
-          <t>D. 권한 이양·성장 시스템</t>
+          <t>D. 권한 이양·성장</t>
         </is>
       </c>
       <c r="C34" s="19" t="inlineStr">
@@ -2939,7 +3572,7 @@
       </c>
       <c r="D34" s="20" t="inlineStr">
         <is>
-          <t>진학 등 전환 시 한도·주기 자동 재제안 + 레벨업 애니메이션</t>
+          <t>진학 등 전환 시점의 한도·주기 자동 재제안과 레벨업 연출</t>
         </is>
       </c>
       <c r="E34" s="21" t="inlineStr">
@@ -2959,13 +3592,53 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>학제 전환(초→중→고)이나 단계 이동 시, "새로운 단계를 위한 설정 위저드"와 함께 레벨업 애니메이션을 제공한다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F34" s="21" t="inlineStr"/>
+            <t xml:space="preserve">진학 등 학제 전환 시점에 자동으로 한도와 주기가 재제안된다. "중학생이 된 너, 새로운 권한이 열렸다" 형태의 레벨업 애니메이션이 제공된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 학제 전환 시점이 자동 감지된다.
+2. 새 단계의 한도·주기가 자동 재제안된다.
+3. 레벨업 페이지에서 새 권한이 시각적으로 안내된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F34" s="21" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>권한 확대가 게임의 레벨업 경험으로 재구성된다. 학제 전환이 추가 사용 동기로 작용한다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="35" ht="351" customHeight="1">
+    <row r="35" ht="156" customHeight="1">
       <c r="A35" s="17" t="inlineStr">
         <is>
           <t>D-8</t>
@@ -2973,7 +3646,7 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>D. 권한 이양·성장 시스템</t>
+          <t>D. 권한 이양·성장</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
@@ -2983,7 +3656,7 @@
       </c>
       <c r="D35" s="20" t="inlineStr">
         <is>
-          <t>부모 자산을 증여 전 "자녀가 의사결정"하는 영역으로 지정 → 일정 기간 운용 결과 통과 시 명의 이전</t>
+          <t>부모 자산 일부에 자녀 의사결정권만 위임 → 결과 통과 시 명의 이전</t>
         </is>
       </c>
       <c r="E35" s="21" t="inlineStr">
@@ -3003,7 +3676,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">부자조차 19%가 "상속·증여 자산의 관리·운용 자신감 부족"을 우려한다. 동시에 68%는 "재산 많이 물려줄수록 자녀에게 성장 기회 생긴다"고 답했다. 두 우려를 동시에 해소하는 단계가 "증여 전 시범 운용 기간"이다.
+            <t xml:space="preserve">한국 부자의 19%는 자녀의 운용 자신감 부족을, 68%는 "많이 물려줄수록 성장 기회가 생긴다"는 인식을 동시에 가지고 있다. 두 우려를 동시에 해소하는 단계로 증여 전 시범 운용 기간이 도입된다.
 </t>
           </r>
           <r>
@@ -3021,14 +3694,10 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">1. 부모가 자산 일부(예: 1,000만원)를 시범 운용 영역으로 지정 (소유는 끝까지 부모)
-2. 자녀가 매수/매도 의사결정을 제안 → 부모가 1탭 승인/거부
-3. 운영 기간(예: 6개월) + 운용 결과 기준
-- 수익률 임계치(예: -10% 이상)
-- 의사결정 빈도 (월 N회 이상)
-- 학습 미션 이행률 (N% 이상)
-4. 통과 시 해당 자산을 비과세 한도 내 일반 증여로 명의 이전 ([[A-13]] 흐름과 자동 연결)
-5. 미통과 시 부모 의사로 시범 기간 연장 또는 회수
+            <t xml:space="preserve">1. 부모가 자산 일부(예: 1,000만원)를 시범 운용 영역으로 지정한다(소유권은 부모 보유).
+2. 자녀가 매수·매도 의사결정을 제안하면 부모가 1-탭으로 승인 또는 거부한다.
+3. 운영 기간(예: 6개월) 종료 시점에 수익률·결정 빈도·학습 미션 이행률이 자동 평가된다.
+4. 기준 통과 시 비과세 한도 내 일반 증여로 명의가 이전된다.
 </t>
           </r>
           <r>
@@ -3046,7 +3715,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>정식 신탁상품이 아니라 부모 계좌 안의 가상 영역이다. 명의·소유는 끝까지 부모가 보유하고, 자녀에게는 의사결정 권한만 위임된다. 명의 이전이 일어나는 시점에 일반 증여로 처리되어 비과세 한도가 적용된다. 추가 신탁 계약 없이 앱 내부 권한 분리만으로 운용 가능.</t>
+            <t>정식 신탁상품이 아닌 부모 계좌 안의 가상 영역으로 권한만 분리된다. 명의 이전 시점에 일반 증여로 처리되어 비과세 한도가 적용된다. 추가 신탁 계약 없이 앱 내부 권한 분리만으로 운용이 가능하다.</t>
           </r>
         </is>
       </c>
@@ -3067,9 +3736,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">부모: "자녀에게 운용을 맡기기 불안하다"는 우려를 6개월 시범으로 해소
-자녀: 진짜 자산을 운용하는 경험 — 모의투자보다 압박감과 학습 효과가 크다
-하나은행: 증여 전 단계에서 부모-자녀 모두를 앱에 묶어두는 지속 사용 유인
+            <t xml:space="preserve">부모의 운용 자신감 부족 우려가 시범 기간을 통해 해소된다. 자녀는 모의투자보다 실효성 있는 운용 경험을 누적한다.
 </t>
           </r>
           <r>
@@ -3087,12 +3754,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>기존 [[D-1]] 자녀 금융 신용 점수는 자녀 자체 자산의 권한 확대. 증여 직전 단계로, 부모 자산의 운용 의사결정만 빌려주는 별도 트랙이다.</t>
+            <t>기존 자녀 금융 신용 점수가 자녀 자체 자산의 권한 확대 구조라면, 본 아이디어는 증여 직전 단계에서 부모 자산의 운용 의사결정만 빌려주는 별도 트랙이다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="36" ht="143" customHeight="1">
+    <row r="36" ht="104" customHeight="1">
       <c r="A36" s="22" t="inlineStr">
         <is>
           <t>E-1</t>
@@ -3100,7 +3767,7 @@
       </c>
       <c r="B36" s="23" t="inlineStr">
         <is>
-          <t>E. 게임화·보상·커뮤니케이션</t>
+          <t>E. 게임화·보상</t>
         </is>
       </c>
       <c r="C36" s="24" t="inlineStr">
@@ -3110,7 +3777,7 @@
       </c>
       <c r="D36" s="25" t="inlineStr">
         <is>
-          <t>달성 기반 배지 수집 + 칭호 부여. 금융 성장에 연동</t>
+          <t>달성 기반 배지 수집과 칭호 부여</t>
         </is>
       </c>
       <c r="E36" s="26" t="inlineStr">
@@ -3130,13 +3797,53 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>금융 달성 기반으로 배지를 수집하고 칭호를 얻는다. 단순한 트로피가 아니라 실제 혜택과 연결된다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F36" s="26" t="inlineStr"/>
+            <t xml:space="preserve">자산 형성과 행동 달성 단계에 따라 배지가 부여되고 칭호가 표시된다. "100만 장자", "16살 기준 일론 머스크보다 부자" 등 자녀의 흥미를 자극하는 칭호가 금융적 성장에 연동된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 달성 조건이 충족되면 배지가 자동 발급된다.
+2. 특정 배지 조합이나 임계치 달성 시 칭호가 부여된다.
+3. 획득한 배지·칭호는 프로필에 노출되고 친구에게 공유될 수 있다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F36" s="26" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>수집욕을 자극하는 마이크로 인터랙션이 행동 동기로 전환된다. 칭호는 자녀의 자산 성장 정체성을 강화한다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="37" ht="117" customHeight="1">
+    <row r="37" ht="104" customHeight="1">
       <c r="A37" s="22" t="inlineStr">
         <is>
           <t>E-2</t>
@@ -3144,17 +3851,17 @@
       </c>
       <c r="B37" s="23" t="inlineStr">
         <is>
-          <t>E. 게임화·보상·커뮤니케이션</t>
+          <t>E. 게임화·보상</t>
         </is>
       </c>
       <c r="C37" s="24" t="inlineStr">
         <is>
-          <t>프로필 커스터마이징 (아바타·캐릭터)</t>
+          <t>프로필 커스터마이징</t>
         </is>
       </c>
       <c r="D37" s="25" t="inlineStr">
         <is>
-          <t>모은 자산이 없을 때는 심플 → 돈 많이 모으면 리치해지는 아이콘 진화</t>
+          <t>자산 규모에 따라 아이콘이 진화하는 프로필</t>
         </is>
       </c>
       <c r="E37" s="26" t="inlineStr">
@@ -3174,13 +3881,53 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>카카오톡처럼 자기 프로필을 꾸밀 수 있다. 단, 자산이 늘어날수록 아바타/캐릭터가 자동으로 "리치"해진다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F37" s="26" t="inlineStr"/>
+            <t xml:space="preserve">카카오톡처럼 자기 프로필을 꾸밀 수 있다. 자산이 적을 때는 단순한 아이콘으로 시작해 자산 누적과 함께 점차 풍요로운 모습으로 진화한다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 자녀가 아바타와 배경을 선택해 프로필을 꾸민다.
+2. 총 자산 규모에 따라 아이콘이 자동으로 진화한다.
+3. 친구와 프로필을 공유하거나 비교할 수 있다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F37" s="26" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>자산 성장이 시각적 정체성의 일부가 되어 이탈 비용이 높아진다. 자기 표현 욕구가 자산 형성 동기와 결합한다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="38" ht="117" customHeight="1">
+    <row r="38" ht="104" customHeight="1">
       <c r="A38" s="22" t="inlineStr">
         <is>
           <t>E-4</t>
@@ -3188,7 +3935,7 @@
       </c>
       <c r="B38" s="23" t="inlineStr">
         <is>
-          <t>E. 게임화·보상·커뮤니케이션</t>
+          <t>E. 게임화·보상</t>
         </is>
       </c>
       <c r="C38" s="24" t="inlineStr">
@@ -3198,7 +3945,7 @@
       </c>
       <c r="D38" s="25" t="inlineStr">
         <is>
-          <t>자산 성장 과정의 마일스톤을 카드로 수집</t>
+          <t>자산 성장 마일스톤을 카드 형태로 수집</t>
         </is>
       </c>
       <c r="E38" s="26" t="inlineStr">
@@ -3218,11 +3965,51 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>자산 성장의 주요 순간마다 수집형 카드가 발급된다. 카카오톡 선물하기 이력처럼 모이고 쌓인다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F38" s="26" t="inlineStr"/>
+            <t xml:space="preserve">"첫 주식 수익", "100만 원 돌파" 등 자산 성장의 주요 마일스톤이 카드 형태로 발급되어 수집된다. 카카오톡 선물하기 이력처럼 시각적 컬렉션으로 누적된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 마일스톤 달성 시 카드가 자동 발급된다.
+2. 수집된 카드는 갤러리에 누적 보관된다.
+3. 특정 카드 조합 달성 시 추가 보상이 지급된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F38" s="26" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>자산 성장의 무형 성과가 시각적 자산으로 전환된다. 수집욕이 장기 사용 동기로 작용한다.</t>
+          </r>
+        </is>
+      </c>
     </row>
     <row r="39" ht="104" customHeight="1">
       <c r="A39" s="22" t="inlineStr">
@@ -3232,17 +4019,17 @@
       </c>
       <c r="B39" s="23" t="inlineStr">
         <is>
-          <t>E. 게임화·보상·커뮤니케이션</t>
+          <t>E. 게임화·보상</t>
         </is>
       </c>
       <c r="C39" s="24" t="inlineStr">
         <is>
-          <t>연속 달성 보상 구조</t>
+          <t>연속 달성 보상</t>
         </is>
       </c>
       <c r="D39" s="25" t="inlineStr">
         <is>
-          <t>연속 저축/미션 달성 시 보상. 부모가 미리 보상금을 걸어두는 구조</t>
+          <t>연속 저축·미션 달성 시 보상 적립</t>
         </is>
       </c>
       <c r="E39" s="26" t="inlineStr">
@@ -3262,13 +4049,53 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>연속으로 저축 또는 미션을 달성하면 보상이 제공된다. 부모가 미리 보상금을 예약해두고, 자녀가 달성하면 수령하는 구조.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F39" s="26" t="inlineStr"/>
+            <t xml:space="preserve">연속 저축이나 미션 달성 시 추가 보상이 적립된다. 부모가 매칭 제안 시점에 보상금을 미리 걸어두고, 자녀가 달성하면 자동으로 수령한다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 부모가 보상금과 달성 조건을 사전 등록한다.
+2. 자녀가 조건 달성 시 보상이 자동 지급된다.
+3. 연속 달성 횟수에 따라 보상 배율이 상향된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F39" s="26" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>행동 연속성이 명시적 보상과 결합되어 습관 형성이 가속된다. 부모의 약속이 앱을 통해 자동 집행되어 신뢰가 강화된다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="40" ht="143" customHeight="1">
+    <row r="40" ht="104" customHeight="1">
       <c r="A40" s="27" t="inlineStr">
         <is>
           <t>F-1</t>
@@ -3276,17 +4103,17 @@
       </c>
       <c r="B40" s="28" t="inlineStr">
         <is>
-          <t>F. 진입·리텐션 관련</t>
+          <t>F. 진입·리텐션</t>
         </is>
       </c>
       <c r="C40" s="29" t="inlineStr">
         <is>
-          <t>부모 반복 트리거 5가지</t>
+          <t>부모 반복 트리거 5종</t>
         </is>
       </c>
       <c r="D40" s="30" t="inlineStr">
         <is>
-          <t>부모가 앱을 반복 사용하게 만드는 5가지 핵심 훅</t>
+          <t>자녀 인사이트·자산 통합·성장 리포트·세무 도구·성과 알림</t>
         </is>
       </c>
       <c r="E40" s="31" t="inlineStr">
@@ -3306,7 +4133,29 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>부모가 아이부자를 반복해서 열게 만드는 5가지 핵심 리텐션 훅.</t>
+            <t xml:space="preserve">부모의 반복 사용을 유도하는 5가지 핵심 트리거가 제공된다. ① 자녀 맞춤 인사이트 피드, ② 가족 자산 통합 뷰, ③ 분기 자녀 재무 성장 리포트, ④ 세무·증여 전략 도구, ⑤ 자녀 성과 알림.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 자녀의 행동 데이터를 기반으로 인사이트 피드가 자동 생성된다.
+2. 가족 전체 자산이 통합 뷰로 시각화된다.
+3. 분기별로 자녀의 재무 성장 리포트가 발행된다.
+4. 세무·증여 관련 의사결정 도구가 제공된다.
+5. 자녀의 주요 성과가 실시간 알림으로 전달된다.</t>
           </r>
         </is>
       </c>
@@ -3327,13 +4176,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>- 각 훅은 독립적으로 앱 오픈 트리거가 됨
-- 주간·분기·이벤트 기반으로 다양한 주기 커버</t>
+            <t>부모의 반복 진입 동기가 다층화된다. 한 가지 트리거가 약해도 다른 트리거로 보완되어 장기 리텐션이 안정화된다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="41" ht="156" customHeight="1">
+    <row r="41" ht="104" customHeight="1">
       <c r="A41" s="27" t="inlineStr">
         <is>
           <t>F-2</t>
@@ -3341,17 +4189,17 @@
       </c>
       <c r="B41" s="28" t="inlineStr">
         <is>
-          <t>F. 진입·리텐션 관련</t>
+          <t>F. 진입·리텐션</t>
         </is>
       </c>
       <c r="C41" s="29" t="inlineStr">
         <is>
-          <t>7가지 이벤트 트리거</t>
+          <t>조건·이벤트 트리거 7종</t>
         </is>
       </c>
       <c r="D41" s="30" t="inlineStr">
         <is>
-          <t>세뱃돈 시즌, 절약 감지, 배당 발생, 학제 전환 등 자연 발생 트리거 7가지</t>
+          <t>외부 이벤트와 연동된 진입 트리거 7개</t>
         </is>
       </c>
       <c r="E41" s="31" t="inlineStr">
@@ -3371,13 +4219,53 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>일상 속 자연스러운 이벤트를 앱 재진입 트리거로 활용하는 7가지 시나리오.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F41" s="31" t="inlineStr"/>
+            <t xml:space="preserve">사용자의 외부 이벤트와 연동된 7가지 진입 트리거가 운영된다. 세뱃돈 시즌, 월말·연말, 절약 감지, 배당·이자 발생, 학제 전환, 경제 뉴스, 조부모·친척 송금 시점이 포함된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 각 이벤트 발생 시점이 시스템에 자동 감지된다.
+2. 이벤트 맥락에 맞는 추천 알림이 발송된다.
+3. 알림 클릭 시 이벤트에 최적화된 액션 화면으로 이동한다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F41" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>사용자의 일상 흐름과 동기화된 진입 동기가 형성된다. 외부 이벤트가 곧 앱 사용의 트리거가 된다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="42" ht="156" customHeight="1">
+    <row r="42" ht="104" customHeight="1">
       <c r="A42" s="27" t="inlineStr">
         <is>
           <t>F-3</t>
@@ -3385,17 +4273,17 @@
       </c>
       <c r="B42" s="28" t="inlineStr">
         <is>
-          <t>F. 진입·리텐션 관련</t>
+          <t>F. 진입·리텐션</t>
         </is>
       </c>
       <c r="C42" s="29" t="inlineStr">
         <is>
-          <t>중학교 이탈 방어 5가지 장치</t>
+          <t>중학교 이탈 방어 5종</t>
         </is>
       </c>
       <c r="D42" s="30" t="inlineStr">
         <is>
-          <t>13~15세 최고 이탈 구간을 막는 5가지 UX 설계</t>
+          <t>감시감 제거·비교 전환·기여감·현실 효용·소셜 방어 UX</t>
         </is>
       </c>
       <c r="E42" s="31" t="inlineStr">
@@ -3415,13 +4303,55 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>13~15세(S3 구간)는 또래 문화가 정점이고 아이부자와 가장 크게 충돌하는 시기다. 5가지 방어 장치로 이탈을 막는다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F42" s="31" t="inlineStr"/>
+            <t xml:space="preserve">중학교 진학기에 발생하는 자녀 이탈을 방어하는 5가지 장치가 적용된다. ① 감시감 제거(소비 세부의 부모 노출 기본 OFF), ② 또래에서 가족 단위로 비교 전환, ③ 기여감 부여, ④ 현실 효용 강조, ⑤ 소셜 방어 UX 언어.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 중학교 입학 시점이 감지되면 감시감 제거 모드가 자동 활성화된다.
+2. 비교 지표가 또래에서 가족 단위로 전환된다.
+3. 자녀의 기여 활동이 우선 노출된다.
+4. 현실 효용 중심의 콘텐츠가 큐레이션된다.
+5. 소셜 친화적 UX 언어가 적용된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F42" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>사춘기 자율성 욕구와 충돌하지 않는 형태로 앱 사용이 지속된다. 중학교 이탈 위험이 구조적으로 완화된다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="43" ht="143" customHeight="1">
+    <row r="43" ht="104" customHeight="1">
       <c r="A43" s="27" t="inlineStr">
         <is>
           <t>F-4</t>
@@ -3429,17 +4359,17 @@
       </c>
       <c r="B43" s="28" t="inlineStr">
         <is>
-          <t>F. 진입·리텐션 관련</t>
+          <t>F. 진입·리텐션</t>
         </is>
       </c>
       <c r="C43" s="29" t="inlineStr">
         <is>
-          <t>사전 허락 리스트 (카테고리별 한도)</t>
+          <t>사전 허락 리스트</t>
         </is>
       </c>
       <c r="D43" s="30" t="inlineStr">
         <is>
-          <t>카테고리별 소비 한도를 부모가 사전 지정 — 민법 제6조 프레임 활용</t>
+          <t>민법 제6조 프레임 기반 카테고리별 사전 한도 지정</t>
         </is>
       </c>
       <c r="E43" s="31" t="inlineStr">
@@ -3459,13 +4389,53 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>편의점, 문구, 학용품 등 카테고리별 소비 한도를 부모가 사전에 지정해두면, 그 안에서 자녀가 자유롭게 소비할 수 있다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F43" s="31" t="inlineStr"/>
+            <t xml:space="preserve">편의점, 문구, 학용품 등 카테고리별 소비 한도가 부모에 의해 사전에 지정된다. 민법 제6조의 "처분을 허락한 재산" 프레임을 응용한 구조다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 부모가 카테고리별 월별 한도를 사전 설정한다.
+2. 자녀의 소비가 자동으로 카테고리에 분류된다.
+3. 한도 내 소비는 자유롭게, 초과 시 부모 승인 알림이 발송된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F43" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>건별 승인 부담이 사라지고 자녀의 자율 영역이 명시적으로 정의된다. 법적 프레임을 차용해 부모의 권한 행사가 정당화된다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="44" ht="130" customHeight="1">
+    <row r="44" ht="104" customHeight="1">
       <c r="A44" s="27" t="inlineStr">
         <is>
           <t>F-5</t>
@@ -3473,7 +4443,7 @@
       </c>
       <c r="B44" s="28" t="inlineStr">
         <is>
-          <t>F. 진입·리텐션 관련</t>
+          <t>F. 진입·리텐션</t>
         </is>
       </c>
       <c r="C44" s="29" t="inlineStr">
@@ -3483,7 +4453,7 @@
       </c>
       <c r="D44" s="30" t="inlineStr">
         <is>
-          <t>월 1회 가족이 함께 투자 현황을 리뷰하는 템플릿 제공</t>
+          <t>월 1회 가족 투자 현황 리뷰 진행 템플릿</t>
         </is>
       </c>
       <c r="E44" s="31" t="inlineStr">
@@ -3503,7 +4473,27 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>월 1회 가족이 함께 앉아 투자 현황을 리뷰하는 구조화된 템플릿을 제공한다. 부모 포트폴리오 일부를 자녀에게 공개해 교육 소재로 활용한다.</t>
+            <t xml:space="preserve">월 1회 가족 구성원이 함께 투자 현황을 리뷰할 수 있도록 회의 진행 템플릿이 제공된다. 부모의 포트폴리오 일부를 교육 소재로 공개하는 옵션이 포함된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 월 1회 가족 회의 일정이 사전 설정된다.
+2. 회의 시점에 자녀·부모 자산 리포트가 자동 생성된다.
+3. 토론 주제와 의사결정 항목이 템플릿으로 제공된다.</t>
           </r>
         </is>
       </c>
@@ -3524,14 +4514,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>- 부모가 먼저 자산을 공개 → 자녀의 개방 동기 강화
-- 판단·평가 없이 현황 공유 → 심리적 안전감
-- 월 1회의 리추얼 → 금융 대화를 가족 문화로</t>
+            <t>투자가 개인 활동이 아닌 가족 단위 활동으로 재구성된다. 부모의 실제 투자 행태가 자녀의 학습 자료로 활용된다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="45" ht="143" customHeight="1">
+    <row r="45" ht="104" customHeight="1">
       <c r="A45" s="27" t="inlineStr">
         <is>
           <t>F-6</t>
@@ -3539,7 +4527,7 @@
       </c>
       <c r="B45" s="28" t="inlineStr">
         <is>
-          <t>F. 진입·리텐션 관련</t>
+          <t>F. 진입·리텐션</t>
         </is>
       </c>
       <c r="C45" s="29" t="inlineStr">
@@ -3549,7 +4537,7 @@
       </c>
       <c r="D45" s="30" t="inlineStr">
         <is>
-          <t>10년 단위 비과세 한도 누계 관리, 증여 신고 시뮬레이션, 세무사 제휴 연결</t>
+          <t>10년 단위 비과세 한도 추적과 증여 시뮬레이션, 세무사 제휴 연결</t>
         </is>
       </c>
       <c r="E45" s="31" t="inlineStr">
@@ -3569,7 +4557,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">비과세 증여 한도(미성년자 2천만원, 10년 주기)를 추적하고, 증여 신고를 시뮬레이션하며, 필요시 세무사와 연결하는 서비스.
+            <t xml:space="preserve">비과세 증여 한도(미성년 10년 2,000만원)가 자동 추적되고, 증여 신고 시뮬레이션이 제공된다. 복잡한 케이스는 제휴 세무사와 연결된다.
 </t>
           </r>
           <r>
@@ -3587,10 +4575,10 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 한도 잔여량 추적: "현재 증여 누계: 1,200만원 / 한도 2,000만원. 잔여 800만원"
-2. 증여 시뮬레이션: "지금 300만원 더 증여하면 증여세 0원, 이 방식으로 신고하세요"
-3. 타이밍 알림: "10년 한도 리셋까지 D-365"
-4. 세무사 연결: 복잡한 케이스는 제휴 세무사에게 바로 연결</t>
+            <t>1. 현재 증여 누계와 한도 잔여량이 상시 표시된다.
+2. 추가 증여 시 절세 시나리오가 시뮬레이션된다.
+3. 한도 리셋 시점이 D-Day로 안내된다.
+4. 복잡한 케이스는 제휴 세무사와의 1-탭 연결을 지원한다.</t>
           </r>
         </is>
       </c>
@@ -3611,13 +4599,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>- 증여를 체계적으로 관리하고 싶은 부모 → 아이부자에 장기 로열티
-- 고자산 부모층에 특히 강력한 훅</t>
+            <t>증여 의사결정의 정보 비대칭이 해소된다. 고자산 부모층의 장기 로열티를 형성하는 강력한 훅이 된다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="46" ht="130" customHeight="1">
+    <row r="46" ht="104" customHeight="1">
       <c r="A46" s="27" t="inlineStr">
         <is>
           <t>F-7</t>
@@ -3625,7 +4612,7 @@
       </c>
       <c r="B46" s="28" t="inlineStr">
         <is>
-          <t>F. 진입·리텐션 관련</t>
+          <t>F. 진입·리텐션</t>
         </is>
       </c>
       <c r="C46" s="29" t="inlineStr">
@@ -3635,7 +4622,7 @@
       </c>
       <c r="D46" s="30" t="inlineStr">
         <is>
-          <t>성년 도달 시 하나원큐로 자동 이관 + 18년의 여정을 담은 졸업 페이지</t>
+          <t>성년 도달 시 하나원큐 자동 이관과 졸업 페이지</t>
         </is>
       </c>
       <c r="E46" s="31" t="inlineStr">
@@ -3655,13 +4642,53 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>성년(18세)이 되는 날, 아이부자에서 하나원큐로 자동 이관이 이루어지며, 지금까지의 금융 여정을 담은 졸업 페이지가 제공된다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F46" s="31" t="inlineStr"/>
+            <t xml:space="preserve">자녀가 성년에 도달하면 하나원큐로 자동 이관되며 "18년의 습관이 이제 너의 시스템이 된다"는 졸업 페이지가 제공된다. 기존 데이터가 완전히 이관된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 성년 도달 시점이 자동 감지된다.
+2. 기존 자산·히스토리·신용 점수가 하나원큐로 완전 이관된다.
+3. 졸업 페이지에서 18년의 여정이 시각적으로 정리된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F46" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>아이부자 종료가 단절이 아닌 다음 단계로의 전환으로 인식된다. 하나은행 성인 상품으로의 자연스러운 지속 사용 유인이 형성된다.</t>
+          </r>
+        </is>
+      </c>
     </row>
-    <row r="47" ht="286" customHeight="1">
+    <row r="47" ht="104" customHeight="1">
       <c r="A47" s="27" t="inlineStr">
         <is>
           <t>F-8</t>
@@ -3669,7 +4696,7 @@
       </c>
       <c r="B47" s="28" t="inlineStr">
         <is>
-          <t>F. 진입·리텐션 관련</t>
+          <t>F. 진입·리텐션</t>
         </is>
       </c>
       <c r="C47" s="29" t="inlineStr">
@@ -3679,7 +4706,7 @@
       </c>
       <c r="D47" s="30" t="inlineStr">
         <is>
-          <t>10년 단위 비과세 한도 사용률을 부모 메인 화면에 상시 노출하는 게이지</t>
+          <t>10년 단위 비과세 한도 사용률을 부모 메인 화면에 상시 게이지로 노출</t>
         </is>
       </c>
       <c r="E47" s="31" t="inlineStr">
@@ -3699,7 +4726,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">한국 부자의 79%가 상속·증여 설계에서 가장 큰 우려로 꼽은 것은 "상속세·증여세 부담"이다. 해법은 비과세 한도(미성년 10년 2,000만원, 성년 5,000만원)를 끝까지 활용하는 것. 그런데 한도는 잊기 쉽고, 시점을 놓치면 그 사이클은 영구히 사라진다.
+            <t xml:space="preserve">한국 부자의 79%가 상속·증여 설계에서 가장 큰 우려로 꼽은 것은 상속세·증여세 부담이다. 비과세 한도를 끝까지 활용하지 않으면 사이클 단위로 한도가 소멸한다는 점에서, 한도 사용률이 부모 메인 화면에 상시 노출된다.
 </t>
           </r>
           <r>
@@ -3717,15 +4744,10 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 부모 메인 화면 상단 게이지 바
-```
-[████████░░░░] 비과세 한도 1,400만원 / 2,000만원 (잔여 600만원)
-다음 리셋 D-365 (2027.04.27)
-```
-2. 한도 만료 90일 전 알림: "12월 31일 만료, 지금 입금 시 N% 절세"
-3. 10년 누계 그래프: 두 사이클을 하나의 타임라인에
-4. 분할 증여 제안: "잔여 600만원, 10·11·12월 분할 시 평가 변동 위험 분산"
-5. [[A-13]] 주식 직접 증여 트리거: 잔여 한도 클릭 → 증여 흐름 진입</t>
+            <t>1. 부모 메인 화면 상단에 비과세 한도 사용률 게이지 바가 상시 표시된다.
+2. 한도 만료 90일 전 자동 알림이 발송된다.
+3. 10년 누계 그래프와 분할 증여 시나리오가 제공된다.
+4. 잔여 한도 클릭 시 주식 직접 증여 흐름으로 즉시 진입할 수 있다.</t>
           </r>
         </is>
       </c>
@@ -3746,7 +4768,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">부자 79%의 1순위 우려를 정면 해소. 한도 미사용 = 손실이라는 감각을 부모 화면 상시 노출로 만든다. 매번 시뮬레이터에 들어가지 않아도 실시간 인지 가능.
+            <t xml:space="preserve">한도 미사용이 곧 손실이라는 감각이 부모의 일상 인지에 자리잡는다. 시뮬레이터에 별도 진입하지 않아도 의사결정 시점이 포착된다.
 </t>
           </r>
           <r>
@@ -3764,12 +4786,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>기존 [[F-6]] 증여 시뮬레이터는 사용자가 진입해야 하는 도구. 상시 노출 게이지로, 진입 없이도 자연스럽게 인식된다.</t>
+            <t>기존 증여 시뮬레이터는 사용자가 직접 진입해야 하는 도구이지만, 본 아이디어는 상시 노출 게이지로서 진입 없이도 인지가 발생한다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="48" ht="312" customHeight="1">
+    <row r="48" ht="104" customHeight="1">
       <c r="A48" s="27" t="inlineStr">
         <is>
           <t>F-9</t>
@@ -3777,7 +4799,7 @@
       </c>
       <c r="B48" s="28" t="inlineStr">
         <is>
-          <t>F. 진입·리텐션 관련</t>
+          <t>F. 진입·리텐션</t>
         </is>
       </c>
       <c r="C48" s="29" t="inlineStr">
@@ -3787,7 +4809,7 @@
       </c>
       <c r="D48" s="30" t="inlineStr">
         <is>
-          <t>조부모-부모-자녀 3대 자산을 한 화면에 — 세대생략 증여까지 시뮬레이션</t>
+          <t>조부모-부모-자녀 3대 자산을 한 화면에, 세대생략 증여까지 포괄</t>
         </is>
       </c>
       <c r="E48" s="31" t="inlineStr">
@@ -3807,7 +4829,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">부의 주 원천이 "상속·증여"인 부자 비중이 2011년 13.7%에서 2023년 20.0%로 상승했다. 한국 부자의 57%는 "자산이전 시점을 분산해 여러 번 증여하는 것이 바람직하다"고 답했다. 자산이전이 더 이상 부모-자녀 1:1이 아니라 가문 단위 60년 곡선이 되고 있다.
+            <t xml:space="preserve">한국 부의 원천 중 상속·증여 비중이 2011년 13.7%에서 2023년 20.0%로 상승했다. 부자의 57%가 시점 분산 증여를 바람직하다고 답했다. 자산이전이 부모-자녀 1:1을 넘어 가문 단위 60년 곡선으로 재구성된다.
 </t>
           </r>
           <r>
@@ -3825,14 +4847,10 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 3대 입력: 조부모(70대), 부모(40대), 자녀(10세)의 현재 자산 입력
-2. 시나리오 비교
-- 시나리오 A (전통 2단계): 조부모 → 부모 → 자녀
-- 시나리오 B (세대생략 증여): 조부모 → 자녀 직접 (30% 할증, 단 30년 이상 단축)
-- 시나리오 C (병행): 조부모 → 손자녀 비과세 한도 + 부모는 보강
-3. 60년 가문 자산 곡선 그래프 (3개 시나리오 동시)
-4. 세금·비과세 한도·증여 시점 자동 최적화 추천
-5. 조부모용 진입 화면 분리 — 손자녀 명의 비과세 한도 잔여 표시</t>
+            <t>1. 조부모, 부모, 자녀의 현재 자산이 입력된다.
+2. 전통 2단계, 세대생략 증여, 병행 시나리오 3종이 비교된다.
+3. 60년 가문 자산 곡선과 세금·비과세 한도 최적화가 자동 계산된다.
+4. 조부모 전용 진입 화면이 별도로 제공된다.</t>
           </r>
         </is>
       </c>
@@ -3853,7 +4871,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">단순 부모-자녀 시뮬을 넘어 가문 단위 사고로 확장. 조부모층을 신규 사용자층으로 끌어들이는 진입 카드가 되며, 세대생략 증여라는 고급 절세 옵션을 가시화한다. 부의 원천에서 상속·증여 비중 증가 트렌드(13.7% → 20%)에 직접 매칭.
+            <t xml:space="preserve">단순 부모-자녀 시뮬을 넘어 가문 단위 사고가 가능해진다. 조부모층이 신규 사용자층으로 유입되며, 세대생략 증여라는 고급 절세 옵션이 가시화된다.
 </t>
           </r>
           <r>
@@ -3871,12 +4889,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>기존 [[F-6]] 증여 시뮬레이터는 부모-자녀 2대. 3대 + 세대생략 증여까지 포괄하는 확장판.</t>
+            <t>기존 증여 시뮬레이터가 부모-자녀 2대를 대상으로 한다면, 본 아이디어는 3대와 세대생략 증여까지 포괄한다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="49" ht="156" customHeight="1">
+    <row r="49" ht="104" customHeight="1">
       <c r="A49" s="32" t="inlineStr">
         <is>
           <t>G-2</t>
@@ -3884,17 +4902,17 @@
       </c>
       <c r="B49" s="33" t="inlineStr">
         <is>
-          <t>G. 행동 전환·정체성 형성</t>
+          <t>G. 행동 전환·정체성</t>
         </is>
       </c>
       <c r="C49" s="34" t="inlineStr">
         <is>
-          <t>투자자 명함 기능</t>
+          <t>투자자 명함</t>
         </is>
       </c>
       <c r="D49" s="35" t="inlineStr">
         <is>
-          <t>나의 투자 프로필을 카드 형태로 자동 생성. 친구에게 공유 가능</t>
+          <t>투자 프로필을 카드 형태로 자동 생성하고 친구에게 공유</t>
         </is>
       </c>
       <c r="E49" s="36" t="inlineStr">
@@ -3914,33 +4932,27 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">투자 프로필을 카드 형태로 자동 생성해, 친구에게 공유할 수 있다. "감시앱"이라는 낙인에서 벗어나 "나 이런 거 하는 앱이야"라는 정체성 도구가 된다.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 참고
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>· 명함 예시
-```
-💼 OO의 투자자 명함
-삼성전자 주주 | SK하이닉스 주주
-첫 투자일: 2027.03.15
-누적 수익: +12,400원 (+8.3%)
-투자 스타일: 장기 적립형
-[친구에게 공유하기]
-```</t>
+            <t xml:space="preserve">자녀의 투자 프로필이 카드 형태로 자동 생성된다. "삼성전자 주주 | 첫 투자일 2027.3.15 | 누적 수익 +12,400원" 등 투자 정체성이 시각화되며 친구에게 공유될 수 있다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 보유 종목·첫 투자일·누적 수익·투자 스타일이 자동 카드화된다.
+2. 친구에게 카드 형태로 공유될 수 있다.
+3. 프로필 카드의 디자인은 자녀가 일부 커스터마이징할 수 있다.</t>
           </r>
         </is>
       </c>
@@ -3961,16 +4973,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>&gt; 투자 경험 → "나는 돈을 키우는 사람"이라는 정체성 형성
-- "나 이런 앱 써" → 소셜 확산
-- 또래 이미지 보호: 부모 감시 도구이 아니라 "투자자가 쓰는 앱"
-- 친구가 보고 "나도 해볼래?" → 바이럴 가입
-- 공유 수 = 브랜드 캠페인 지표로 활용</t>
+            <t>감시 도구라는 부정적 인식이 투자자의 도구라는 정체성으로 전환된다. 친구 공유는 자연스러운 바이럴 채널로 작동하며 브랜드 인지도 지표로 활용된다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="50" ht="130" customHeight="1">
+    <row r="50" ht="104" customHeight="1">
       <c r="A50" s="32" t="inlineStr">
         <is>
           <t>G-3</t>
@@ -3978,7 +4986,7 @@
       </c>
       <c r="B50" s="33" t="inlineStr">
         <is>
-          <t>G. 행동 전환·정체성 형성</t>
+          <t>G. 행동 전환·정체성</t>
         </is>
       </c>
       <c r="C50" s="34" t="inlineStr">
@@ -3988,7 +4996,7 @@
       </c>
       <c r="D50" s="35" t="inlineStr">
         <is>
-          <t>저축/투자 직후 즉시 총 자산 변화 피드백 + 그래프 실시간 반영</t>
+          <t>저축·투자 직후 즉각적인 자산 변화 시각화</t>
         </is>
       </c>
       <c r="E50" s="36" t="inlineStr">
@@ -4008,7 +5016,27 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>저축 또는 투자 직후, 즉시 "네 총 자산이 방금 OO원이 됐어!"라는 피드백을 준다. 작은 행동의 결과가 즉시 눈에 보여야 반복 동기가 생긴다.</t>
+            <t xml:space="preserve">자녀가 저축이나 투자를 실행한 직후 자산 변동이 즉시 시각화된다. "네 총 자산이 방금 124,300원에서 127,300원이 됐다"는 피드백과 함께 자산 그래프가 실시간으로 갱신된다. 매칭이 추가될 경우 "엄마가 3,000원 보태서 130,300원이 됐다"는 추가 표시가 노출된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 저축·투자 행동 직후 자산 변동 알림이 즉시 발송된다.
+2. 자산 그래프가 실시간 갱신된다.
+3. 매칭이 추가될 경우 추가 변동이 별도로 시각화된다.</t>
           </r>
         </is>
       </c>
@@ -4029,14 +5057,12 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>&gt; 작은 행동의 결과가 즉시 눈에 보여야 반복 동기가 생김
-- 저축 → 즉각 피드백 → 도파민 → 반복
-- 매칭이 붙으면 "엄마/아빠가 보태줬어!" 추가 → 감사함 + 책임감</t>
+            <t>작은 행동의 결과가 즉각 가시화되어 반복 동기가 강화된다. 행동과 결과의 시간 격차가 사라져 학습 효과가 극대화된다.</t>
           </r>
         </is>
       </c>
     </row>
-    <row r="51" ht="130" customHeight="1">
+    <row r="51" ht="104" customHeight="1">
       <c r="A51" s="32" t="inlineStr">
         <is>
           <t>G-4</t>
@@ -4044,7 +5070,7 @@
       </c>
       <c r="B51" s="33" t="inlineStr">
         <is>
-          <t>G. 행동 전환·정체성 형성</t>
+          <t>G. 행동 전환·정체성</t>
         </is>
       </c>
       <c r="C51" s="34" t="inlineStr">
@@ -4054,7 +5080,7 @@
       </c>
       <c r="D51" s="35" t="inlineStr">
         <is>
-          <t>총 자산 규모에 따라 앱 배경·아이콘·잠금화면 위젯이 자동 변화</t>
+          <t>총 자산 규모에 따라 앱 배경·아이콘·위젯이 자동 진화</t>
         </is>
       </c>
       <c r="E51" s="36" t="inlineStr">
@@ -4074,7 +5100,27 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>총 자산 규모에 따라 앱의 배경, 아이콘, 잠금화면 위젯이 자동으로 변화한다. 자산 감소 시 시각적으로도 축소된다.</t>
+            <t xml:space="preserve">총 자산 규모에 따라 앱의 배경, 아이콘, 잠금화면 위젯이 자동으로 변화한다. 10만원 미만은 새싹, 50만원은 나무, 100만원은 숲, 500만원은 도시, 1,000만원은 금융 제국 등 시각적 진화가 적용된다. 자산 감소 시에는 시각 요소도 함께 축소된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 총 자산 변동에 따라 앱 테마가 자동 적용된다.
+2. 잠금화면 위젯과 아이콘이 동시에 변화한다.
+3. 자산 감소 시 시각적 축소(나무가 줄어드는 효과 등)가 발생한다.</t>
           </r>
         </is>
       </c>
@@ -4095,7 +5141,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>&gt; 자산 누적이 시각적 정체성의 일부가 되면 이탈 비용이 높아짐</t>
+            <t>자산 누적이 자녀의 시각적 정체성으로 자리잡아 이탈 비용이 높아진다. 자산 변동이 외부에 가시화되어 자기 표현 욕구와 결합한다.</t>
           </r>
         </is>
       </c>

</xml_diff>

<commit_message>
vault backup: 2026-04-27 14:55:56
</commit_message>
<xml_diff>
--- a/content/Consulting/05_Tobe전략/아이디어풀/아이디어_상세설명_260427.xlsx
+++ b/content/Consulting/05_Tobe전략/아이디어풀/아이디어_상세설명_260427.xlsx
@@ -816,7 +816,7 @@
     <row r="3" ht="104" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>A-1-1</t>
+          <t>A-2</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -900,7 +900,7 @@
     <row r="4" ht="104" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>A-2</t>
+          <t>A-3</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -984,7 +984,7 @@
     <row r="5" ht="104" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>A-3</t>
+          <t>A-4</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1068,7 +1068,7 @@
     <row r="6" ht="104" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>A-4</t>
+          <t>A-5</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -2427,7 +2427,7 @@
     <row r="21" ht="104" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>B-7</t>
+          <t>B-6</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
@@ -2511,7 +2511,7 @@
     <row r="22" ht="104" customHeight="1">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>B-8</t>
+          <t>B-7</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
@@ -2595,7 +2595,7 @@
     <row r="23" ht="104" customHeight="1">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>C-2</t>
+          <t>C-1</t>
         </is>
       </c>
       <c r="B23" s="13" t="inlineStr">
@@ -2679,7 +2679,7 @@
     <row r="24" ht="104" customHeight="1">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>C-3</t>
+          <t>C-2</t>
         </is>
       </c>
       <c r="B24" s="13" t="inlineStr">
@@ -2763,7 +2763,7 @@
     <row r="25" ht="104" customHeight="1">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>C-4</t>
+          <t>C-3</t>
         </is>
       </c>
       <c r="B25" s="13" t="inlineStr">
@@ -2847,7 +2847,7 @@
     <row r="26" ht="104" customHeight="1">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>C-5</t>
+          <t>C-4</t>
         </is>
       </c>
       <c r="B26" s="13" t="inlineStr">
@@ -2950,7 +2950,7 @@
     <row r="27" ht="104" customHeight="1">
       <c r="A27" s="12" t="inlineStr">
         <is>
-          <t>C-6</t>
+          <t>C-5</t>
         </is>
       </c>
       <c r="B27" s="13" t="inlineStr">
@@ -3930,7 +3930,7 @@
     <row r="38" ht="104" customHeight="1">
       <c r="A38" s="22" t="inlineStr">
         <is>
-          <t>E-4</t>
+          <t>E-3</t>
         </is>
       </c>
       <c r="B38" s="23" t="inlineStr">
@@ -4014,7 +4014,7 @@
     <row r="39" ht="104" customHeight="1">
       <c r="A39" s="22" t="inlineStr">
         <is>
-          <t>E-5</t>
+          <t>E-4</t>
         </is>
       </c>
       <c r="B39" s="23" t="inlineStr">
@@ -4897,7 +4897,7 @@
     <row r="49" ht="104" customHeight="1">
       <c r="A49" s="32" t="inlineStr">
         <is>
-          <t>G-2</t>
+          <t>G-1</t>
         </is>
       </c>
       <c r="B49" s="33" t="inlineStr">
@@ -4981,7 +4981,7 @@
     <row r="50" ht="104" customHeight="1">
       <c r="A50" s="32" t="inlineStr">
         <is>
-          <t>G-3</t>
+          <t>G-2</t>
         </is>
       </c>
       <c r="B50" s="33" t="inlineStr">
@@ -5065,7 +5065,7 @@
     <row r="51" ht="104" customHeight="1">
       <c r="A51" s="32" t="inlineStr">
         <is>
-          <t>G-4</t>
+          <t>G-3</t>
         </is>
       </c>
       <c r="B51" s="33" t="inlineStr">

</xml_diff>

<commit_message>
vault backup: 2026-04-27 15:00:59
</commit_message>
<xml_diff>
--- a/content/Consulting/05_Tobe전략/아이디어풀/아이디어_상세설명_260427.xlsx
+++ b/content/Consulting/05_Tobe전략/아이디어풀/아이디어_상세설명_260427.xlsx
@@ -1607,7 +1607,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">한국 부자의 94%는 투자 수익을 재투자한다. 일반 대중(74%) 대비 격차가 분명한 이 행동 패턴이 부의 격차를 만드는 핵심 메커니즘이라는 분석에 기반한다. 자녀의 모든 인커밍(이자·배당·매칭금·세뱃돈·친척 송금)을 의사결정 단계 없이 기본값으로 재투자 슬롯에 배치한다.
+            <t xml:space="preserve">자녀 계좌에 들어오는 모든 수익(이자·배당·매칭금·세뱃돈·친척 송금)이 별도 의사결정 없이 기본값으로 재투자 슬롯에 배치된다. 작은 단위의 인커밍이 사라지지 않고 자산으로 누적되도록, 자산가 가정에서 보편적으로 나타나는 "수익 재투자" 행동을 자녀의 기본값으로 학습시키는 구조다.
 </t>
           </r>
           <r>
@@ -1710,7 +1710,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">K-EMILLI(50세 이하 자산 60억대 직장인 부자)의 해외주식 비중은 30%로 일반 부자(24%)의 1.25배다. 영리치 30대의 46%는 취업 이전에 주식을 시작했다. 자녀가 일찍부터 해외주식 진입로에 노출되는 것이 K-EMILLI 행동 패턴의 출발점이라는 가설에 기반한다.
+            <t xml:space="preserve">자녀가 알 만한 글로벌 브랜드(닌텐도·디즈니·애플·로블록스 등)를 중심으로 해외주식 1주 매수를 안내하는 모듈이다. 환율과 달러 배당 등 한국 주식과 다른 개념을 30~60초 미니퀘스트로 학습하면서 자연스럽게 해외주식 진입 경험이 누적된다.
 </t>
           </r>
           <r>
@@ -1776,7 +1776,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="182" customHeight="1">
+    <row r="14" ht="195" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>A-13</t>
@@ -1814,7 +1814,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">한국 부자가 자녀에게 이전하는 자산의 80%가 현금·예금이고 29%가 주식이며, 50대 이하 부자는 주식 비중이 더 높다. 세대 교체와 함께 주식 이전이 주류화되는 흐름에 대응해, 매도→입금→재매수의 3단계 마찰을 제거한 1-탭 증여 흐름을 제공한다.
+            <t xml:space="preserve">부모가 보유 중인 주식을 매도하지 않고 그대로 자녀 계좌로 이전하는 1-탭 증여 흐름이다. 매도→입금→재매수의 3단계 절차가 사라지고, 부모가 신뢰하는 종목이 그대로 자녀의 첫 종목이 된다. 증권사가 운영 중인 "증여 대체 출고" 절차와 비과세 한도 신고가 앱 내에서 자동화된다.
 </t>
           </r>
           <r>
@@ -1936,7 +1936,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">한국 부자가 꼽은 자산관리 1위 지혜는 "지속적인 금융지식 습득"(15.0%)이다. K-EMILLI의 47%는 "공부를 먼저 하고 투자한다"는 원칙을 따르며, 일반 부자(39%) 대비 1.2배 높다. 학습 → 투자의 시퀀스를 UX 차원에서 강제한다.
+            <t xml:space="preserve">신규 종목·ETF의 첫 매수 화면 진입 시 회사 정보와 핵심 지표를 30~60초 미니 학습으로 익히고 3문항 퀴즈를 통과해야 매수 버튼이 활성화되는 구조다. 매수 직전이 학습 동기가 가장 높은 시점이라는 점을 활용해 "공부 먼저, 투자 나중"의 시퀀스를 UX 차원에서 강제한다.
 </t>
           </r>
           <r>
@@ -2844,7 +2844,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="104" customHeight="1">
+    <row r="26" ht="130" customHeight="1">
       <c r="A26" s="12" t="inlineStr">
         <is>
           <t>C-4</t>
@@ -2882,7 +2882,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">최근 10년 내 부자 반열에 오른 K-EMILLI(평균 51세·자산 60억대 직장인)의 평균 포트폴리오 구성이 벤치마크로 제공된다. 자녀 포트폴리오와의 갭이 정량 비교되며, 미래 페르소나 모델링이 유도된다.
+            <t xml:space="preserve">자녀와 비슷한 출발점에서 부자 반열에 오른 K-EMILLI(평균 51세·자산 60억대 직장인 부자) 그룹의 평균 포트폴리오를 벤치마크로 보여주고, 자녀 포트폴리오와의 갭을 정량 비교 시각화한다. 막연한 "부자처럼"이 아니라 "나중에 닮을 모델 페르소나"와의 거리감을 자녀가 직관적으로 인식하도록 돕는다.
 </t>
           </r>
           <r>
@@ -2947,7 +2947,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="104" customHeight="1">
+    <row r="27" ht="117" customHeight="1">
       <c r="A27" s="12" t="inlineStr">
         <is>
           <t>C-5</t>
@@ -2985,7 +2985,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">한국 미성년자 주식 보유 규모는 약 7조원, 계좌 수는 5년간 7.7배 성장했다. 영리치의 5%는 미성년기에 주식을 시작했다. 또래의 실재가 데이터가 아닌 개별 스토리로 자녀에게 노출된다.
+            <t xml:space="preserve">익명화된 동년배 자녀의 자산 형성 사례를 카드 형태로 큐레이션하는 라이브러리다. 평균값 통계가 아닌 개별 스토리(예: "9살 김OO, ETF 첫 매수 후 3년 누적 +18%")로 또래의 실재가 드러나며, 자녀가 닮고 싶은 사례를 "내 모델"로 즐겨찾기할 수 있다.
 </t>
           </r>
           <r>
@@ -3638,7 +3638,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="156" customHeight="1">
+    <row r="35" ht="169" customHeight="1">
       <c r="A35" s="17" t="inlineStr">
         <is>
           <t>D-8</t>
@@ -3676,7 +3676,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">한국 부자의 19%는 자녀의 운용 자신감 부족을, 68%는 "많이 물려줄수록 성장 기회가 생긴다"는 인식을 동시에 가지고 있다. 두 우려를 동시에 해소하는 단계로 증여 전 시범 운용 기간이 도입된다.
+            <t xml:space="preserve">부모가 자산 일부를 "시범 운용 영역"으로 지정하면, 자녀가 매수·매도 의사결정을 제안하고 부모가 승인하는 구조다. 일정 기간(예: 6개월) 운용 결과가 기준에 부합하면 해당 자산이 정식 증여로 명의 이전되는, 증여 직전 단계의 트랙을 제공한다.
 </t>
           </r>
           <r>
@@ -4688,7 +4688,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="104" customHeight="1">
+    <row r="47" ht="117" customHeight="1">
       <c r="A47" s="27" t="inlineStr">
         <is>
           <t>F-8</t>
@@ -4726,7 +4726,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">한국 부자의 79%가 상속·증여 설계에서 가장 큰 우려로 꼽은 것은 상속세·증여세 부담이다. 비과세 한도를 끝까지 활용하지 않으면 사이클 단위로 한도가 소멸한다는 점에서, 한도 사용률이 부모 메인 화면에 상시 노출된다.
+            <t xml:space="preserve">10년 단위 비과세 증여 한도(미성년 2,000만원·성년 5,000만원)의 사용률과 만료까지의 시간이 부모 메인 화면 상단에 게이지 바로 상시 노출된다. 한도를 놓치면 사이클 단위로 소멸되는 절세 기회를 부모가 잊지 않도록, 시뮬레이터에 진입하지 않아도 즉시 인지할 수 있는 형태로 정보가 제공된다.
 </t>
           </r>
           <r>
@@ -4829,7 +4829,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">한국 부의 원천 중 상속·증여 비중이 2011년 13.7%에서 2023년 20.0%로 상승했다. 부자의 57%가 시점 분산 증여를 바람직하다고 답했다. 자산이전이 부모-자녀 1:1을 넘어 가문 단위 60년 곡선으로 재구성된다.
+            <t xml:space="preserve">조부모-부모-자녀 3대의 자산을 한 화면에 입력해 자산이전 시나리오를 비교 시뮬레이션한다. 전통 2단계(조부모→부모→자녀), 세대생략 증여(조부모→자녀 직접), 병행 시나리오의 3종을 60년 가문 자산 곡선으로 동시 비교하며, 비과세 한도와 세금이 자동 최적화된다.
 </t>
           </r>
           <r>

</xml_diff>

<commit_message>
vault backup: 2026-04-27 15:06:02
</commit_message>
<xml_diff>
--- a/content/Consulting/05_Tobe전략/아이디어풀/아이디어_상세설명_260427.xlsx
+++ b/content/Consulting/05_Tobe전략/아이디어풀/아이디어_상세설명_260427.xlsx
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1898,28 +1898,28 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="130" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>A-14</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>A. 투자·자산</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>매수 전 학습 게이트</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>신규 종목·ETF 첫 매수 전 미니 학습 통과 의무화</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
+    <row r="15" ht="104" customHeight="1">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>B-1</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>B. 소비·저축 행동</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>소비 예측 알림</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>현재 소비 패턴 기반 목표 달성 시뮬레이션 알림</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1936,7 +1936,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">신규 종목·ETF의 첫 매수 화면 진입 시 회사 정보와 핵심 지표를 30~60초 미니 학습으로 익히고 3문항 퀴즈를 통과해야 매수 버튼이 활성화되는 구조다. 매수 직전이 학습 동기가 가장 높은 시점이라는 점을 활용해 "공부 먼저, 투자 나중"의 시퀀스를 UX 차원에서 강제한다.
+            <t xml:space="preserve">현재의 소비 패턴을 기반으로 자녀가 목표한 물품의 도달 시점이 자동 계산되어 "이렇게 쓰면 에어팟까지 6개월" 형태로 안내된다.
 </t>
           </r>
           <r>
@@ -1954,15 +1954,13 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 신규 종목·ETF 매수 화면 진입 시 학습 게이트가 활성화된다.
-2. 회사 정보(제품·매출·CEO)를 30초 카드로 학습한다.
-3. PER·배당수익률·52주 변동폭 등 핵심 지표를 30초 카드로 학습한다.
-4. 3문항 미니 퀴즈 통과 시에만 매수 버튼이 활성화된다.
-5. 통과 후에는 동일 종목 3개월 패스가 적용되며, 학습 카드는 "투자 노트"에 누적된다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
+            <t>1. 자녀의 소비 패턴이 일별·주별로 분석된다.
+2. 현재 페이스 유지 시 목표 물품의 도달 시점이 자동 계산된다.
+3. 주요 분기점(목표 50%, 80% 등)에 알림이 발송된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -1979,25 +1977,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">K-EMILLI의 "先공부後투자" 행동 원칙이 자녀의 투자 의사결정 기본값으로 자리잡는다. 매수 직전이 학습 동기가 가장 높은 시점이라는 점에서 학습 효율이 극대화된다.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 차별 포인트
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>기존 첫 손실 가이드가 손실 발생 후 사후 교육이라면, 본 아이디어는 매수 전 사전 학습 게이팅으로 시점이 다르다. 두 기능이 결합되면 사전·사후 학습 사이클이 완성된다.</t>
+            <t>추상적 소비 결정이 구체적 시간 단위로 환산되어 자녀의 자기 조절 행동이 유도된다.</t>
           </r>
         </is>
       </c>
@@ -2005,7 +1985,7 @@
     <row r="16" ht="104" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>B-1</t>
+          <t>B-2</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
@@ -2015,12 +1995,12 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>소비 예측 알림</t>
+          <t>용돈 분배기</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>현재 소비 패턴 기반 목표 달성 시뮬레이션 알림</t>
+          <t>용돈 수령 직후 소비·저축·투자 비율 개인화 추천</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -2040,7 +2020,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">현재의 소비 패턴을 기반으로 자녀가 목표한 물품의 도달 시점이 자동 계산되어 "이렇게 쓰면 에어팟까지 6개월" 형태로 안내된다.
+            <t xml:space="preserve">용돈 수령 직후 자녀의 최근 소비 패턴이 분석되어 "이번 달은 저축 OO원, 투자 OO원, 소비 OO원이 적절하다"는 개인화 가이드가 제시된다.
 </t>
           </r>
           <r>
@@ -2058,9 +2038,9 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 자녀의 소비 패턴이 일별·주별로 분석된다.
-2. 현재 페이스 유지 시 목표 물품의 도달 시점이 자동 계산된다.
-3. 주요 분기점(목표 50%, 80% 등)에 알림이 발송된다.</t>
+            <t>1. 용돈 입금 즉시 분배 추천 화면이 노출된다.
+2. 최근 소비 패턴과 목표 진척도를 기반으로 비율이 자동 산출된다.
+3. 자녀가 수정 또는 수락하면 즉시 분배가 실행된다.</t>
           </r>
         </is>
       </c>
@@ -2081,7 +2061,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>추상적 소비 결정이 구체적 시간 단위로 환산되어 자녀의 자기 조절 행동이 유도된다.</t>
+            <t>수령 시점이 의사결정 동기가 가장 높은 순간이라는 점을 활용해 분배 행동이 자연스럽게 유도된다. 무계획 소비가 사전에 차단된다.</t>
           </r>
         </is>
       </c>
@@ -2089,7 +2069,7 @@
     <row r="17" ht="104" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>B-2</t>
+          <t>B-3</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
@@ -2099,12 +2079,12 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>용돈 분배기</t>
+          <t>위시리스트 → 매칭 목표 자동 제안</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>용돈 수령 직후 소비·저축·투자 비율 개인화 추천</t>
+          <t>자녀 위시리스트 등록 시 부모 매칭 저축 목표 자동 제안</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
@@ -2124,7 +2104,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">용돈 수령 직후 자녀의 최근 소비 패턴이 분석되어 "이번 달은 저축 OO원, 투자 OO원, 소비 OO원이 적절하다"는 개인화 가이드가 제시된다.
+            <t xml:space="preserve">자녀가 갖고 싶은 물건이나 투자 상품을 위시리스트에 등록하면 부모에게 "이 목표로 함께 저축해보시겠습니까"라는 매칭 저축 제안이 자동 발송된다.
 </t>
           </r>
           <r>
@@ -2142,9 +2122,9 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 용돈 입금 즉시 분배 추천 화면이 노출된다.
-2. 최근 소비 패턴과 목표 진척도를 기반으로 비율이 자동 산출된다.
-3. 자녀가 수정 또는 수락하면 즉시 분배가 실행된다.</t>
+            <t>1. 자녀가 위시리스트에 항목을 추가한다.
+2. 부모에게 매칭 저축 제안 알림이 전송된다.
+3. 부모가 수락하면 해당 목표 전용 저축 트랙이 활성화된다.</t>
           </r>
         </is>
       </c>
@@ -2165,7 +2145,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>수령 시점이 의사결정 동기가 가장 높은 순간이라는 점을 활용해 분배 행동이 자연스럽게 유도된다. 무계획 소비가 사전에 차단된다.</t>
+            <t>자녀의 욕구가 부모와의 협업 목표로 전환된다. 단순 구매 요청이 함께 모으는 활동으로 재구성된다.</t>
           </r>
         </is>
       </c>
@@ -2173,7 +2153,7 @@
     <row r="18" ht="104" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>B-3</t>
+          <t>B-4</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
@@ -2183,99 +2163,15 @@
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>위시리스트 → 매칭 목표 자동 제안</t>
+          <t>위시리스트 기반 저축 시뮬레이터</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>자녀 위시리스트 등록 시 부모 매칭 저축 목표 자동 제안</t>
+          <t>자동차 옵션 카탈로그 형태로 구성된 저축 플래너</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 개요
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">자녀가 갖고 싶은 물건이나 투자 상품을 위시리스트에 등록하면 부모에게 "이 목표로 함께 저축해보시겠습니까"라는 매칭 저축 제안이 자동 발송된다.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 동작 방식
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. 자녀가 위시리스트에 항목을 추가한다.
-2. 부모에게 매칭 저축 제안 알림이 전송된다.
-3. 부모가 수락하면 해당 목표 전용 저축 트랙이 활성화된다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F18" s="11" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 기대 효과
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>자녀의 욕구가 부모와의 협업 목표로 전환된다. 단순 구매 요청이 함께 모으는 활동으로 재구성된다.</t>
-          </r>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="104" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>B-4</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>B. 소비·저축 행동</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>위시리스트 기반 저축 시뮬레이터</t>
-        </is>
-      </c>
-      <c r="D19" s="10" t="inlineStr">
-        <is>
-          <t>자동차 옵션 카탈로그 형태로 구성된 저축 플래너</t>
-        </is>
-      </c>
-      <c r="E19" s="11" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2317,7 +2213,7 @@
           </r>
         </is>
       </c>
-      <c r="F19" s="11" t="inlineStr">
+      <c r="F18" s="11" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2339,28 +2235,28 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="104" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
+    <row r="19" ht="104" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>B-5</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>B. 소비·저축 행동</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C19" s="9" t="inlineStr">
         <is>
           <t>선수금 기반 저축 게임화</t>
         </is>
       </c>
-      <c r="D20" s="10" t="inlineStr">
+      <c r="D19" s="10" t="inlineStr">
         <is>
           <t>부모 선수금 + 자녀 분할 저축 + 실패 시 패널티 구조</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2402,6 +2298,90 @@
           </r>
         </is>
       </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>부모의 무조건적 지원이 아닌 함께 모으는 경험이 형성된다. 패널티 구조는 자녀의 책임감과 약속 이행 동기를 강화한다.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="104" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>B-6</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>B. 소비·저축 행동</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>세뱃돈·이벤트돈 → 투자 시드 전환</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>이벤트성 일시 수령 자금의 1-탭 투자 시드 전환</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 개요
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">세뱃돈, 조부모 송금 등 일시적으로 수령한 이벤트성 자금을 1-탭으로 투자 시드로 전환할 수 있다. "세뱃돈 절반을 투자하면 여름방학에 얼마가 될까" 형태의 시뮬레이션이 함께 제공된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 이벤트성 송금이 감지되면 시드 전환 추천 알림이 발송된다.
+2. 전환 비율(전액·절반·1/3 등)을 선택할 수 있다.
+3. 선택 즉시 투자 슬롯으로 이체되며, 미래 시뮬레이션이 함께 표시된다.</t>
+          </r>
+        </is>
+      </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
           <r>
@@ -2419,7 +2399,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>부모의 무조건적 지원이 아닌 함께 모으는 경험이 형성된다. 패널티 구조는 자녀의 책임감과 약속 이행 동기를 강화한다.</t>
+            <t>흔히 소비로 흘러가는 이벤트성 자금이 자산 형성으로 회수된다. 일시 수령액이 장기 자산으로 전환되는 경험이 누적된다.</t>
           </r>
         </is>
       </c>
@@ -2427,7 +2407,7 @@
     <row r="21" ht="104" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>B-6</t>
+          <t>B-7</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
@@ -2437,99 +2417,15 @@
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>세뱃돈·이벤트돈 → 투자 시드 전환</t>
+          <t>절약 감지 → 매칭 부스트</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>이벤트성 일시 수령 자금의 1-탭 투자 시드 전환</t>
+          <t>자녀 절약 행동 자동 감지 시 매칭 배율 동적 상향</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 개요
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">세뱃돈, 조부모 송금 등 일시적으로 수령한 이벤트성 자금을 1-탭으로 투자 시드로 전환할 수 있다. "세뱃돈 절반을 투자하면 여름방학에 얼마가 될까" 형태의 시뮬레이션이 함께 제공된다.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 동작 방식
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. 이벤트성 송금이 감지되면 시드 전환 추천 알림이 발송된다.
-2. 전환 비율(전액·절반·1/3 등)을 선택할 수 있다.
-3. 선택 즉시 투자 슬롯으로 이체되며, 미래 시뮬레이션이 함께 표시된다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F21" s="11" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 기대 효과
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>흔히 소비로 흘러가는 이벤트성 자금이 자산 형성으로 회수된다. 일시 수령액이 장기 자산으로 전환되는 경험이 누적된다.</t>
-          </r>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="104" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>B-7</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>B. 소비·저축 행동</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>절약 감지 → 매칭 부스트</t>
-        </is>
-      </c>
-      <c r="D22" s="10" t="inlineStr">
-        <is>
-          <t>자녀 절약 행동 자동 감지 시 매칭 배율 동적 상향</t>
-        </is>
-      </c>
-      <c r="E22" s="11" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2570,7 +2466,7 @@
           </r>
         </is>
       </c>
-      <c r="F22" s="11" t="inlineStr">
+      <c r="F21" s="11" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2588,6 +2484,90 @@
               <sz val="10"/>
             </rPr>
             <t>절약 행동이 즉각적 보상으로 연결된다. 자녀의 자기 조절 행동이 일회성이 아닌 반복 동기로 강화된다.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="104" customHeight="1">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>C-1</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>C. AI·개인화</t>
+        </is>
+      </c>
+      <c r="C22" s="14" t="inlineStr">
+        <is>
+          <t>부모 AI 어시스턴트</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>또래 평균 대비 자녀의 금융 행동 비교 시각화</t>
+        </is>
+      </c>
+      <c r="E22" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 개요
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">동년배 평균 저축률 등이 자녀의 데이터와 비교되어 시각화된다. 절대 금액이 아닌 용돈 대비 저축률 또는 소비 대비 저축률 등 상대 지표로 표시된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 자녀의 저축·소비·투자 데이터가 일별 집계된다.
+2. 동년배 평균과 비교한 리포트가 부모 화면에 제공된다.
+3. 특이 패턴 감지 시 부모에게 인사이트가 제안된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F22" s="16" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>절대 금액이 아닌 상대 지표가 사용되어 자산 격차에 의한 위화감이 제거된다. 부모의 비교 본능이 자녀의 행동 개선으로 전환된다.</t>
           </r>
         </is>
       </c>
@@ -2595,7 +2575,7 @@
     <row r="23" ht="104" customHeight="1">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>C-1</t>
+          <t>C-2</t>
         </is>
       </c>
       <c r="B23" s="13" t="inlineStr">
@@ -2605,12 +2585,12 @@
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>부모 AI 어시스턴트</t>
+          <t>AI 대화형 설정 UI</t>
         </is>
       </c>
       <c r="D23" s="15" t="inlineStr">
         <is>
-          <t>또래 평균 대비 자녀의 금융 행동 비교 시각화</t>
+          <t>단계별 페이지가 아닌 AI 대화 형태의 자연스러운 설정 흐름</t>
         </is>
       </c>
       <c r="E23" s="16" t="inlineStr">
@@ -2630,7 +2610,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">동년배 평균 저축률 등이 자녀의 데이터와 비교되어 시각화된다. 절대 금액이 아닌 용돈 대비 저축률 또는 소비 대비 저축률 등 상대 지표로 표시된다.
+            <t xml:space="preserve">기능 설정이 페이지 단위 프로세스가 아닌 AI 대화 형태로 구성된다. "뭐 사고 싶은데 어떻게 해야 되지" 같은 자연어 입력에 대해 계획이 자동 생성되며, 한 화면에서 기본값을 먼저 제시하고 수정만 팝업으로 처리된다.
 </t>
           </r>
           <r>
@@ -2648,9 +2628,9 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 자녀의 저축·소비·투자 데이터가 일별 집계된다.
-2. 동년배 평균과 비교한 리포트가 부모 화면에 제공된다.
-3. 특이 패턴 감지 시 부모에게 인사이트가 제안된다.</t>
+            <t>1. 자녀의 자연어 입력에 대해 AI가 기본 계획을 생성한다.
+2. 한 화면에 추천값이 먼저 표시된다.
+3. 수정이 필요한 항목만 탭하면 팝업으로 변경된다.</t>
           </r>
         </is>
       </c>
@@ -2671,7 +2651,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>절대 금액이 아닌 상대 지표가 사용되어 자산 격차에 의한 위화감이 제거된다. 부모의 비교 본능이 자녀의 행동 개선으로 전환된다.</t>
+            <t>단계별 페이지의 답답함이 제거되고, 기능이 도구처럼 노출되지 않는다. 사용 마찰이 낮아져 진입 장벽이 줄어든다.</t>
           </r>
         </is>
       </c>
@@ -2679,7 +2659,7 @@
     <row r="24" ht="104" customHeight="1">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>C-2</t>
+          <t>C-3</t>
         </is>
       </c>
       <c r="B24" s="13" t="inlineStr">
@@ -2689,99 +2669,15 @@
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>AI 대화형 설정 UI</t>
+          <t>데이터 기반 용돈 제안</t>
         </is>
       </c>
       <c r="D24" s="15" t="inlineStr">
         <is>
-          <t>단계별 페이지가 아닌 AI 대화 형태의 자연스러운 설정 흐름</t>
+          <t>지역·연령 데이터 기반 용돈 기본 세팅 자동 제안</t>
         </is>
       </c>
       <c r="E24" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 개요
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">기능 설정이 페이지 단위 프로세스가 아닌 AI 대화 형태로 구성된다. "뭐 사고 싶은데 어떻게 해야 되지" 같은 자연어 입력에 대해 계획이 자동 생성되며, 한 화면에서 기본값을 먼저 제시하고 수정만 팝업으로 처리된다.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 동작 방식
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. 자녀의 자연어 입력에 대해 AI가 기본 계획을 생성한다.
-2. 한 화면에 추천값이 먼저 표시된다.
-3. 수정이 필요한 항목만 탭하면 팝업으로 변경된다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F24" s="16" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 기대 효과
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>단계별 페이지의 답답함이 제거되고, 기능이 도구처럼 노출되지 않는다. 사용 마찰이 낮아져 진입 장벽이 줄어든다.</t>
-          </r>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="104" customHeight="1">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>C-3</t>
-        </is>
-      </c>
-      <c r="B25" s="13" t="inlineStr">
-        <is>
-          <t>C. AI·개인화</t>
-        </is>
-      </c>
-      <c r="C25" s="14" t="inlineStr">
-        <is>
-          <t>데이터 기반 용돈 제안</t>
-        </is>
-      </c>
-      <c r="D25" s="15" t="inlineStr">
-        <is>
-          <t>지역·연령 데이터 기반 용돈 기본 세팅 자동 제안</t>
-        </is>
-      </c>
-      <c r="E25" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2822,7 +2718,7 @@
           </r>
         </is>
       </c>
-      <c r="F25" s="16" t="inlineStr">
+      <c r="F24" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2844,28 +2740,28 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="130" customHeight="1">
-      <c r="A26" s="12" t="inlineStr">
+    <row r="25" ht="130" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>C-4</t>
         </is>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B25" s="13" t="inlineStr">
         <is>
           <t>C. AI·개인화</t>
         </is>
       </c>
-      <c r="C26" s="14" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr">
         <is>
           <t>K-EMILLI 미러 포트폴리오</t>
         </is>
       </c>
-      <c r="D26" s="15" t="inlineStr">
+      <c r="D25" s="15" t="inlineStr">
         <is>
           <t>K-EMILLI 평균 포트폴리오를 벤치마크로 자녀 자산 갭 시각화</t>
         </is>
       </c>
-      <c r="E26" s="16" t="inlineStr">
+      <c r="E25" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2907,7 +2803,7 @@
           </r>
         </is>
       </c>
-      <c r="F26" s="16" t="inlineStr">
+      <c r="F25" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -2947,28 +2843,28 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="117" customHeight="1">
-      <c r="A27" s="12" t="inlineStr">
+    <row r="26" ht="117" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>C-5</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B26" s="13" t="inlineStr">
         <is>
           <t>C. AI·개인화</t>
         </is>
       </c>
-      <c r="C27" s="14" t="inlineStr">
+      <c r="C26" s="14" t="inlineStr">
         <is>
           <t>또래 부자 가정 자녀 케이스북</t>
         </is>
       </c>
-      <c r="D27" s="15" t="inlineStr">
+      <c r="D26" s="15" t="inlineStr">
         <is>
           <t>익명화된 동년배 자산 형성 사례를 카드 형태로 큐레이션</t>
         </is>
       </c>
-      <c r="E27" s="16" t="inlineStr">
+      <c r="E26" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3010,7 +2906,7 @@
           </r>
         </is>
       </c>
-      <c r="F27" s="16" t="inlineStr">
+      <c r="F26" s="16" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3046,6 +2942,90 @@
               <sz val="10"/>
             </rPr>
             <t>기존 부모 AI 어시스턴트의 또래 비교가 평균값 통계라면, 본 아이디어는 개별 사례 스토리 큐레이션이라는 점에서 결이 다르다.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="104" customHeight="1">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>D-1</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>D. 권한 이양·성장</t>
+        </is>
+      </c>
+      <c r="C27" s="19" t="inlineStr">
+        <is>
+          <t>자녀 금융 신용 점수</t>
+        </is>
+      </c>
+      <c r="D27" s="20" t="inlineStr">
+        <is>
+          <t>저축률·목표 달성률·약속 이행률 기반 신용 점수와 자율 한도 자동 확대</t>
+        </is>
+      </c>
+      <c r="E27" s="21" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 개요
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">자녀의 저축률·목표 달성률·부모 약속 이행률 등을 종합한 금융 신용 점수가 산출된다. 점수 상승 시 자율 소비·투자 한도가 자동으로 확대된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 자녀의 저축·소비·약속 이행 데이터가 점수에 누적 반영된다.
+2. 점수가 임계치를 넘으면 자율 한도가 자동 확대된다.
+3. 성년 도달 시 누적 점수가 하나은행 금리 우대 등 실제 혜택과 연계된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F27" s="21" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>권한 확대가 부모의 자의적 판단이 아닌 데이터 기반으로 이루어진다. 자녀의 행동이 정량 평가되어 권한과 책임의 비례 관계가 명확해진다.</t>
           </r>
         </is>
       </c>
@@ -3053,7 +3033,7 @@
     <row r="28" ht="104" customHeight="1">
       <c r="A28" s="17" t="inlineStr">
         <is>
-          <t>D-1</t>
+          <t>D-2</t>
         </is>
       </c>
       <c r="B28" s="18" t="inlineStr">
@@ -3063,12 +3043,12 @@
       </c>
       <c r="C28" s="19" t="inlineStr">
         <is>
-          <t>자녀 금융 신용 점수</t>
+          <t>부모-자녀 금융 계약서</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
         <is>
-          <t>저축률·목표 달성률·약속 이행률 기반 신용 점수와 자율 한도 자동 확대</t>
+          <t>부모와 자녀 간의 금융 약속을 공식 문서로 기록</t>
         </is>
       </c>
       <c r="E28" s="21" t="inlineStr">
@@ -3088,7 +3068,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">자녀의 저축률·목표 달성률·부모 약속 이행률 등을 종합한 금융 신용 점수가 산출된다. 점수 상승 시 자율 소비·투자 한도가 자동으로 확대된다.
+            <t xml:space="preserve">"네가 OO세까지 OO원을 모으면 다음부터 용돈을 6개월에 한 번 목돈으로 지급한다" 형태의 부모-자녀 약속이 공식 계약서로 기록된다.
 </t>
           </r>
           <r>
@@ -3106,9 +3086,9 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 자녀의 저축·소비·약속 이행 데이터가 점수에 누적 반영된다.
-2. 점수가 임계치를 넘으면 자율 한도가 자동 확대된다.
-3. 성년 도달 시 누적 점수가 하나은행 금리 우대 등 실제 혜택과 연계된다.</t>
+            <t>1. 부모와 자녀가 함께 약속 조건을 입력한다.
+2. 양측이 디지털 서명하면 계약서가 발효된다.
+3. 조건 충족 시점에 자동으로 약속 이행 절차가 실행된다.</t>
           </r>
         </is>
       </c>
@@ -3129,7 +3109,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>권한 확대가 부모의 자의적 판단이 아닌 데이터 기반으로 이루어진다. 자녀의 행동이 정량 평가되어 권한과 책임의 비례 관계가 명확해진다.</t>
+            <t>암묵적 약속이 명시적 문서로 전환되어 양측의 신뢰와 책임이 강화된다. 자녀에게는 첫 계약 경험으로 작용한다.</t>
           </r>
         </is>
       </c>
@@ -3137,7 +3117,7 @@
     <row r="29" ht="104" customHeight="1">
       <c r="A29" s="17" t="inlineStr">
         <is>
-          <t>D-2</t>
+          <t>D-3</t>
         </is>
       </c>
       <c r="B29" s="18" t="inlineStr">
@@ -3147,12 +3127,12 @@
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>부모-자녀 금융 계약서</t>
+          <t>연간 용돈 일괄 지급 자격</t>
         </is>
       </c>
       <c r="D29" s="20" t="inlineStr">
         <is>
-          <t>부모와 자녀 간의 금융 약속을 공식 문서로 기록</t>
+          <t>금융 퀴즈·신용 점수·계약 이행 기반 자격 심사</t>
         </is>
       </c>
       <c r="E29" s="21" t="inlineStr">
@@ -3172,7 +3152,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">"네가 OO세까지 OO원을 모으면 다음부터 용돈을 6개월에 한 번 목돈으로 지급한다" 형태의 부모-자녀 약속이 공식 계약서로 기록된다.
+            <t xml:space="preserve">금융 퀴즈, 신용 점수, 계약 이행 이력을 종합한 자격 심사를 통과한 자녀에게 용돈이 연 단위 목돈으로 일괄 지급된다.
 </t>
           </r>
           <r>
@@ -3190,9 +3170,9 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 부모와 자녀가 함께 약속 조건을 입력한다.
-2. 양측이 디지털 서명하면 계약서가 발효된다.
-3. 조건 충족 시점에 자동으로 약속 이행 절차가 실행된다.</t>
+            <t>1. 자녀가 금융 퀴즈에 응시한다.
+2. 신용 점수와 계약 이행 이력이 자동 집계된다.
+3. 자격 통과 시 부모는 연 단위 일괄 지급 옵션을 활성화할 수 있다.</t>
           </r>
         </is>
       </c>
@@ -3213,7 +3193,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>암묵적 약속이 명시적 문서로 전환되어 양측의 신뢰와 책임이 강화된다. 자녀에게는 첫 계약 경험으로 작용한다.</t>
+            <t>단순 용돈 수령에서 자기 자금 관리로 권한이 이양된다. 일괄 지급된 자금을 12개월 동안 분배·운용하는 경험이 자산 관리 역량으로 누적된다.</t>
           </r>
         </is>
       </c>
@@ -3221,7 +3201,7 @@
     <row r="30" ht="104" customHeight="1">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>D-3</t>
+          <t>D-4</t>
         </is>
       </c>
       <c r="B30" s="18" t="inlineStr">
@@ -3231,12 +3211,12 @@
       </c>
       <c r="C30" s="19" t="inlineStr">
         <is>
-          <t>연간 용돈 일괄 지급 자격</t>
+          <t>연령별 메인 화면 변화 (Complexity Growth)</t>
         </is>
       </c>
       <c r="D30" s="20" t="inlineStr">
         <is>
-          <t>금융 퀴즈·신용 점수·계약 이행 기반 자격 심사</t>
+          <t>연령에 따른 메인 화면 정보 복잡도 단계적 확장</t>
         </is>
       </c>
       <c r="E30" s="21" t="inlineStr">
@@ -3256,7 +3236,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">금융 퀴즈, 신용 점수, 계약 이행 이력을 종합한 자격 심사를 통과한 자녀에게 용돈이 연 단위 목돈으로 일괄 지급된다.
+            <t xml:space="preserve">어린 시절에는 저금통과 용돈 요청 중심의 단순한 화면이, 성장과 함께 자산·주식·투자 방법 등 복잡한 정보가 점진적으로 노출된다. 19세에는 완전한 자산 관리 화면으로 전환된다.
 </t>
           </r>
           <r>
@@ -3274,9 +3254,9 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 자녀가 금융 퀴즈에 응시한다.
-2. 신용 점수와 계약 이행 이력이 자동 집계된다.
-3. 자격 통과 시 부모는 연 단위 일괄 지급 옵션을 활성화할 수 있다.</t>
+            <t>1. 연령·학제·신용 점수에 따라 화면 구성 단계가 자동 전환된다.
+2. 각 단계에서 새 기능이 단계적으로 노출된다.
+3. 전환 시 레벨업 애니메이션과 안내 카드가 제공된다.</t>
           </r>
         </is>
       </c>
@@ -3297,7 +3277,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>단순 용돈 수령에서 자기 자금 관리로 권한이 이양된다. 일괄 지급된 자금을 12개월 동안 분배·운용하는 경험이 자산 관리 역량으로 누적된다.</t>
+            <t>복잡도 증가가 자녀의 인지 발달과 보조를 맞춘다. 동일한 앱 안에서 18년의 성장 경험이 시각적으로 형성된다.</t>
           </r>
         </is>
       </c>
@@ -3305,7 +3285,7 @@
     <row r="31" ht="104" customHeight="1">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>D-4</t>
+          <t>D-5</t>
         </is>
       </c>
       <c r="B31" s="18" t="inlineStr">
@@ -3315,12 +3295,12 @@
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>연령별 메인 화면 변화 (Complexity Growth)</t>
+          <t>제안 투표 (매칭금 배분 자녀 참여)</t>
         </is>
       </c>
       <c r="D31" s="20" t="inlineStr">
         <is>
-          <t>연령에 따른 메인 화면 정보 복잡도 단계적 확장</t>
+          <t>매칭금 일부 배분에 대한 자녀 직접 제안·투표</t>
         </is>
       </c>
       <c r="E31" s="21" t="inlineStr">
@@ -3340,7 +3320,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">어린 시절에는 저금통과 용돈 요청 중심의 단순한 화면이, 성장과 함께 자산·주식·투자 방법 등 복잡한 정보가 점진적으로 노출된다. 19세에는 완전한 자산 관리 화면으로 전환된다.
+            <t xml:space="preserve">부모의 매칭금 일부를 자녀가 어떻게 배분할지 제안하고 투표한다. "네 한 표가 이번 달 매칭금의 30%를 움직인다"는 메시지로 참여 동기가 강화된다.
 </t>
           </r>
           <r>
@@ -3358,9 +3338,9 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 연령·학제·신용 점수에 따라 화면 구성 단계가 자동 전환된다.
-2. 각 단계에서 새 기능이 단계적으로 노출된다.
-3. 전환 시 레벨업 애니메이션과 안내 카드가 제공된다.</t>
+            <t>1. 이번 달 매칭금 중 자녀 결정권 비율이 사전 합의된다.
+2. 자녀가 배분 방식을 제안하고 가족 투표가 이루어진다.
+3. 투표 결과에 따라 매칭금이 자동 배분된다.</t>
           </r>
         </is>
       </c>
@@ -3381,7 +3361,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>복잡도 증가가 자녀의 인지 발달과 보조를 맞춘다. 동일한 앱 안에서 18년의 성장 경험이 시각적으로 형성된다.</t>
+            <t>수동적 수령자가 아닌 능동적 의사결정자로 자녀의 역할이 전환된다. 자금에 대한 주인 의식이 형성된다.</t>
           </r>
         </is>
       </c>
@@ -3389,7 +3369,7 @@
     <row r="32" ht="104" customHeight="1">
       <c r="A32" s="17" t="inlineStr">
         <is>
-          <t>D-5</t>
+          <t>D-6</t>
         </is>
       </c>
       <c r="B32" s="18" t="inlineStr">
@@ -3399,12 +3379,12 @@
       </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
-          <t>제안 투표 (매칭금 배분 자녀 참여)</t>
+          <t>5단계 권한 이양 프레임</t>
         </is>
       </c>
       <c r="D32" s="20" t="inlineStr">
         <is>
-          <t>매칭금 일부 배분에 대한 자녀 직접 제안·투표</t>
+          <t>관찰자→선택자→제안자→운용자→독립견습 5단계 자율성 이양</t>
         </is>
       </c>
       <c r="E32" s="21" t="inlineStr">
@@ -3424,7 +3404,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">부모의 매칭금 일부를 자녀가 어떻게 배분할지 제안하고 투표한다. "네 한 표가 이번 달 매칭금의 30%를 움직인다"는 메시지로 참여 동기가 강화된다.
+            <t xml:space="preserve">관찰자, 선택자, 제안자, 운용자, 독립견습의 5단계로 자녀의 자율성이 이양된다. 연령·학제·부모 판단의 3축으로 단계 전환이 결정되며, 각 단계에서 권한 범위가 자동 확대된다.
 </t>
           </r>
           <r>
@@ -3442,9 +3422,9 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 이번 달 매칭금 중 자녀 결정권 비율이 사전 합의된다.
-2. 자녀가 배분 방식을 제안하고 가족 투표가 이루어진다.
-3. 투표 결과에 따라 매칭금이 자동 배분된다.</t>
+            <t>1. 현재 단계에 따라 자녀의 권한 범위와 기본값이 다르게 적용된다.
+2. 전환 조건(연령·학제·부모 판단) 충족 시 다음 단계가 활성화된다.
+3. 단계 전환 시 새 권한과 책임이 안내된다.</t>
           </r>
         </is>
       </c>
@@ -3465,7 +3445,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>수동적 수령자가 아닌 능동적 의사결정자로 자녀의 역할이 전환된다. 자금에 대한 주인 의식이 형성된다.</t>
+            <t>권한 이양이 일회성 이벤트가 아닌 단계적 구조로 정착한다. 자녀의 성장 단계에 맞는 자율성이 보장된다.</t>
           </r>
         </is>
       </c>
@@ -3473,7 +3453,7 @@
     <row r="33" ht="104" customHeight="1">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>D-6</t>
+          <t>D-7</t>
         </is>
       </c>
       <c r="B33" s="18" t="inlineStr">
@@ -3483,99 +3463,15 @@
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>5단계 권한 이양 프레임</t>
+          <t>단계 전환 위저드 + 레벨업 페이지</t>
         </is>
       </c>
       <c r="D33" s="20" t="inlineStr">
         <is>
-          <t>관찰자→선택자→제안자→운용자→독립견습 5단계 자율성 이양</t>
+          <t>진학 등 전환 시점의 한도·주기 자동 재제안과 레벨업 연출</t>
         </is>
       </c>
       <c r="E33" s="21" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 개요
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">관찰자, 선택자, 제안자, 운용자, 독립견습의 5단계로 자녀의 자율성이 이양된다. 연령·학제·부모 판단의 3축으로 단계 전환이 결정되며, 각 단계에서 권한 범위가 자동 확대된다.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 동작 방식
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. 현재 단계에 따라 자녀의 권한 범위와 기본값이 다르게 적용된다.
-2. 전환 조건(연령·학제·부모 판단) 충족 시 다음 단계가 활성화된다.
-3. 단계 전환 시 새 권한과 책임이 안내된다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F33" s="21" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 기대 효과
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>권한 이양이 일회성 이벤트가 아닌 단계적 구조로 정착한다. 자녀의 성장 단계에 맞는 자율성이 보장된다.</t>
-          </r>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="104" customHeight="1">
-      <c r="A34" s="17" t="inlineStr">
-        <is>
-          <t>D-7</t>
-        </is>
-      </c>
-      <c r="B34" s="18" t="inlineStr">
-        <is>
-          <t>D. 권한 이양·성장</t>
-        </is>
-      </c>
-      <c r="C34" s="19" t="inlineStr">
-        <is>
-          <t>단계 전환 위저드 + 레벨업 페이지</t>
-        </is>
-      </c>
-      <c r="D34" s="20" t="inlineStr">
-        <is>
-          <t>진학 등 전환 시점의 한도·주기 자동 재제안과 레벨업 연출</t>
-        </is>
-      </c>
-      <c r="E34" s="21" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3616,7 +3512,7 @@
           </r>
         </is>
       </c>
-      <c r="F34" s="21" t="inlineStr">
+      <c r="F33" s="21" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3638,28 +3534,28 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="169" customHeight="1">
-      <c r="A35" s="17" t="inlineStr">
+    <row r="34" ht="169" customHeight="1">
+      <c r="A34" s="17" t="inlineStr">
         <is>
           <t>D-8</t>
         </is>
       </c>
-      <c r="B35" s="18" t="inlineStr">
+      <c r="B34" s="18" t="inlineStr">
         <is>
           <t>D. 권한 이양·성장</t>
         </is>
       </c>
-      <c r="C35" s="19" t="inlineStr">
+      <c r="C34" s="19" t="inlineStr">
         <is>
           <t>사전 운용권 분리 (증여 전 시범 운용)</t>
         </is>
       </c>
-      <c r="D35" s="20" t="inlineStr">
+      <c r="D34" s="20" t="inlineStr">
         <is>
           <t>부모 자산 일부에 자녀 의사결정권만 위임 → 결과 통과 시 명의 이전</t>
         </is>
       </c>
-      <c r="E35" s="21" t="inlineStr">
+      <c r="E34" s="21" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3719,7 +3615,7 @@
           </r>
         </is>
       </c>
-      <c r="F35" s="21" t="inlineStr">
+      <c r="F34" s="21" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3755,6 +3651,90 @@
               <sz val="10"/>
             </rPr>
             <t>기존 자녀 금융 신용 점수가 자녀 자체 자산의 권한 확대 구조라면, 본 아이디어는 증여 직전 단계에서 부모 자산의 운용 의사결정만 빌려주는 별도 트랙이다.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="104" customHeight="1">
+      <c r="A35" s="22" t="inlineStr">
+        <is>
+          <t>E-1</t>
+        </is>
+      </c>
+      <c r="B35" s="23" t="inlineStr">
+        <is>
+          <t>E. 게임화·보상</t>
+        </is>
+      </c>
+      <c r="C35" s="24" t="inlineStr">
+        <is>
+          <t>배지·칭호 시스템</t>
+        </is>
+      </c>
+      <c r="D35" s="25" t="inlineStr">
+        <is>
+          <t>달성 기반 배지 수집과 칭호 부여</t>
+        </is>
+      </c>
+      <c r="E35" s="26" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 개요
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">자산 형성과 행동 달성 단계에 따라 배지가 부여되고 칭호가 표시된다. "100만 장자", "16살 기준 일론 머스크보다 부자" 등 자녀의 흥미를 자극하는 칭호가 금융적 성장에 연동된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 달성 조건이 충족되면 배지가 자동 발급된다.
+2. 특정 배지 조합이나 임계치 달성 시 칭호가 부여된다.
+3. 획득한 배지·칭호는 프로필에 노출되고 친구에게 공유될 수 있다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F35" s="26" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>수집욕을 자극하는 마이크로 인터랙션이 행동 동기로 전환된다. 칭호는 자녀의 자산 성장 정체성을 강화한다.</t>
           </r>
         </is>
       </c>
@@ -3762,7 +3742,7 @@
     <row r="36" ht="104" customHeight="1">
       <c r="A36" s="22" t="inlineStr">
         <is>
-          <t>E-1</t>
+          <t>E-2</t>
         </is>
       </c>
       <c r="B36" s="23" t="inlineStr">
@@ -3772,12 +3752,12 @@
       </c>
       <c r="C36" s="24" t="inlineStr">
         <is>
-          <t>배지·칭호 시스템</t>
+          <t>프로필 커스터마이징</t>
         </is>
       </c>
       <c r="D36" s="25" t="inlineStr">
         <is>
-          <t>달성 기반 배지 수집과 칭호 부여</t>
+          <t>자산 규모에 따라 아이콘이 진화하는 프로필</t>
         </is>
       </c>
       <c r="E36" s="26" t="inlineStr">
@@ -3797,7 +3777,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">자산 형성과 행동 달성 단계에 따라 배지가 부여되고 칭호가 표시된다. "100만 장자", "16살 기준 일론 머스크보다 부자" 등 자녀의 흥미를 자극하는 칭호가 금융적 성장에 연동된다.
+            <t xml:space="preserve">카카오톡처럼 자기 프로필을 꾸밀 수 있다. 자산이 적을 때는 단순한 아이콘으로 시작해 자산 누적과 함께 점차 풍요로운 모습으로 진화한다.
 </t>
           </r>
           <r>
@@ -3815,9 +3795,9 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 달성 조건이 충족되면 배지가 자동 발급된다.
-2. 특정 배지 조합이나 임계치 달성 시 칭호가 부여된다.
-3. 획득한 배지·칭호는 프로필에 노출되고 친구에게 공유될 수 있다.</t>
+            <t>1. 자녀가 아바타와 배경을 선택해 프로필을 꾸민다.
+2. 총 자산 규모에 따라 아이콘이 자동으로 진화한다.
+3. 친구와 프로필을 공유하거나 비교할 수 있다.</t>
           </r>
         </is>
       </c>
@@ -3838,7 +3818,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>수집욕을 자극하는 마이크로 인터랙션이 행동 동기로 전환된다. 칭호는 자녀의 자산 성장 정체성을 강화한다.</t>
+            <t>자산 성장이 시각적 정체성의 일부가 되어 이탈 비용이 높아진다. 자기 표현 욕구가 자산 형성 동기와 결합한다.</t>
           </r>
         </is>
       </c>
@@ -3846,7 +3826,7 @@
     <row r="37" ht="104" customHeight="1">
       <c r="A37" s="22" t="inlineStr">
         <is>
-          <t>E-2</t>
+          <t>E-3</t>
         </is>
       </c>
       <c r="B37" s="23" t="inlineStr">
@@ -3856,12 +3836,12 @@
       </c>
       <c r="C37" s="24" t="inlineStr">
         <is>
-          <t>프로필 커스터마이징</t>
+          <t>금융 히스토리 카드 수집</t>
         </is>
       </c>
       <c r="D37" s="25" t="inlineStr">
         <is>
-          <t>자산 규모에 따라 아이콘이 진화하는 프로필</t>
+          <t>자산 성장 마일스톤을 카드 형태로 수집</t>
         </is>
       </c>
       <c r="E37" s="26" t="inlineStr">
@@ -3881,7 +3861,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">카카오톡처럼 자기 프로필을 꾸밀 수 있다. 자산이 적을 때는 단순한 아이콘으로 시작해 자산 누적과 함께 점차 풍요로운 모습으로 진화한다.
+            <t xml:space="preserve">"첫 주식 수익", "100만 원 돌파" 등 자산 성장의 주요 마일스톤이 카드 형태로 발급되어 수집된다. 카카오톡 선물하기 이력처럼 시각적 컬렉션으로 누적된다.
 </t>
           </r>
           <r>
@@ -3899,9 +3879,9 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 자녀가 아바타와 배경을 선택해 프로필을 꾸민다.
-2. 총 자산 규모에 따라 아이콘이 자동으로 진화한다.
-3. 친구와 프로필을 공유하거나 비교할 수 있다.</t>
+            <t>1. 마일스톤 달성 시 카드가 자동 발급된다.
+2. 수집된 카드는 갤러리에 누적 보관된다.
+3. 특정 카드 조합 달성 시 추가 보상이 지급된다.</t>
           </r>
         </is>
       </c>
@@ -3922,7 +3902,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>자산 성장이 시각적 정체성의 일부가 되어 이탈 비용이 높아진다. 자기 표현 욕구가 자산 형성 동기와 결합한다.</t>
+            <t>자산 성장의 무형 성과가 시각적 자산으로 전환된다. 수집욕이 장기 사용 동기로 작용한다.</t>
           </r>
         </is>
       </c>
@@ -3930,7 +3910,7 @@
     <row r="38" ht="104" customHeight="1">
       <c r="A38" s="22" t="inlineStr">
         <is>
-          <t>E-3</t>
+          <t>E-4</t>
         </is>
       </c>
       <c r="B38" s="23" t="inlineStr">
@@ -3940,99 +3920,15 @@
       </c>
       <c r="C38" s="24" t="inlineStr">
         <is>
-          <t>금융 히스토리 카드 수집</t>
+          <t>연속 달성 보상</t>
         </is>
       </c>
       <c r="D38" s="25" t="inlineStr">
         <is>
-          <t>자산 성장 마일스톤을 카드 형태로 수집</t>
+          <t>연속 저축·미션 달성 시 보상 적립</t>
         </is>
       </c>
       <c r="E38" s="26" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 개요
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">"첫 주식 수익", "100만 원 돌파" 등 자산 성장의 주요 마일스톤이 카드 형태로 발급되어 수집된다. 카카오톡 선물하기 이력처럼 시각적 컬렉션으로 누적된다.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 동작 방식
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. 마일스톤 달성 시 카드가 자동 발급된다.
-2. 수집된 카드는 갤러리에 누적 보관된다.
-3. 특정 카드 조합 달성 시 추가 보상이 지급된다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F38" s="26" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 기대 효과
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>자산 성장의 무형 성과가 시각적 자산으로 전환된다. 수집욕이 장기 사용 동기로 작용한다.</t>
-          </r>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="104" customHeight="1">
-      <c r="A39" s="22" t="inlineStr">
-        <is>
-          <t>E-4</t>
-        </is>
-      </c>
-      <c r="B39" s="23" t="inlineStr">
-        <is>
-          <t>E. 게임화·보상</t>
-        </is>
-      </c>
-      <c r="C39" s="24" t="inlineStr">
-        <is>
-          <t>연속 달성 보상</t>
-        </is>
-      </c>
-      <c r="D39" s="25" t="inlineStr">
-        <is>
-          <t>연속 저축·미션 달성 시 보상 적립</t>
-        </is>
-      </c>
-      <c r="E39" s="26" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4073,7 +3969,7 @@
           </r>
         </is>
       </c>
-      <c r="F39" s="26" t="inlineStr">
+      <c r="F38" s="26" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4095,28 +3991,28 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="104" customHeight="1">
-      <c r="A40" s="27" t="inlineStr">
+    <row r="39" ht="104" customHeight="1">
+      <c r="A39" s="27" t="inlineStr">
         <is>
           <t>F-1</t>
         </is>
       </c>
-      <c r="B40" s="28" t="inlineStr">
+      <c r="B39" s="28" t="inlineStr">
         <is>
           <t>F. 진입·리텐션</t>
         </is>
       </c>
-      <c r="C40" s="29" t="inlineStr">
+      <c r="C39" s="29" t="inlineStr">
         <is>
           <t>부모 반복 트리거 5종</t>
         </is>
       </c>
-      <c r="D40" s="30" t="inlineStr">
+      <c r="D39" s="30" t="inlineStr">
         <is>
           <t>자녀 인사이트·자산 통합·성장 리포트·세무 도구·성과 알림</t>
         </is>
       </c>
-      <c r="E40" s="31" t="inlineStr">
+      <c r="E39" s="31" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4159,6 +4055,90 @@
           </r>
         </is>
       </c>
+      <c r="F39" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>부모의 반복 진입 동기가 다층화된다. 한 가지 트리거가 약해도 다른 트리거로 보완되어 장기 리텐션이 안정화된다.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="104" customHeight="1">
+      <c r="A40" s="27" t="inlineStr">
+        <is>
+          <t>F-2</t>
+        </is>
+      </c>
+      <c r="B40" s="28" t="inlineStr">
+        <is>
+          <t>F. 진입·리텐션</t>
+        </is>
+      </c>
+      <c r="C40" s="29" t="inlineStr">
+        <is>
+          <t>조건·이벤트 트리거 7종</t>
+        </is>
+      </c>
+      <c r="D40" s="30" t="inlineStr">
+        <is>
+          <t>외부 이벤트와 연동된 진입 트리거 7개</t>
+        </is>
+      </c>
+      <c r="E40" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 개요
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">사용자의 외부 이벤트와 연동된 7가지 진입 트리거가 운영된다. 세뱃돈 시즌, 월말·연말, 절약 감지, 배당·이자 발생, 학제 전환, 경제 뉴스, 조부모·친척 송금 시점이 포함된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 각 이벤트 발생 시점이 시스템에 자동 감지된다.
+2. 이벤트 맥락에 맞는 추천 알림이 발송된다.
+3. 알림 클릭 시 이벤트에 최적화된 액션 화면으로 이동한다.</t>
+          </r>
+        </is>
+      </c>
       <c r="F40" s="31" t="inlineStr">
         <is>
           <r>
@@ -4176,7 +4156,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>부모의 반복 진입 동기가 다층화된다. 한 가지 트리거가 약해도 다른 트리거로 보완되어 장기 리텐션이 안정화된다.</t>
+            <t>사용자의 일상 흐름과 동기화된 진입 동기가 형성된다. 외부 이벤트가 곧 앱 사용의 트리거가 된다.</t>
           </r>
         </is>
       </c>
@@ -4184,7 +4164,7 @@
     <row r="41" ht="104" customHeight="1">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>F-2</t>
+          <t>F-3</t>
         </is>
       </c>
       <c r="B41" s="28" t="inlineStr">
@@ -4194,99 +4174,15 @@
       </c>
       <c r="C41" s="29" t="inlineStr">
         <is>
-          <t>조건·이벤트 트리거 7종</t>
+          <t>중학교 이탈 방어 5종</t>
         </is>
       </c>
       <c r="D41" s="30" t="inlineStr">
         <is>
-          <t>외부 이벤트와 연동된 진입 트리거 7개</t>
+          <t>감시감 제거·비교 전환·기여감·현실 효용·소셜 방어 UX</t>
         </is>
       </c>
       <c r="E41" s="31" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 개요
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">사용자의 외부 이벤트와 연동된 7가지 진입 트리거가 운영된다. 세뱃돈 시즌, 월말·연말, 절약 감지, 배당·이자 발생, 학제 전환, 경제 뉴스, 조부모·친척 송금 시점이 포함된다.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 동작 방식
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. 각 이벤트 발생 시점이 시스템에 자동 감지된다.
-2. 이벤트 맥락에 맞는 추천 알림이 발송된다.
-3. 알림 클릭 시 이벤트에 최적화된 액션 화면으로 이동한다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F41" s="31" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 기대 효과
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>사용자의 일상 흐름과 동기화된 진입 동기가 형성된다. 외부 이벤트가 곧 앱 사용의 트리거가 된다.</t>
-          </r>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="104" customHeight="1">
-      <c r="A42" s="27" t="inlineStr">
-        <is>
-          <t>F-3</t>
-        </is>
-      </c>
-      <c r="B42" s="28" t="inlineStr">
-        <is>
-          <t>F. 진입·리텐션</t>
-        </is>
-      </c>
-      <c r="C42" s="29" t="inlineStr">
-        <is>
-          <t>중학교 이탈 방어 5종</t>
-        </is>
-      </c>
-      <c r="D42" s="30" t="inlineStr">
-        <is>
-          <t>감시감 제거·비교 전환·기여감·현실 효용·소셜 방어 UX</t>
-        </is>
-      </c>
-      <c r="E42" s="31" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4329,6 +4225,90 @@
           </r>
         </is>
       </c>
+      <c r="F41" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>사춘기 자율성 욕구와 충돌하지 않는 형태로 앱 사용이 지속된다. 중학교 이탈 위험이 구조적으로 완화된다.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="104" customHeight="1">
+      <c r="A42" s="27" t="inlineStr">
+        <is>
+          <t>F-4</t>
+        </is>
+      </c>
+      <c r="B42" s="28" t="inlineStr">
+        <is>
+          <t>F. 진입·리텐션</t>
+        </is>
+      </c>
+      <c r="C42" s="29" t="inlineStr">
+        <is>
+          <t>사전 허락 리스트</t>
+        </is>
+      </c>
+      <c r="D42" s="30" t="inlineStr">
+        <is>
+          <t>민법 제6조 프레임 기반 카테고리별 사전 한도 지정</t>
+        </is>
+      </c>
+      <c r="E42" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 개요
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">편의점, 문구, 학용품 등 카테고리별 소비 한도가 부모에 의해 사전에 지정된다. 민법 제6조의 "처분을 허락한 재산" 프레임을 응용한 구조다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 부모가 카테고리별 월별 한도를 사전 설정한다.
+2. 자녀의 소비가 자동으로 카테고리에 분류된다.
+3. 한도 내 소비는 자유롭게, 초과 시 부모 승인 알림이 발송된다.</t>
+          </r>
+        </is>
+      </c>
       <c r="F42" s="31" t="inlineStr">
         <is>
           <r>
@@ -4346,7 +4326,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>사춘기 자율성 욕구와 충돌하지 않는 형태로 앱 사용이 지속된다. 중학교 이탈 위험이 구조적으로 완화된다.</t>
+            <t>건별 승인 부담이 사라지고 자녀의 자율 영역이 명시적으로 정의된다. 법적 프레임을 차용해 부모의 권한 행사가 정당화된다.</t>
           </r>
         </is>
       </c>
@@ -4354,7 +4334,7 @@
     <row r="43" ht="104" customHeight="1">
       <c r="A43" s="27" t="inlineStr">
         <is>
-          <t>F-4</t>
+          <t>F-5</t>
         </is>
       </c>
       <c r="B43" s="28" t="inlineStr">
@@ -4364,12 +4344,12 @@
       </c>
       <c r="C43" s="29" t="inlineStr">
         <is>
-          <t>사전 허락 리스트</t>
+          <t>가족 투자 회의 템플릿</t>
         </is>
       </c>
       <c r="D43" s="30" t="inlineStr">
         <is>
-          <t>민법 제6조 프레임 기반 카테고리별 사전 한도 지정</t>
+          <t>월 1회 가족 투자 현황 리뷰 진행 템플릿</t>
         </is>
       </c>
       <c r="E43" s="31" t="inlineStr">
@@ -4389,7 +4369,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">편의점, 문구, 학용품 등 카테고리별 소비 한도가 부모에 의해 사전에 지정된다. 민법 제6조의 "처분을 허락한 재산" 프레임을 응용한 구조다.
+            <t xml:space="preserve">월 1회 가족 구성원이 함께 투자 현황을 리뷰할 수 있도록 회의 진행 템플릿이 제공된다. 부모의 포트폴리오 일부를 교육 소재로 공개하는 옵션이 포함된다.
 </t>
           </r>
           <r>
@@ -4407,9 +4387,9 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 부모가 카테고리별 월별 한도를 사전 설정한다.
-2. 자녀의 소비가 자동으로 카테고리에 분류된다.
-3. 한도 내 소비는 자유롭게, 초과 시 부모 승인 알림이 발송된다.</t>
+            <t>1. 월 1회 가족 회의 일정이 사전 설정된다.
+2. 회의 시점에 자녀·부모 자산 리포트가 자동 생성된다.
+3. 토론 주제와 의사결정 항목이 템플릿으로 제공된다.</t>
           </r>
         </is>
       </c>
@@ -4430,7 +4410,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>건별 승인 부담이 사라지고 자녀의 자율 영역이 명시적으로 정의된다. 법적 프레임을 차용해 부모의 권한 행사가 정당화된다.</t>
+            <t>투자가 개인 활동이 아닌 가족 단위 활동으로 재구성된다. 부모의 실제 투자 행태가 자녀의 학습 자료로 활용된다.</t>
           </r>
         </is>
       </c>
@@ -4438,7 +4418,7 @@
     <row r="44" ht="104" customHeight="1">
       <c r="A44" s="27" t="inlineStr">
         <is>
-          <t>F-5</t>
+          <t>F-6</t>
         </is>
       </c>
       <c r="B44" s="28" t="inlineStr">
@@ -4448,99 +4428,15 @@
       </c>
       <c r="C44" s="29" t="inlineStr">
         <is>
-          <t>가족 투자 회의 템플릿</t>
+          <t>증여 시뮬레이터 + 세무사 연결</t>
         </is>
       </c>
       <c r="D44" s="30" t="inlineStr">
         <is>
-          <t>월 1회 가족 투자 현황 리뷰 진행 템플릿</t>
+          <t>10년 단위 비과세 한도 추적과 증여 시뮬레이션, 세무사 제휴 연결</t>
         </is>
       </c>
       <c r="E44" s="31" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 개요
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">월 1회 가족 구성원이 함께 투자 현황을 리뷰할 수 있도록 회의 진행 템플릿이 제공된다. 부모의 포트폴리오 일부를 교육 소재로 공개하는 옵션이 포함된다.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 동작 방식
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. 월 1회 가족 회의 일정이 사전 설정된다.
-2. 회의 시점에 자녀·부모 자산 리포트가 자동 생성된다.
-3. 토론 주제와 의사결정 항목이 템플릿으로 제공된다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F44" s="31" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 기대 효과
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>투자가 개인 활동이 아닌 가족 단위 활동으로 재구성된다. 부모의 실제 투자 행태가 자녀의 학습 자료로 활용된다.</t>
-          </r>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="104" customHeight="1">
-      <c r="A45" s="27" t="inlineStr">
-        <is>
-          <t>F-6</t>
-        </is>
-      </c>
-      <c r="B45" s="28" t="inlineStr">
-        <is>
-          <t>F. 진입·리텐션</t>
-        </is>
-      </c>
-      <c r="C45" s="29" t="inlineStr">
-        <is>
-          <t>증여 시뮬레이터 + 세무사 연결</t>
-        </is>
-      </c>
-      <c r="D45" s="30" t="inlineStr">
-        <is>
-          <t>10년 단위 비과세 한도 추적과 증여 시뮬레이션, 세무사 제휴 연결</t>
-        </is>
-      </c>
-      <c r="E45" s="31" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4582,7 +4478,7 @@
           </r>
         </is>
       </c>
-      <c r="F45" s="31" t="inlineStr">
+      <c r="F44" s="31" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4604,28 +4500,28 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="104" customHeight="1">
-      <c r="A46" s="27" t="inlineStr">
+    <row r="45" ht="104" customHeight="1">
+      <c r="A45" s="27" t="inlineStr">
         <is>
           <t>F-7</t>
         </is>
       </c>
-      <c r="B46" s="28" t="inlineStr">
+      <c r="B45" s="28" t="inlineStr">
         <is>
           <t>F. 진입·리텐션</t>
         </is>
       </c>
-      <c r="C46" s="29" t="inlineStr">
+      <c r="C45" s="29" t="inlineStr">
         <is>
           <t>자동 이관 + Graduation 페이지</t>
         </is>
       </c>
-      <c r="D46" s="30" t="inlineStr">
+      <c r="D45" s="30" t="inlineStr">
         <is>
           <t>성년 도달 시 하나원큐 자동 이관과 졸업 페이지</t>
         </is>
       </c>
-      <c r="E46" s="31" t="inlineStr">
+      <c r="E45" s="31" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4666,7 +4562,7 @@
           </r>
         </is>
       </c>
-      <c r="F46" s="31" t="inlineStr">
+      <c r="F45" s="31" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4688,28 +4584,28 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="117" customHeight="1">
-      <c r="A47" s="27" t="inlineStr">
+    <row r="46" ht="117" customHeight="1">
+      <c r="A46" s="27" t="inlineStr">
         <is>
           <t>F-8</t>
         </is>
       </c>
-      <c r="B47" s="28" t="inlineStr">
+      <c r="B46" s="28" t="inlineStr">
         <is>
           <t>F. 진입·리텐션</t>
         </is>
       </c>
-      <c r="C47" s="29" t="inlineStr">
+      <c r="C46" s="29" t="inlineStr">
         <is>
           <t>절세 게이지 시각화</t>
         </is>
       </c>
-      <c r="D47" s="30" t="inlineStr">
+      <c r="D46" s="30" t="inlineStr">
         <is>
           <t>10년 단위 비과세 한도 사용률을 부모 메인 화면에 상시 게이지로 노출</t>
         </is>
       </c>
-      <c r="E47" s="31" t="inlineStr">
+      <c r="E46" s="31" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4751,7 +4647,7 @@
           </r>
         </is>
       </c>
-      <c r="F47" s="31" t="inlineStr">
+      <c r="F46" s="31" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4791,28 +4687,28 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="104" customHeight="1">
-      <c r="A48" s="27" t="inlineStr">
+    <row r="47" ht="104" customHeight="1">
+      <c r="A47" s="27" t="inlineStr">
         <is>
           <t>F-9</t>
         </is>
       </c>
-      <c r="B48" s="28" t="inlineStr">
+      <c r="B47" s="28" t="inlineStr">
         <is>
           <t>F. 진입·리텐션</t>
         </is>
       </c>
-      <c r="C48" s="29" t="inlineStr">
+      <c r="C47" s="29" t="inlineStr">
         <is>
           <t>3대 가문 시뮬레이터</t>
         </is>
       </c>
-      <c r="D48" s="30" t="inlineStr">
+      <c r="D47" s="30" t="inlineStr">
         <is>
           <t>조부모-부모-자녀 3대 자산을 한 화면에, 세대생략 증여까지 포괄</t>
         </is>
       </c>
-      <c r="E48" s="31" t="inlineStr">
+      <c r="E47" s="31" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4854,7 +4750,7 @@
           </r>
         </is>
       </c>
-      <c r="F48" s="31" t="inlineStr">
+      <c r="F47" s="31" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4890,6 +4786,90 @@
               <sz val="10"/>
             </rPr>
             <t>기존 증여 시뮬레이터가 부모-자녀 2대를 대상으로 한다면, 본 아이디어는 3대와 세대생략 증여까지 포괄한다.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="104" customHeight="1">
+      <c r="A48" s="32" t="inlineStr">
+        <is>
+          <t>G-1</t>
+        </is>
+      </c>
+      <c r="B48" s="33" t="inlineStr">
+        <is>
+          <t>G. 행동 전환·정체성</t>
+        </is>
+      </c>
+      <c r="C48" s="34" t="inlineStr">
+        <is>
+          <t>투자자 명함</t>
+        </is>
+      </c>
+      <c r="D48" s="35" t="inlineStr">
+        <is>
+          <t>투자 프로필을 카드 형태로 자동 생성하고 친구에게 공유</t>
+        </is>
+      </c>
+      <c r="E48" s="36" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 개요
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">자녀의 투자 프로필이 카드 형태로 자동 생성된다. "삼성전자 주주 | 첫 투자일 2027.3.15 | 누적 수익 +12,400원" 등 투자 정체성이 시각화되며 친구에게 공유될 수 있다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 보유 종목·첫 투자일·누적 수익·투자 스타일이 자동 카드화된다.
+2. 친구에게 카드 형태로 공유될 수 있다.
+3. 프로필 카드의 디자인은 자녀가 일부 커스터마이징할 수 있다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F48" s="36" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>감시 도구라는 부정적 인식이 투자자의 도구라는 정체성으로 전환된다. 친구 공유는 자연스러운 바이럴 채널로 작동하며 브랜드 인지도 지표로 활용된다.</t>
           </r>
         </is>
       </c>
@@ -4897,7 +4877,7 @@
     <row r="49" ht="104" customHeight="1">
       <c r="A49" s="32" t="inlineStr">
         <is>
-          <t>G-1</t>
+          <t>G-2</t>
         </is>
       </c>
       <c r="B49" s="33" t="inlineStr">
@@ -4907,12 +4887,12 @@
       </c>
       <c r="C49" s="34" t="inlineStr">
         <is>
-          <t>투자자 명함</t>
+          <t>실시간 자산 성장 피드백</t>
         </is>
       </c>
       <c r="D49" s="35" t="inlineStr">
         <is>
-          <t>투자 프로필을 카드 형태로 자동 생성하고 친구에게 공유</t>
+          <t>저축·투자 직후 즉각적인 자산 변화 시각화</t>
         </is>
       </c>
       <c r="E49" s="36" t="inlineStr">
@@ -4932,7 +4912,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">자녀의 투자 프로필이 카드 형태로 자동 생성된다. "삼성전자 주주 | 첫 투자일 2027.3.15 | 누적 수익 +12,400원" 등 투자 정체성이 시각화되며 친구에게 공유될 수 있다.
+            <t xml:space="preserve">자녀가 저축이나 투자를 실행한 직후 자산 변동이 즉시 시각화된다. "네 총 자산이 방금 124,300원에서 127,300원이 됐다"는 피드백과 함께 자산 그래프가 실시간으로 갱신된다. 매칭이 추가될 경우 "엄마가 3,000원 보태서 130,300원이 됐다"는 추가 표시가 노출된다.
 </t>
           </r>
           <r>
@@ -4950,9 +4930,9 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 보유 종목·첫 투자일·누적 수익·투자 스타일이 자동 카드화된다.
-2. 친구에게 카드 형태로 공유될 수 있다.
-3. 프로필 카드의 디자인은 자녀가 일부 커스터마이징할 수 있다.</t>
+            <t>1. 저축·투자 행동 직후 자산 변동 알림이 즉시 발송된다.
+2. 자산 그래프가 실시간 갱신된다.
+3. 매칭이 추가될 경우 추가 변동이 별도로 시각화된다.</t>
           </r>
         </is>
       </c>
@@ -4973,7 +4953,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>감시 도구라는 부정적 인식이 투자자의 도구라는 정체성으로 전환된다. 친구 공유는 자연스러운 바이럴 채널로 작동하며 브랜드 인지도 지표로 활용된다.</t>
+            <t>작은 행동의 결과가 즉각 가시화되어 반복 동기가 강화된다. 행동과 결과의 시간 격차가 사라져 학습 효과가 극대화된다.</t>
           </r>
         </is>
       </c>
@@ -4981,7 +4961,7 @@
     <row r="50" ht="104" customHeight="1">
       <c r="A50" s="32" t="inlineStr">
         <is>
-          <t>G-2</t>
+          <t>G-3</t>
         </is>
       </c>
       <c r="B50" s="33" t="inlineStr">
@@ -4991,99 +4971,15 @@
       </c>
       <c r="C50" s="34" t="inlineStr">
         <is>
-          <t>실시간 자산 성장 피드백</t>
+          <t>자산 연동 앱 테마 (성장형 비주얼)</t>
         </is>
       </c>
       <c r="D50" s="35" t="inlineStr">
         <is>
-          <t>저축·투자 직후 즉각적인 자산 변화 시각화</t>
+          <t>총 자산 규모에 따라 앱 배경·아이콘·위젯이 자동 진화</t>
         </is>
       </c>
       <c r="E50" s="36" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 개요
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">자녀가 저축이나 투자를 실행한 직후 자산 변동이 즉시 시각화된다. "네 총 자산이 방금 124,300원에서 127,300원이 됐다"는 피드백과 함께 자산 그래프가 실시간으로 갱신된다. 매칭이 추가될 경우 "엄마가 3,000원 보태서 130,300원이 됐다"는 추가 표시가 노출된다.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 동작 방식
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. 저축·투자 행동 직후 자산 변동 알림이 즉시 발송된다.
-2. 자산 그래프가 실시간 갱신된다.
-3. 매칭이 추가될 경우 추가 변동이 별도로 시각화된다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F50" s="36" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 기대 효과
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>작은 행동의 결과가 즉각 가시화되어 반복 동기가 강화된다. 행동과 결과의 시간 격차가 사라져 학습 효과가 극대화된다.</t>
-          </r>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="104" customHeight="1">
-      <c r="A51" s="32" t="inlineStr">
-        <is>
-          <t>G-3</t>
-        </is>
-      </c>
-      <c r="B51" s="33" t="inlineStr">
-        <is>
-          <t>G. 행동 전환·정체성</t>
-        </is>
-      </c>
-      <c r="C51" s="34" t="inlineStr">
-        <is>
-          <t>자산 연동 앱 테마 (성장형 비주얼)</t>
-        </is>
-      </c>
-      <c r="D51" s="35" t="inlineStr">
-        <is>
-          <t>총 자산 규모에 따라 앱 배경·아이콘·위젯이 자동 진화</t>
-        </is>
-      </c>
-      <c r="E51" s="36" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -5124,7 +5020,7 @@
           </r>
         </is>
       </c>
-      <c r="F51" s="36" t="inlineStr">
+      <c r="F50" s="36" t="inlineStr">
         <is>
           <r>
             <rPr>

</xml_diff>

<commit_message>
vault backup: 2026-04-27 18:13:43
</commit_message>
<xml_diff>
--- a/content/Consulting/05_Tobe전략/아이디어풀/아이디어_상세설명_260427.xlsx
+++ b/content/Consulting/05_Tobe전략/아이디어풀/아이디어_상세설명_260427.xlsx
@@ -685,7 +685,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4004,12 +4004,12 @@
       </c>
       <c r="C39" s="29" t="inlineStr">
         <is>
-          <t>부모 반복 트리거 5종</t>
+          <t>자녀 맞춤 인사이트 피드</t>
         </is>
       </c>
       <c r="D39" s="30" t="inlineStr">
         <is>
-          <t>자녀 인사이트·자산 통합·성장 리포트·세무 도구·성과 알림</t>
+          <t>자녀 행동 데이터 기반 부모 메인 화면 인사이트 카드 자동 생성</t>
         </is>
       </c>
       <c r="E39" s="31" t="inlineStr">
@@ -4029,7 +4029,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">부모의 반복 사용을 유도하는 5가지 핵심 트리거가 제공된다. ① 자녀 맞춤 인사이트 피드, ② 가족 자산 통합 뷰, ③ 분기 자녀 재무 성장 리포트, ④ 세무·증여 전략 도구, ⑤ 자녀 성과 알림.
+            <t xml:space="preserve">자녀의 저축·소비·투자 데이터를 매일 분석해 부모 메인 화면에 1~2장의 발견 카드가 자동으로 노출된다. "이번 주 저축률이 평소보다 30% 높음", "또래 평균 대비 지출 20% 낮음" 식으로 부모가 매일 들어와 확인할 만한 짧은 인사이트를 제공한다.
 </t>
           </r>
           <r>
@@ -4047,11 +4047,10 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 자녀의 행동 데이터를 기반으로 인사이트 피드가 자동 생성된다.
-2. 가족 전체 자산이 통합 뷰로 시각화된다.
-3. 분기별로 자녀의 재무 성장 리포트가 발행된다.
-4. 세무·증여 관련 의사결정 도구가 제공된다.
-5. 자녀의 주요 성과가 실시간 알림으로 전달된다.</t>
+            <t>1. 자녀 행동 데이터(저축·소비·투자)를 일별 집계·분석한다.
+2. 인사이트 후보를 자동 추출한다(평소 대비 변화·또래 대비 위치·마일스톤 임박 등).
+3. 부모 메인 화면 상단에 1~2장 카드로 자동 노출된다.
+4. 카드 탭 시 상세 분석 화면으로 진입한다.</t>
           </r>
         </is>
       </c>
@@ -4072,7 +4071,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>부모의 반복 진입 동기가 다층화된다. 한 가지 트리거가 약해도 다른 트리거로 보완되어 장기 리텐션이 안정화된다.</t>
+            <t>매일 들어와 "오늘은 무슨 변화가 있나" 확인하는 습관을 만든다. 부모가 자녀 데이터를 직접 파헤치지 않아도 자동으로 의미 있는 발견이 떠오르므로 인지 부하가 낮다.</t>
           </r>
         </is>
       </c>
@@ -4090,12 +4089,12 @@
       </c>
       <c r="C40" s="29" t="inlineStr">
         <is>
-          <t>조건·이벤트 트리거 7종</t>
+          <t>가족 자산 통합 뷰</t>
         </is>
       </c>
       <c r="D40" s="30" t="inlineStr">
         <is>
-          <t>외부 이벤트와 연동된 진입 트리거 7개</t>
+          <t>부모와 자녀 계좌 자산을 가족 단위로 통합 시각화</t>
         </is>
       </c>
       <c r="E40" s="31" t="inlineStr">
@@ -4115,7 +4114,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">사용자의 외부 이벤트와 연동된 7가지 진입 트리거가 운영된다. 세뱃돈 시즌, 월말·연말, 절약 감지, 배당·이자 발생, 학제 전환, 경제 뉴스, 조부모·친척 송금 시점이 포함된다.
+            <t xml:space="preserve">부모 본인 자산과 자녀 계좌 자산이 한 화면에 통합되어 보인다. 가족 전체 자산 중 자녀 비중과 증감 추세가 시각화되며, 자녀 자산이 가족 미래(예: 대학자금, 가족 여행)에 어떻게 기여하는지 한 눈에 파악된다.
 </t>
           </r>
           <r>
@@ -4133,9 +4132,10 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 각 이벤트 발생 시점이 시스템에 자동 감지된다.
-2. 이벤트 맥락에 맞는 추천 알림이 발송된다.
-3. 알림 클릭 시 이벤트에 최적화된 액션 화면으로 이동한다.</t>
+            <t>1. 부모·자녀 계좌가 연결된 통합 대시보드 화면을 제공한다.
+2. 가족 총 자산, 자녀 자산 비중, 가족 목표 진척률을 표시한다.
+3. 분기·연도별 가족 자산 변화 추세 그래프를 제공한다.
+4. 부모 자산과 자녀 자산이 함께 그려지는 "가족 곡선"을 시각화한다.</t>
           </r>
         </is>
       </c>
@@ -4156,7 +4156,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>사용자의 일상 흐름과 동기화된 진입 동기가 형성된다. 외부 이벤트가 곧 앱 사용의 트리거가 된다.</t>
+            <t>자녀 자산 관리가 "애 용돈 챙겨주기"가 아니라 "가족 전체 자산 형성"의 일부로 인식된다. 부모의 본인 자산 관리 동기와 자녀 자산 관리 동기가 한 흐름으로 결합된다.</t>
           </r>
         </is>
       </c>
@@ -4174,12 +4174,12 @@
       </c>
       <c r="C41" s="29" t="inlineStr">
         <is>
-          <t>중학교 이탈 방어 5종</t>
+          <t>분기 자녀 재무 성장 리포트</t>
         </is>
       </c>
       <c r="D41" s="30" t="inlineStr">
         <is>
-          <t>감시감 제거·비교 전환·기여감·현실 효용·소셜 방어 UX</t>
+          <t>분기별 자녀 자산·저축·투자 성장 종합 리포트 자동 발행</t>
         </is>
       </c>
       <c r="E41" s="31" t="inlineStr">
@@ -4199,7 +4199,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t xml:space="preserve">중학교 진학기에 발생하는 자녀 이탈을 방어하는 5가지 장치가 적용된다. ① 감시감 제거(소비 세부의 부모 노출 기본 OFF), ② 또래에서 가족 단위로 비교 전환, ③ 기여감 부여, ④ 현실 효용 강조, ⑤ 소셜 방어 UX 언어.
+            <t xml:space="preserve">분기마다 자녀의 자산 변동, 저축률 추이, 투자 수익률, 행동 패턴이 종합된 리포트가 부모에게 자동으로 발행된다. 한 분기를 돌아보고 다음 분기 방향을 잡을 수 있는 미니 자산 보고서 형태다.
 </t>
           </r>
           <r>
@@ -4217,11 +4217,10 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>1. 중학교 입학 시점이 감지되면 감시감 제거 모드가 자동 활성화된다.
-2. 비교 지표가 또래에서 가족 단위로 전환된다.
-3. 자녀의 기여 활동이 우선 노출된다.
-4. 현실 효용 중심의 콘텐츠가 큐레이션된다.
-5. 소셜 친화적 UX 언어가 적용된다.</t>
+            <t>1. 분기 종료 시점에 자산 증감·저축률·수익률·주요 이벤트가 자동 집계된다.
+2. 리포트 카드/PDF가 자동 생성되어 부모에게 알림이 발송된다.
+3. 자녀에게도 "분기 성장 카드" 형태로 공유 옵션이 제공된다.
+4. 다음 분기 목표·전략 제안 섹션이 함께 포함된다.</t>
           </r>
         </is>
       </c>
@@ -4242,7 +4241,7 @@
               <rFont val="맑은 고딕"/>
               <sz val="10"/>
             </rPr>
-            <t>사춘기 자율성 욕구와 충돌하지 않는 형태로 앱 사용이 지속된다. 중학교 이탈 위험이 구조적으로 완화된다.</t>
+            <t>매일·매주 단위 인사이트와 별도로, 분기 단위의 큰 흐름을 회고할 수 있다. 학기·분기 단위로 돌아가는 자녀 일상 리듬과 동기화되어 자연스럽게 부모의 검토 루틴이 형성된다.</t>
           </r>
         </is>
       </c>
@@ -4260,15 +4259,699 @@
       </c>
       <c r="C42" s="29" t="inlineStr">
         <is>
+          <t>세무·증여 전략 도구</t>
+        </is>
+      </c>
+      <c r="D42" s="30" t="inlineStr">
+        <is>
+          <t>부모의 증여 의사결정을 돕는 절세·전략 도구 패키지</t>
+        </is>
+      </c>
+      <c r="E42" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 개요
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">비과세 한도 추적, 증여 시점 시뮬레이션, 세무사 연결까지 부모의 증여 관련 의사결정을 종합 지원하는 도구. F-14 증여 시뮬레이터, F-16 절세 게이지의 통합 진입점으로 작동한다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 부모 메인에 "증여 전략" 통합 진입 카드가 노출된다.
+2. 진입 시 비과세 한도 잔여, 만료 D-day, 분할 증여 시뮬, 세무사 연결 옵션이 한 화면에 노출된다.
+3. 증여 의사결정 단계별 가이드가 제공된다(현재 상황 진단 → 시나리오 비교 → 실행).
+4. 복잡한 케이스는 제휴 세무사와의 1-탭 연결을 지원한다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F42" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>증여 관련 기능들이 흩어져 있으면 부모가 어디서 시작할지 헷갈린다. 통합 진입점 하나로 묶으면 "증여 = 여기 들어가면 다 있다"는 인지가 형성되어 고자산 부모층의 장기 로열티 훅으로 작동한다.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="104" customHeight="1">
+      <c r="A43" s="27" t="inlineStr">
+        <is>
+          <t>F-5</t>
+        </is>
+      </c>
+      <c r="B43" s="28" t="inlineStr">
+        <is>
+          <t>F. 진입·리텐션</t>
+        </is>
+      </c>
+      <c r="C43" s="29" t="inlineStr">
+        <is>
+          <t>자녀 성과 알림</t>
+        </is>
+      </c>
+      <c r="D43" s="30" t="inlineStr">
+        <is>
+          <t>자녀의 저축·투자 주요 성과를 부모에게 실시간 푸시</t>
+        </is>
+      </c>
+      <c r="E43" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 개요
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">자녀가 첫 매수, 첫 배당, 목표 달성, 마일스톤 도달 등 의미 있는 성과를 만들 때마다 부모에게 실시간 알림이 전송된다. 부모가 "애가 지금 뭘 하고 있는지" 자연스럽게 알게 되는 핵심 채널이다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 성과 이벤트가 자동 감지된다(첫 매수·첫 배당·자산 임계치 도달·매칭 달성 등).
+2. 즉시 부모에게 푸시 알림이 발송된다.
+3. 알림 탭 시 자녀 성과 상세 카드로 진입한다.
+4. "축하 메시지 보내기" 1-탭 액션으로 자녀에게 응원 메시지가 전달된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F43" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>자녀의 성장 순간을 부모가 놓치지 않게 한다. 알림 자체가 부모의 앱 진입 트리거가 되며, "축하" 액션을 통해 부모-자녀 사이 긍정 피드백 루프가 형성된다.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="143" customHeight="1">
+      <c r="A44" s="27" t="inlineStr">
+        <is>
+          <t>F-6</t>
+        </is>
+      </c>
+      <c r="B44" s="28" t="inlineStr">
+        <is>
+          <t>F. 진입·리텐션</t>
+        </is>
+      </c>
+      <c r="C44" s="29" t="inlineStr">
+        <is>
+          <t>조건·이벤트 트리거 7종</t>
+        </is>
+      </c>
+      <c r="D44" s="30" t="inlineStr">
+        <is>
+          <t>일상 속 주요 이벤트를 자동 감지해 그 시점에 가장 필요한 행동을 안내하는 트리거 시스템</t>
+        </is>
+      </c>
+      <c r="E44" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 개요
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">사용자가 직접 떠올리지 않아도 아이부자가 일상의 주요 이벤트를 자동 감지하고, 그 시점에 가장 적절한 행동이나 학습 콘텐츠를 안내한다. 시간 이벤트, 금융 이벤트, 행동 이벤트, 외부 시장 이벤트의 4가지 축에서 총 7개 트리거가 동작한다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 명절 시즌(설날·추석 D-7) → 부모에게 세뱃돈 관리·이체 안내
+2. 월말·연말 → 자녀와 부모에게 소비 회고·다음 기간 계획 카드
+3. 학제 전환(자녀 만 7·13·16·19세) → 단계 전환 위저드 자동 진입
+4. 배당·이자 발생 → 패시브 인컴 학습 카드(첫 발생 시 학습 콘텐츠 동반)
+5. 절약 감지(주간 소비 평균 대비 감소) → 매칭 부스트 활성화 알림
+6. 경제 뉴스(보유 종목 관련) → 자녀 자산 변동과 연결한 알림
+7. 조부모·친척 송금 입금 → 시드 전환 추천 화면</t>
+          </r>
+        </is>
+      </c>
+      <c r="F44" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>사용자의 일상 흐름과 동기화된 진입 동기가 자동으로 만들어진다. 외부 이벤트가 곧 앱 사용의 트리거가 되며, 7개의 다층 트리거가 각자 다른 시점에 작동해 한 가지가 약해도 다른 트리거로 진입이 보완된다.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="104" customHeight="1">
+      <c r="A45" s="27" t="inlineStr">
+        <is>
+          <t>F-7</t>
+        </is>
+      </c>
+      <c r="B45" s="28" t="inlineStr">
+        <is>
+          <t>F. 진입·리텐션</t>
+        </is>
+      </c>
+      <c r="C45" s="29" t="inlineStr">
+        <is>
+          <t>감시감 제거</t>
+        </is>
+      </c>
+      <c r="D45" s="30" t="inlineStr">
+        <is>
+          <t>사춘기 진입 시점부터 소비 세부 내역의 부모 노출을 기본값 OFF로 전환</t>
+        </is>
+      </c>
+      <c r="E45" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 개요
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">자녀가 중학교에 진입하는 시점부터 자녀의 소비 세부 내역이 부모 화면에서 기본적으로 가려진다. 부모는 큰 흐름(주간·월간 합계)만 볼 수 있고, 자녀는 "감시받지 않는다"는 감각을 갖게 된다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 자녀 중학교 진입(만 13세) 시점이 자동 감지된다.
+2. 부모 화면의 자녀 소비 상세 항목이 기본값 OFF로 전환된다.
+3. 부모는 "주간·월간 총 합계" 같은 큰 흐름 통계만 노출된다.
+4. 부모가 명시적으로 권한 요청 시 자녀 동의 후에만 상세 열람된다.
+5. 자녀에게 "이제 부모가 네 소비를 자세히 보지 않는다"는 안내 카드가 제공된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F45" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>청소년기 자녀가 "감시받는다"는 인식을 갖는 순간 앱 사용은 빠르게 이탈로 이어진다. 권한 자체를 사춘기 진입 시점에 자동으로 줄이는 구조는 자녀의 자율 사용을 우선해 장기 사용을 가능하게 한다.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="104" customHeight="1">
+      <c r="A46" s="27" t="inlineStr">
+        <is>
+          <t>F-8</t>
+        </is>
+      </c>
+      <c r="B46" s="28" t="inlineStr">
+        <is>
+          <t>F. 진입·리텐션</t>
+        </is>
+      </c>
+      <c r="C46" s="29" t="inlineStr">
+        <is>
+          <t>또래→가족 비교 전환</t>
+        </is>
+      </c>
+      <c r="D46" s="30" t="inlineStr">
+        <is>
+          <t>동년배 비교 지표를 "또래"에서 "가족 단위"로 전환</t>
+        </is>
+      </c>
+      <c r="E46" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 개요
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">사춘기 자녀에게 "또래 평균 대비 너의 위치" 같은 비교는 부담스럽다. 비교 기준을 "가족 단위 자산 형성에 너의 기여"로 전환해 비교 압박을 줄이고, 동시에 가족 정체성을 강화한다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 자녀 중학교 진입(만 13세) 시점부터 비교 지표 UI가 자동 전환된다.
+2. "또래 대비 저축률 OO%"를 "가족 자산 중 너의 기여 OO원" 식 표현으로 변경한다.
+3. 또래 데이터는 보조 지표로만 노출되고 가족 데이터를 메인으로 표시한다.
+4. 가족 목표(가족 여행·자녀 대학자금 등) 대비 진척률을 표시한다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F46" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>또래 비교는 "내가 부족하다"는 인식을 만들어 동기 저하로 이어질 수 있다. 가족 단위 비교로 전환하면 "내가 가족에 도움이 된다"는 긍정적 정체성이 형성되어 사용 동기가 유지된다.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="104" customHeight="1">
+      <c r="A47" s="27" t="inlineStr">
+        <is>
+          <t>F-9</t>
+        </is>
+      </c>
+      <c r="B47" s="28" t="inlineStr">
+        <is>
+          <t>F. 진입·리텐션</t>
+        </is>
+      </c>
+      <c r="C47" s="29" t="inlineStr">
+        <is>
+          <t>기여감 부여</t>
+        </is>
+      </c>
+      <c r="D47" s="30" t="inlineStr">
+        <is>
+          <t>자녀의 저축·투자가 가족 자산에 기여한다는 감각을 시각화</t>
+        </is>
+      </c>
+      <c r="E47" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 개요
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">자녀의 자산 성장이 가족 통합 자산에 어떤 비중을 차지하는지, 가족 목표(예: 가족 여행, 자녀 대학자금)에 얼마나 기여하는지 시각화한다. "내가 가족에 도움이 된다"는 정체성을 형성해 사춘기 이탈을 방어한다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 가족 통합 자산 화면에서 자녀 기여 비중이 시각화된다.
+2. 가족 목표 진척률 화면에 자녀 기여 영역이 별도로 표시된다.
+3. "이번 달 자녀가 가족 자산에 +120,000원 기여" 식의 카드형 알림이 제공된다.
+4. 분기별 "자녀 기여 리포트"가 종합되어 발행된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F47" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>청소년기 자녀에게 "가족에 기여한다"는 인식은 자존감과 사용 동기를 동시에 강화한다. 자녀의 행동이 추상적 "내 자산"에서 구체적 "가족 자산 형성"으로 의미가 확장되어 책임감이 증가한다.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="117" customHeight="1">
+      <c r="A48" s="27" t="inlineStr">
+        <is>
+          <t>F-10</t>
+        </is>
+      </c>
+      <c r="B48" s="28" t="inlineStr">
+        <is>
+          <t>F. 진입·리텐션</t>
+        </is>
+      </c>
+      <c r="C48" s="29" t="inlineStr">
+        <is>
+          <t>현실 효용</t>
+        </is>
+      </c>
+      <c r="D48" s="30" t="inlineStr">
+        <is>
+          <t>자녀의 자산이 실제 현실에 어떤 효용을 가져오는지 매칭 표시</t>
+        </is>
+      </c>
+      <c r="E48" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 개요
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">자녀의 자산이 실제로 무엇을 살 수 있는지, 어떤 경험을 가능하게 하는지를 구체적인 사물·경험과 매칭해 표시한다. "네 자산으로 닌텐도 스위치 OO개", "네 자산으로 일본 여행 항공권 OO장" 식으로 자산이 "가능한 경험"으로 인식되도록 한다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 자녀 총 자산 변동 시 자동으로 현실 매칭 카드가 생성된다.
+2. 자녀 위시리스트·관심 항목 데이터를 활용해 매칭 대상이 개인화된다.
+3. 매칭 단위는 사물(닌텐도, 자전거 등), 경험(여행, 콘서트), 미래 자산(대학 등록금 OO%)으로 다양화된다.
+4. 자녀가 직접 "이 항목으로 환산해보기"를 선택할 수 있다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F48" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>청소년기 자녀에게 "OO만원"은 추상적이지만 "닌텐도 스위치 2개"는 구체적이다. 자산을 현실 효용으로 환산해 보여주면 저축·투자 행동의 의미가 직관적으로 이해되고, 사용 동기가 유지된다.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="104" customHeight="1">
+      <c r="A49" s="27" t="inlineStr">
+        <is>
+          <t>F-11</t>
+        </is>
+      </c>
+      <c r="B49" s="28" t="inlineStr">
+        <is>
+          <t>F. 진입·리텐션</t>
+        </is>
+      </c>
+      <c r="C49" s="29" t="inlineStr">
+        <is>
+          <t>소셜 방어 UX 언어</t>
+        </is>
+      </c>
+      <c r="D49" s="30" t="inlineStr">
+        <is>
+          <t>또래에게 노출됐을 때 "감시앱"처럼 보이지 않도록 UI 톤·언어 조정</t>
+        </is>
+      </c>
+      <c r="E49" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 개요
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">친구가 자녀의 핸드폰을 봤을 때 "부모가 감시하는 앱"으로 보이지 않도록, 자녀 화면의 톤·아이콘·언어가 "투자자가 쓰는 도구"로 일관 조정된다. 사춘기 자녀의 사회적 이미지를 보호하면서 앱 사용을 지속하게 한다.
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 동작 방식
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>1. 자녀 화면의 모든 텍스트·시각 요소가 사춘기 친화적 톤으로 자동 적용된다.
+2. "용돈", "부모" 같은 단어 노출이 최소화된다("내 자금", "파트너" 등으로 대체).
+3. 메인 화면 디자인이 금융 앱 스타일(차트·그래프·종목명 위주)로 노출된다.
+4. "엄마가 본다" 인지를 만드는 시각적 단서가 모두 제거된다.</t>
+          </r>
+        </is>
+      </c>
+      <c r="F49" s="31" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <b val="1"/>
+              <color rgb="001F3864"/>
+              <sz val="10"/>
+            </rPr>
+            <t xml:space="preserve">▣ 기대 효과
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="맑은 고딕"/>
+              <sz val="10"/>
+            </rPr>
+            <t>또래 앞에서의 사회적 이미지가 사춘기 사용 지속의 핵심 변수다. 자녀가 친구에게 "이게 뭐야?"라고 물을 때 "투자 앱"이라고 자신 있게 답할 수 있는 톤이면 이탈이 일어나지 않는다.</t>
+          </r>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="104" customHeight="1">
+      <c r="A50" s="27" t="inlineStr">
+        <is>
+          <t>F-12</t>
+        </is>
+      </c>
+      <c r="B50" s="28" t="inlineStr">
+        <is>
+          <t>F. 진입·리텐션</t>
+        </is>
+      </c>
+      <c r="C50" s="29" t="inlineStr">
+        <is>
           <t>사전 허락 리스트</t>
         </is>
       </c>
-      <c r="D42" s="30" t="inlineStr">
+      <c r="D50" s="30" t="inlineStr">
         <is>
           <t>민법 제6조 프레임 기반 카테고리별 사전 한도 지정</t>
         </is>
       </c>
-      <c r="E42" s="31" t="inlineStr">
+      <c r="E50" s="31" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4309,7 +4992,7 @@
           </r>
         </is>
       </c>
-      <c r="F42" s="31" t="inlineStr">
+      <c r="F50" s="31" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4331,28 +5014,28 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="104" customHeight="1">
-      <c r="A43" s="27" t="inlineStr">
-        <is>
-          <t>F-5</t>
-        </is>
-      </c>
-      <c r="B43" s="28" t="inlineStr">
+    <row r="51" ht="104" customHeight="1">
+      <c r="A51" s="27" t="inlineStr">
+        <is>
+          <t>F-13</t>
+        </is>
+      </c>
+      <c r="B51" s="28" t="inlineStr">
         <is>
           <t>F. 진입·리텐션</t>
         </is>
       </c>
-      <c r="C43" s="29" t="inlineStr">
+      <c r="C51" s="29" t="inlineStr">
         <is>
           <t>가족 투자 회의 템플릿</t>
         </is>
       </c>
-      <c r="D43" s="30" t="inlineStr">
+      <c r="D51" s="30" t="inlineStr">
         <is>
           <t>월 1회 가족 투자 현황 리뷰 진행 템플릿</t>
         </is>
       </c>
-      <c r="E43" s="31" t="inlineStr">
+      <c r="E51" s="31" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4393,7 +5076,7 @@
           </r>
         </is>
       </c>
-      <c r="F43" s="31" t="inlineStr">
+      <c r="F51" s="31" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4415,28 +5098,28 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="104" customHeight="1">
-      <c r="A44" s="27" t="inlineStr">
-        <is>
-          <t>F-6</t>
-        </is>
-      </c>
-      <c r="B44" s="28" t="inlineStr">
+    <row r="52" ht="104" customHeight="1">
+      <c r="A52" s="27" t="inlineStr">
+        <is>
+          <t>F-14</t>
+        </is>
+      </c>
+      <c r="B52" s="28" t="inlineStr">
         <is>
           <t>F. 진입·리텐션</t>
         </is>
       </c>
-      <c r="C44" s="29" t="inlineStr">
+      <c r="C52" s="29" t="inlineStr">
         <is>
           <t>증여 시뮬레이터 + 세무사 연결</t>
         </is>
       </c>
-      <c r="D44" s="30" t="inlineStr">
+      <c r="D52" s="30" t="inlineStr">
         <is>
           <t>10년 단위 비과세 한도 추적과 증여 시뮬레이션, 세무사 제휴 연결</t>
         </is>
       </c>
-      <c r="E44" s="31" t="inlineStr">
+      <c r="E52" s="31" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4478,7 +5161,7 @@
           </r>
         </is>
       </c>
-      <c r="F44" s="31" t="inlineStr">
+      <c r="F52" s="31" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4500,28 +5183,28 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="104" customHeight="1">
-      <c r="A45" s="27" t="inlineStr">
-        <is>
-          <t>F-7</t>
-        </is>
-      </c>
-      <c r="B45" s="28" t="inlineStr">
+    <row r="53" ht="104" customHeight="1">
+      <c r="A53" s="27" t="inlineStr">
+        <is>
+          <t>F-15</t>
+        </is>
+      </c>
+      <c r="B53" s="28" t="inlineStr">
         <is>
           <t>F. 진입·리텐션</t>
         </is>
       </c>
-      <c r="C45" s="29" t="inlineStr">
+      <c r="C53" s="29" t="inlineStr">
         <is>
           <t>자동 이관 + Graduation 페이지</t>
         </is>
       </c>
-      <c r="D45" s="30" t="inlineStr">
+      <c r="D53" s="30" t="inlineStr">
         <is>
           <t>성년 도달 시 하나원큐 자동 이관과 졸업 페이지</t>
         </is>
       </c>
-      <c r="E45" s="31" t="inlineStr">
+      <c r="E53" s="31" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4562,7 +5245,7 @@
           </r>
         </is>
       </c>
-      <c r="F45" s="31" t="inlineStr">
+      <c r="F53" s="31" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4584,28 +5267,28 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="117" customHeight="1">
-      <c r="A46" s="27" t="inlineStr">
-        <is>
-          <t>F-8</t>
-        </is>
-      </c>
-      <c r="B46" s="28" t="inlineStr">
+    <row r="54" ht="117" customHeight="1">
+      <c r="A54" s="27" t="inlineStr">
+        <is>
+          <t>F-16</t>
+        </is>
+      </c>
+      <c r="B54" s="28" t="inlineStr">
         <is>
           <t>F. 진입·리텐션</t>
         </is>
       </c>
-      <c r="C46" s="29" t="inlineStr">
+      <c r="C54" s="29" t="inlineStr">
         <is>
           <t>절세 게이지 시각화</t>
         </is>
       </c>
-      <c r="D46" s="30" t="inlineStr">
+      <c r="D54" s="30" t="inlineStr">
         <is>
           <t>10년 단위 비과세 한도 사용률을 부모 메인 화면에 상시 게이지로 노출</t>
         </is>
       </c>
-      <c r="E46" s="31" t="inlineStr">
+      <c r="E54" s="31" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4647,7 +5330,7 @@
           </r>
         </is>
       </c>
-      <c r="F46" s="31" t="inlineStr">
+      <c r="F54" s="31" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4687,131 +5370,28 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="104" customHeight="1">
-      <c r="A47" s="27" t="inlineStr">
-        <is>
-          <t>F-9</t>
-        </is>
-      </c>
-      <c r="B47" s="28" t="inlineStr">
-        <is>
-          <t>F. 진입·리텐션</t>
-        </is>
-      </c>
-      <c r="C47" s="29" t="inlineStr">
-        <is>
-          <t>3대 가문 시뮬레이터</t>
-        </is>
-      </c>
-      <c r="D47" s="30" t="inlineStr">
-        <is>
-          <t>조부모-부모-자녀 3대 자산을 한 화면에, 세대생략 증여까지 포괄</t>
-        </is>
-      </c>
-      <c r="E47" s="31" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 개요
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">조부모-부모-자녀 3대의 자산을 한 화면에 입력해 자산이전 시나리오를 비교 시뮬레이션한다. 전통 2단계(조부모→부모→자녀), 세대생략 증여(조부모→자녀 직접), 병행 시나리오의 3종을 60년 가문 자산 곡선으로 동시 비교하며, 비과세 한도와 세금이 자동 최적화된다.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 동작 방식
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>1. 조부모, 부모, 자녀의 현재 자산이 입력된다.
-2. 전통 2단계, 세대생략 증여, 병행 시나리오 3종이 비교된다.
-3. 60년 가문 자산 곡선과 세금·비과세 한도 최적화가 자동 계산된다.
-4. 조부모 전용 진입 화면이 별도로 제공된다.</t>
-          </r>
-        </is>
-      </c>
-      <c r="F47" s="31" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 기대 효과
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">단순 부모-자녀 시뮬을 넘어 가문 단위 사고가 가능해진다. 조부모층이 신규 사용자층으로 유입되며, 세대생략 증여라는 고급 절세 옵션이 가시화된다.
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <b val="1"/>
-              <color rgb="001F3864"/>
-              <sz val="10"/>
-            </rPr>
-            <t xml:space="preserve">▣ 차별 포인트
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="맑은 고딕"/>
-              <sz val="10"/>
-            </rPr>
-            <t>기존 증여 시뮬레이터가 부모-자녀 2대를 대상으로 한다면, 본 아이디어는 3대와 세대생략 증여까지 포괄한다.</t>
-          </r>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="104" customHeight="1">
-      <c r="A48" s="32" t="inlineStr">
+    <row r="55" ht="104" customHeight="1">
+      <c r="A55" s="32" t="inlineStr">
         <is>
           <t>G-1</t>
         </is>
       </c>
-      <c r="B48" s="33" t="inlineStr">
+      <c r="B55" s="33" t="inlineStr">
         <is>
           <t>G. 행동 전환·정체성</t>
         </is>
       </c>
-      <c r="C48" s="34" t="inlineStr">
+      <c r="C55" s="34" t="inlineStr">
         <is>
           <t>투자자 명함</t>
         </is>
       </c>
-      <c r="D48" s="35" t="inlineStr">
+      <c r="D55" s="35" t="inlineStr">
         <is>
           <t>투자 프로필을 카드 형태로 자동 생성하고 친구에게 공유</t>
         </is>
       </c>
-      <c r="E48" s="36" t="inlineStr">
+      <c r="E55" s="36" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4852,7 +5432,7 @@
           </r>
         </is>
       </c>
-      <c r="F48" s="36" t="inlineStr">
+      <c r="F55" s="36" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4874,28 +5454,28 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="104" customHeight="1">
-      <c r="A49" s="32" t="inlineStr">
+    <row r="56" ht="104" customHeight="1">
+      <c r="A56" s="32" t="inlineStr">
         <is>
           <t>G-2</t>
         </is>
       </c>
-      <c r="B49" s="33" t="inlineStr">
+      <c r="B56" s="33" t="inlineStr">
         <is>
           <t>G. 행동 전환·정체성</t>
         </is>
       </c>
-      <c r="C49" s="34" t="inlineStr">
+      <c r="C56" s="34" t="inlineStr">
         <is>
           <t>실시간 자산 성장 피드백</t>
         </is>
       </c>
-      <c r="D49" s="35" t="inlineStr">
+      <c r="D56" s="35" t="inlineStr">
         <is>
           <t>저축·투자 직후 즉각적인 자산 변화 시각화</t>
         </is>
       </c>
-      <c r="E49" s="36" t="inlineStr">
+      <c r="E56" s="36" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4936,7 +5516,7 @@
           </r>
         </is>
       </c>
-      <c r="F49" s="36" t="inlineStr">
+      <c r="F56" s="36" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -4958,28 +5538,28 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="104" customHeight="1">
-      <c r="A50" s="32" t="inlineStr">
+    <row r="57" ht="104" customHeight="1">
+      <c r="A57" s="32" t="inlineStr">
         <is>
           <t>G-3</t>
         </is>
       </c>
-      <c r="B50" s="33" t="inlineStr">
+      <c r="B57" s="33" t="inlineStr">
         <is>
           <t>G. 행동 전환·정체성</t>
         </is>
       </c>
-      <c r="C50" s="34" t="inlineStr">
+      <c r="C57" s="34" t="inlineStr">
         <is>
           <t>자산 연동 앱 테마 (성장형 비주얼)</t>
         </is>
       </c>
-      <c r="D50" s="35" t="inlineStr">
+      <c r="D57" s="35" t="inlineStr">
         <is>
           <t>총 자산 규모에 따라 앱 배경·아이콘·위젯이 자동 진화</t>
         </is>
       </c>
-      <c r="E50" s="36" t="inlineStr">
+      <c r="E57" s="36" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -5020,7 +5600,7 @@
           </r>
         </is>
       </c>
-      <c r="F50" s="36" t="inlineStr">
+      <c r="F57" s="36" t="inlineStr">
         <is>
           <r>
             <rPr>

</xml_diff>